<commit_message>
docs: close TTS cache hardening
</commit_message>
<xml_diff>
--- a/docs/governance/sprint-queue.xlsx
+++ b/docs/governance/sprint-queue.xlsx
@@ -1259,9 +1259,7 @@
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="13">
-      <c r="A11" s="20" t="n">
-        <v>1</v>
-      </c>
+      <c r="A11" s="20" t="n"/>
       <c r="B11" s="20" t="inlineStr">
         <is>
           <t>TTS-INTEGRATE-1</t>
@@ -1292,7 +1290,7 @@
       </c>
       <c r="H11" s="20" t="inlineStr">
         <is>
-          <t>Queued</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="I11" s="20" t="inlineStr">
@@ -1316,9 +1314,7 @@
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="13">
-      <c r="A12" s="12" t="n">
-        <v>2</v>
-      </c>
+      <c r="A12" s="12" t="n"/>
       <c r="B12" s="12" t="inlineStr">
         <is>
           <t>TTS-CACHE-HARDEN-1</t>
@@ -1349,12 +1345,12 @@
       </c>
       <c r="H12" s="12" t="inlineStr">
         <is>
-          <t>Queued</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="I12" s="12" t="inlineStr">
         <is>
-          <t>Full Spec</t>
+          <t>Full spec</t>
         </is>
       </c>
       <c r="J12" s="12" t="inlineStr">
@@ -1370,7 +1366,7 @@
     </row>
     <row r="13" ht="15" customHeight="1" s="13">
       <c r="A13" s="20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B13" s="20" t="inlineStr">
         <is>
@@ -1389,7 +1385,7 @@
       </c>
       <c r="E13" s="20" t="inlineStr">
         <is>
-          <t>Precision Infrastructure</t>
+          <t>Stage 2: Event-Driven Sync</t>
         </is>
       </c>
       <c r="F13" s="20" t="n">
@@ -1397,7 +1393,7 @@
       </c>
       <c r="G13" s="20" t="inlineStr">
         <is>
-          <t>TTS-CACHE-HARDEN-1</t>
+          <t>TTS-CACHE-HARDEN-1 (completed 2026-05-16)</t>
         </is>
       </c>
       <c r="H13" s="20" t="inlineStr">
@@ -1427,7 +1423,7 @@
     </row>
     <row r="14" ht="15" customHeight="1" s="13">
       <c r="A14" s="20" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B14" s="20" t="inlineStr">
         <is>
@@ -1446,7 +1442,7 @@
       </c>
       <c r="E14" s="20" t="inlineStr">
         <is>
-          <t>Precision Infrastructure</t>
+          <t>Stage 2: Normalizer Enrichment</t>
         </is>
       </c>
       <c r="F14" s="20" t="n">
@@ -1484,7 +1480,7 @@
     </row>
     <row r="15" ht="15" customHeight="1" s="13">
       <c r="A15" s="20" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B15" s="20" t="inlineStr">
         <is>
@@ -1503,7 +1499,7 @@
       </c>
       <c r="E15" s="20" t="inlineStr">
         <is>
-          <t>Precision Infrastructure</t>
+          <t>Stage 2: Word Position Index</t>
         </is>
       </c>
       <c r="F15" s="20" t="n">
@@ -1541,7 +1537,7 @@
     </row>
     <row r="16" ht="15" customHeight="1" s="13">
       <c r="A16" s="20" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B16" s="20" t="inlineStr">
         <is>
@@ -1560,7 +1556,7 @@
       </c>
       <c r="E16" s="20" t="inlineStr">
         <is>
-          <t>Verification</t>
+          <t>Stage 3: Pipeline Truth</t>
         </is>
       </c>
       <c r="F16" s="20" t="n">
@@ -1594,7 +1590,7 @@
     </row>
     <row r="17" ht="15" customHeight="1" s="13">
       <c r="A17" s="20" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B17" s="20" t="inlineStr">
         <is>
@@ -1613,7 +1609,7 @@
       </c>
       <c r="E17" s="20" t="inlineStr">
         <is>
-          <t>Governance</t>
+          <t>Stage 4: Governance</t>
         </is>
       </c>
       <c r="F17" s="20" t="n">

</xml_diff>

<commit_message>
docs: make sprint queue workbook authoritative
</commit_message>
<xml_diff>
--- a/docs/governance/sprint-queue.xlsx
+++ b/docs/governance/sprint-queue.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -83,8 +83,12 @@
       <strike val="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -127,6 +131,11 @@
         <bgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -147,7 +156,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -217,6 +226,9 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -559,11 +571,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="B1:H3"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="12" min="1" max="1"/>
-    <col width="16" customWidth="1" style="12" min="2" max="8"/>
+    <col width="18" customWidth="1" style="12" min="2" max="8"/>
+    <col width="18" customWidth="1" style="13" min="3" max="3"/>
+    <col width="18" customWidth="1" style="13" min="4" max="4"/>
+    <col width="18" customWidth="1" style="13" min="5" max="5"/>
+    <col width="18" customWidth="1" style="13" min="6" max="6"/>
+    <col width="18" customWidth="1" style="13" min="7" max="7"/>
+    <col width="18" customWidth="1" style="13" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="17.25" customHeight="1" s="13">
@@ -574,70 +592,109 @@
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" s="13">
-      <c r="B2" s="15" t="inlineStr">
+      <c r="B2" s="24" t="inlineStr">
         <is>
           <t>Total Sprints</t>
         </is>
       </c>
-      <c r="C2" s="15" t="inlineStr">
+      <c r="C2" s="24" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="D2" s="15" t="inlineStr">
+      <c r="D2" s="24" t="inlineStr">
         <is>
           <t>Remaining</t>
         </is>
       </c>
-      <c r="E2" s="15" t="inlineStr">
+      <c r="E2" s="24" t="inlineStr">
         <is>
           <t>% Complete</t>
         </is>
       </c>
-      <c r="F2" s="15" t="inlineStr">
+      <c r="F2" s="24" t="inlineStr">
         <is>
           <t>Total LOE</t>
         </is>
       </c>
-      <c r="G2" s="15" t="inlineStr">
+      <c r="G2" s="24" t="inlineStr">
         <is>
           <t>LOE Completed</t>
         </is>
       </c>
-      <c r="H2" s="15" t="inlineStr">
+      <c r="H2" s="24" t="inlineStr">
         <is>
           <t>LOE Remaining</t>
         </is>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="13">
-      <c r="B3" s="16">
-        <f>COUNTA(SprintCatalog[Sprint Code])</f>
-        <v/>
-      </c>
-      <c r="C3" s="16">
-        <f>COUNTIF(SprintCatalog[Implementation Status],"Complete")</f>
-        <v/>
-      </c>
-      <c r="D3" s="16">
-        <f>B3-C3</f>
-        <v/>
-      </c>
-      <c r="E3" s="17">
-        <f>C3/B3</f>
-        <v/>
-      </c>
-      <c r="F3" s="16">
-        <f>SUM(SprintCatalog[LOE])</f>
-        <v/>
-      </c>
-      <c r="G3" s="16">
-        <f>SUMPRODUCT((SprintCatalog[Implementation Status]="Complete")*SprintCatalog[LOE])</f>
-        <v/>
-      </c>
-      <c r="H3" s="16">
-        <f>F3-G3</f>
-        <v/>
+      <c r="B3" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="C3" s="16" t="n">
+        <v>13</v>
+      </c>
+      <c r="D3" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="E3" s="17" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="F3" s="16" t="n">
+        <v>57</v>
+      </c>
+      <c r="G3" s="16" t="n">
+        <v>38</v>
+      </c>
+      <c r="H3" s="16" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="24" t="inlineStr">
+        <is>
+          <t>Queue Source of Truth</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>docs/governance/sprint-queue.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="24" t="inlineStr">
+        <is>
+          <t>Queue Depth</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="24" t="inlineStr">
+        <is>
+          <t>Next Sprint</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>TTS-RENDER-MAP-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="24" t="inlineStr">
+        <is>
+          <t>Last Updated</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1365,9 +1422,7 @@
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="13">
-      <c r="A13" s="20" t="n">
-        <v>1</v>
-      </c>
+      <c r="A13" s="20" t="n"/>
       <c r="B13" s="20" t="inlineStr">
         <is>
           <t>TTS-EVENT-SYNC-1</t>
@@ -1398,7 +1453,7 @@
       </c>
       <c r="H13" s="20" t="inlineStr">
         <is>
-          <t>Queued</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="I13" s="20" t="inlineStr">
@@ -1411,20 +1466,30 @@
           <t>Event-driven word sync from research</t>
         </is>
       </c>
-      <c r="K13" s="20" t="n"/>
+      <c r="K13" s="20" t="inlineStr">
+        <is>
+          <t>sprint/tts-event-sync-1-word-boundary-sync</t>
+        </is>
+      </c>
       <c r="L13" s="20" t="n"/>
-      <c r="M13" s="20" t="n"/>
-      <c r="N13" s="20" t="n"/>
+      <c r="M13" s="20" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="N13" s="20" t="inlineStr">
+        <is>
+          <t>docs/governance/close-outs/CloseOut.TTS-EVENT-SYNC-1.2026-05-16.md</t>
+        </is>
+      </c>
       <c r="O13" s="20" t="inlineStr">
         <is>
-          <t>Research: readest + RealtimeTTS + sioyek</t>
+          <t>Research: readest + RealtimeTTS + sioyek; landed a71df02 via 2c946ad; governance commit 800c9e2</t>
         </is>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="13">
-      <c r="A14" s="20" t="n">
-        <v>2</v>
-      </c>
+      <c r="A14" s="20" t="n"/>
       <c r="B14" s="20" t="inlineStr">
         <is>
           <t>NORMALIZER-ENRICH-1</t>
@@ -1455,7 +1520,7 @@
       </c>
       <c r="H14" s="20" t="inlineStr">
         <is>
-          <t>Queued</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="I14" s="20" t="inlineStr">
@@ -1468,19 +1533,31 @@
           <t>Fill normalizer gaps from abogen research</t>
         </is>
       </c>
-      <c r="K14" s="20" t="n"/>
+      <c r="K14" s="20" t="inlineStr">
+        <is>
+          <t>sprint/normalizer-enrich-1-kokoro-text-normalization</t>
+        </is>
+      </c>
       <c r="L14" s="20" t="n"/>
-      <c r="M14" s="20" t="n"/>
-      <c r="N14" s="20" t="n"/>
+      <c r="M14" s="20" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="N14" s="20" t="inlineStr">
+        <is>
+          <t>docs/governance/close-outs/CloseOut.NORMALIZER-ENRICH-1.2026-05-17.md</t>
+        </is>
+      </c>
       <c r="O14" s="20" t="inlineStr">
         <is>
-          <t>Research: abogen</t>
+          <t>Research: abogen. Landed de5b441, merged dcf8a7d, governance closeout 2c7ada8.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="13">
       <c r="A15" s="20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B15" s="20" t="inlineStr">
         <is>
@@ -1537,7 +1614,7 @@
     </row>
     <row r="16" ht="15" customHeight="1" s="13">
       <c r="A16" s="20" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B16" s="20" t="inlineStr">
         <is>
@@ -1590,7 +1667,7 @@
     </row>
     <row r="17" ht="15" customHeight="1" s="13">
       <c r="A17" s="20" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B17" s="20" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs: close TTS-RENDER-MAP-1 and advance queue
</commit_message>
<xml_diff>
--- a/docs/governance/sprint-queue.xlsx
+++ b/docs/governance/sprint-queue.xlsx
@@ -633,22 +633,22 @@
         <v>20</v>
       </c>
       <c r="C3" s="16" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D3" s="16" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E3" s="17" t="n">
-        <v>0.65</v>
+        <v>0.7</v>
       </c>
       <c r="F3" s="16" t="n">
         <v>57</v>
       </c>
       <c r="G3" s="16" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="H3" s="16" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5">
@@ -681,7 +681,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>TTS-RENDER-MAP-1</t>
+          <t>TTS-PIPELINE-1</t>
         </is>
       </c>
     </row>
@@ -1556,9 +1556,7 @@
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="13">
-      <c r="A15" s="20" t="n">
-        <v>1</v>
-      </c>
+      <c r="A15" s="20" t="n"/>
       <c r="B15" s="20" t="inlineStr">
         <is>
           <t>TTS-RENDER-MAP-1</t>
@@ -1589,7 +1587,7 @@
       </c>
       <c r="H15" s="20" t="inlineStr">
         <is>
-          <t>Queued</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="I15" s="20" t="inlineStr">
@@ -1602,19 +1600,35 @@
           <t>Sioyek-inspired word position index</t>
         </is>
       </c>
-      <c r="K15" s="20" t="n"/>
-      <c r="L15" s="20" t="n"/>
-      <c r="M15" s="20" t="n"/>
-      <c r="N15" s="20" t="n"/>
+      <c r="K15" s="20" t="inlineStr">
+        <is>
+          <t>sprint/tts-render-map-1-word-position-index</t>
+        </is>
+      </c>
+      <c r="L15" s="20" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="M15" s="20" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="N15" s="20" t="inlineStr">
+        <is>
+          <t>docs/governance/close-outs/CloseOut.TTS-RENDER-MAP-1.2026-05-17.md</t>
+        </is>
+      </c>
       <c r="O15" s="20" t="inlineStr">
         <is>
-          <t>Research: sioyek</t>
+          <t>Research: sioyek. Landed 2eabf36, merged 8545895.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="13">
       <c r="A16" s="20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B16" s="20" t="inlineStr">
         <is>
@@ -1667,7 +1681,7 @@
     </row>
     <row r="17" ht="15" customHeight="1" s="13">
       <c r="A17" s="20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B17" s="20" t="inlineStr">
         <is>
@@ -1848,7 +1862,9 @@
       </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="13">
-      <c r="A21" s="23" t="n"/>
+      <c r="A21" s="23" t="n">
+        <v>3</v>
+      </c>
       <c r="B21" s="23" t="inlineStr">
         <is>
           <t>KOKORO-EXPORT-1</t>

</xml_diff>

<commit_message>
docs: close TTS-PIPELINE-1 and advance queue
</commit_message>
<xml_diff>
--- a/docs/governance/sprint-queue.xlsx
+++ b/docs/governance/sprint-queue.xlsx
@@ -571,7 +571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="B1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="12" min="1" max="1"/>
@@ -633,22 +633,22 @@
         <v>20</v>
       </c>
       <c r="C3" s="16" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D3" s="16" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E3" s="17" t="n">
-        <v>0.7</v>
+        <v>0.75</v>
       </c>
       <c r="F3" s="16" t="n">
         <v>57</v>
       </c>
       <c r="G3" s="16" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H3" s="16" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5">
@@ -657,7 +657,7 @@
           <t>Queue Source of Truth</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="12" t="inlineStr">
         <is>
           <t>docs/governance/sprint-queue.xlsx</t>
         </is>
@@ -669,8 +669,8 @@
           <t>Queue Depth</t>
         </is>
       </c>
-      <c r="C6" t="n">
-        <v>3</v>
+      <c r="C6" s="12" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="7">
@@ -679,9 +679,9 @@
           <t>Next Sprint</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>TTS-PIPELINE-1</t>
+      <c r="C7" s="12" t="inlineStr">
+        <is>
+          <t>TTS-ARCH-DOC-1</t>
         </is>
       </c>
     </row>
@@ -691,7 +691,7 @@
           <t>Last Updated</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="12" t="inlineStr">
         <is>
           <t>2026-05-17</t>
         </is>
@@ -1627,9 +1627,7 @@
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="13">
-      <c r="A16" s="20" t="n">
-        <v>1</v>
-      </c>
+      <c r="A16" s="20" t="n"/>
       <c r="B16" s="20" t="inlineStr">
         <is>
           <t>TTS-PIPELINE-1</t>
@@ -1660,7 +1658,7 @@
       </c>
       <c r="H16" s="20" t="inlineStr">
         <is>
-          <t>Queued</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="I16" s="20" t="inlineStr">
@@ -1673,15 +1671,35 @@
           <t>End-to-end pipeline integration tests</t>
         </is>
       </c>
-      <c r="K16" s="20" t="n"/>
-      <c r="L16" s="20" t="n"/>
-      <c r="M16" s="20" t="n"/>
-      <c r="N16" s="20" t="n"/>
-      <c r="O16" s="20" t="n"/>
+      <c r="K16" s="20" t="inlineStr">
+        <is>
+          <t>sprint/tts-pipeline-1-integration-test</t>
+        </is>
+      </c>
+      <c r="L16" s="20" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="M16" s="20" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="N16" s="20" t="inlineStr">
+        <is>
+          <t>docs/governance/close-outs/CloseOut.TTS-PIPELINE-1.2026-05-17.md</t>
+        </is>
+      </c>
+      <c r="O16" s="20" t="inlineStr">
+        <is>
+          <t>Pipeline identity/integration coverage. Landed 022d161, merged 994f218.</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="13">
       <c r="A17" s="20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B17" s="20" t="inlineStr">
         <is>
@@ -1863,7 +1881,7 @@
     </row>
     <row r="21" ht="15" customHeight="1" s="13">
       <c r="A21" s="23" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B21" s="23" t="inlineStr">
         <is>
@@ -1884,13 +1902,21 @@
       <c r="F21" s="23" t="n">
         <v>8</v>
       </c>
-      <c r="G21" s="23" t="n"/>
+      <c r="G21" s="23" t="inlineStr">
+        <is>
+          <t>TTS-ARCH-DOC-1</t>
+        </is>
+      </c>
       <c r="H21" s="23" t="inlineStr">
         <is>
-          <t>Deferred</t>
-        </is>
-      </c>
-      <c r="I21" s="23" t="n"/>
+          <t>Queued</t>
+        </is>
+      </c>
+      <c r="I21" s="23" t="inlineStr">
+        <is>
+          <t>Full spec</t>
+        </is>
+      </c>
       <c r="J21" s="23" t="inlineStr">
         <is>
           <t>Long-form audio export from Kokoro</t>
@@ -1902,7 +1928,7 @@
       <c r="N21" s="23" t="n"/>
       <c r="O21" s="23" t="inlineStr">
         <is>
-          <t>Post-conveyor, deferred until TTS Architecture completes</t>
+          <t>Queued optional future pointer; dispatch only after TTS-ARCH-DOC-1 completes.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: close TTS-ARCH-DOC-1 and mark architecture complete
</commit_message>
<xml_diff>
--- a/docs/governance/sprint-queue.xlsx
+++ b/docs/governance/sprint-queue.xlsx
@@ -633,22 +633,22 @@
         <v>20</v>
       </c>
       <c r="C3" s="16" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D3" s="16" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E3" s="17" t="n">
-        <v>0.75</v>
+        <v>0.8</v>
       </c>
       <c r="F3" s="16" t="n">
         <v>57</v>
       </c>
       <c r="G3" s="16" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H3" s="16" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5">
@@ -670,7 +670,7 @@
         </is>
       </c>
       <c r="C6" s="12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -681,7 +681,7 @@
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>TTS-ARCH-DOC-1</t>
+          <t>KOKORO-EXPORT-1</t>
         </is>
       </c>
     </row>
@@ -1698,9 +1698,7 @@
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="13">
-      <c r="A17" s="20" t="n">
-        <v>1</v>
-      </c>
+      <c r="A17" s="20" t="n"/>
       <c r="B17" s="20" t="inlineStr">
         <is>
           <t>TTS-ARCH-DOC-1</t>
@@ -1731,7 +1729,7 @@
       </c>
       <c r="H17" s="20" t="inlineStr">
         <is>
-          <t>Queued</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="I17" s="20" t="inlineStr">
@@ -1744,11 +1742,31 @@
           <t>Architecture decision records for TTS</t>
         </is>
       </c>
-      <c r="K17" s="20" t="n"/>
-      <c r="L17" s="20" t="n"/>
-      <c r="M17" s="20" t="n"/>
-      <c r="N17" s="20" t="n"/>
-      <c r="O17" s="20" t="n"/>
+      <c r="K17" s="20" t="inlineStr">
+        <is>
+          <t>sprint/tts-arch-doc-1-architecture-decisions</t>
+        </is>
+      </c>
+      <c r="L17" s="20" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="M17" s="20" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="N17" s="20" t="inlineStr">
+        <is>
+          <t>docs/governance/close-outs/CloseOut.TTS-ARCH-DOC-1.2026-05-17.md</t>
+        </is>
+      </c>
+      <c r="O17" s="20" t="inlineStr">
+        <is>
+          <t>Architecture decision record. Landed 66a73b1, merged 65629bc.</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="13">
       <c r="A18" s="21" t="n"/>
@@ -1881,7 +1899,7 @@
     </row>
     <row r="21" ht="15" customHeight="1" s="13">
       <c r="A21" s="23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B21" s="23" t="inlineStr">
         <is>
@@ -1928,7 +1946,7 @@
       <c r="N21" s="23" t="n"/>
       <c r="O21" s="23" t="inlineStr">
         <is>
-          <t>Queued optional future pointer; dispatch only after TTS-ARCH-DOC-1 completes.</t>
+          <t>Optional future pointer after TTS Architecture Complete; run roadmap review/backfill before dispatch unless explicitly authorized.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: backfill queue depth and stage follow-on narration specs
</commit_message>
<xml_diff>
--- a/docs/governance/sprint-queue.xlsx
+++ b/docs/governance/sprint-queue.xlsx
@@ -368,8 +368,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SprintCatalog" displayName="SprintCatalog" ref="A1:O21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:O21"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SprintCatalog" displayName="SprintCatalog" ref="A1:O23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:O23"/>
   <tableColumns count="15">
     <tableColumn id="1" name="Seq"/>
     <tableColumn id="2" name="Sprint Code"/>
@@ -630,25 +630,25 @@
     </row>
     <row r="3" ht="15" customHeight="1" s="13">
       <c r="B3" s="16" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C3" s="16" t="n">
         <v>16</v>
       </c>
       <c r="D3" s="16" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E3" s="17" t="n">
-        <v>0.8</v>
+        <v>0.7272727273</v>
       </c>
       <c r="F3" s="16" t="n">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="G3" s="16" t="n">
         <v>43</v>
       </c>
       <c r="H3" s="16" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5">
@@ -670,7 +670,7 @@
         </is>
       </c>
       <c r="C6" s="12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7">
@@ -683,6 +683,7 @@
         <is>
           <t>KOKORO-EXPORT-1</t>
         </is>
+        <v>KOKORO-EXPORT-1</v>
       </c>
     </row>
     <row r="8">
@@ -713,7 +714,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O21"/>
+  <dimension ref="A1:O23"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="12" min="1" max="1"/>
@@ -809,7 +810,8 @@
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" s="13">
-      <c r="A2" s="19" t="n"/>
+      <c r="A2" s="19" t="n">
+      </c>
       <c r="B2" s="19" t="inlineStr">
         <is>
           <t>KOKORO-DEEPEN-1</t>
@@ -833,7 +835,8 @@
       <c r="F2" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="G2" s="19" t="n"/>
+      <c r="G2" s="19" t="n">
+      </c>
       <c r="H2" s="19" t="inlineStr">
         <is>
           <t>Complete</t>
@@ -849,18 +852,23 @@
           <t>Kokoro readiness and preflight checks</t>
         </is>
       </c>
-      <c r="K2" s="19" t="n"/>
-      <c r="L2" s="19" t="n"/>
+      <c r="K2" s="19" t="n">
+      </c>
+      <c r="L2" s="19" t="n">
+      </c>
       <c r="M2" s="19" t="inlineStr">
         <is>
           <t>2026-05-11</t>
         </is>
       </c>
-      <c r="N2" s="19" t="n"/>
-      <c r="O2" s="19" t="n"/>
+      <c r="N2" s="19" t="n">
+      </c>
+      <c r="O2" s="19" t="n">
+      </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="13">
-      <c r="A3" s="19" t="n"/>
+      <c r="A3" s="19" t="n">
+      </c>
       <c r="B3" s="19" t="inlineStr">
         <is>
           <t>KOKORO-DEEPEN-2</t>
@@ -884,7 +892,8 @@
       <c r="F3" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="G3" s="19" t="n"/>
+      <c r="G3" s="19" t="n">
+      </c>
       <c r="H3" s="19" t="inlineStr">
         <is>
           <t>Complete</t>
@@ -900,18 +909,23 @@
           <t>Natural chunk highlighting for Kokoro TTS</t>
         </is>
       </c>
-      <c r="K3" s="19" t="n"/>
-      <c r="L3" s="19" t="n"/>
+      <c r="K3" s="19" t="n">
+      </c>
+      <c r="L3" s="19" t="n">
+      </c>
       <c r="M3" s="19" t="inlineStr">
         <is>
           <t>2026-05-11</t>
         </is>
       </c>
-      <c r="N3" s="19" t="n"/>
-      <c r="O3" s="19" t="n"/>
+      <c r="N3" s="19" t="n">
+      </c>
+      <c r="O3" s="19" t="n">
+      </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="13">
-      <c r="A4" s="19" t="n"/>
+      <c r="A4" s="19" t="n">
+      </c>
       <c r="B4" s="19" t="inlineStr">
         <is>
           <t>KOKORO-DEEPEN-3</t>
@@ -935,7 +949,8 @@
       <c r="F4" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="G4" s="19" t="n"/>
+      <c r="G4" s="19" t="n">
+      </c>
       <c r="H4" s="19" t="inlineStr">
         <is>
           <t>Complete</t>
@@ -951,18 +966,23 @@
           <t>Voice mixing feasibility study</t>
         </is>
       </c>
-      <c r="K4" s="19" t="n"/>
-      <c r="L4" s="19" t="n"/>
+      <c r="K4" s="19" t="n">
+      </c>
+      <c r="L4" s="19" t="n">
+      </c>
       <c r="M4" s="19" t="inlineStr">
         <is>
           <t>2026-05-11</t>
         </is>
       </c>
-      <c r="N4" s="19" t="n"/>
-      <c r="O4" s="19" t="n"/>
+      <c r="N4" s="19" t="n">
+      </c>
+      <c r="O4" s="19" t="n">
+      </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="13">
-      <c r="A5" s="19" t="n"/>
+      <c r="A5" s="19" t="n">
+      </c>
       <c r="B5" s="19" t="inlineStr">
         <is>
           <t>TTS-REGISTRY-1</t>
@@ -986,7 +1006,8 @@
       <c r="F5" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="G5" s="19" t="n"/>
+      <c r="G5" s="19" t="n">
+      </c>
       <c r="H5" s="19" t="inlineStr">
         <is>
           <t>Complete</t>
@@ -1002,8 +1023,10 @@
           <t>Provider capability truth in ttsProviderRegistry</t>
         </is>
       </c>
-      <c r="K5" s="19" t="n"/>
-      <c r="L5" s="19" t="n"/>
+      <c r="K5" s="19" t="n">
+      </c>
+      <c r="L5" s="19" t="n">
+      </c>
       <c r="M5" s="19" t="inlineStr">
         <is>
           <t>2026-05-12</t>
@@ -1014,10 +1037,12 @@
           <t>ROADMAP_ARCHIVE_2026-05-14.md</t>
         </is>
       </c>
-      <c r="O5" s="19" t="n"/>
+      <c r="O5" s="19" t="n">
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="13">
-      <c r="A6" s="19" t="n"/>
+      <c r="A6" s="19" t="n">
+      </c>
       <c r="B6" s="19" t="inlineStr">
         <is>
           <t>TTS-NORMALIZE-1</t>
@@ -1041,7 +1066,8 @@
       <c r="F6" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="G6" s="19" t="n"/>
+      <c r="G6" s="19" t="n">
+      </c>
       <c r="H6" s="19" t="inlineStr">
         <is>
           <t>Complete</t>
@@ -1057,8 +1083,10 @@
           <t>English-first spoken-text normalization</t>
         </is>
       </c>
-      <c r="K6" s="19" t="n"/>
-      <c r="L6" s="19" t="n"/>
+      <c r="K6" s="19" t="n">
+      </c>
+      <c r="L6" s="19" t="n">
+      </c>
       <c r="M6" s="19" t="inlineStr">
         <is>
           <t>2026-05-13</t>
@@ -1069,10 +1097,12 @@
           <t>ROADMAP_ARCHIVE_2026-05-14.md</t>
         </is>
       </c>
-      <c r="O6" s="19" t="n"/>
+      <c r="O6" s="19" t="n">
+      </c>
     </row>
     <row r="7" ht="23.25" customHeight="1" s="13">
-      <c r="A7" s="19" t="n"/>
+      <c r="A7" s="19" t="n">
+      </c>
       <c r="B7" s="19" t="inlineStr">
         <is>
           <t>TTS-CACHE-TIMING-1</t>
@@ -1096,7 +1126,8 @@
       <c r="F7" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="G7" s="19" t="n"/>
+      <c r="G7" s="19" t="n">
+      </c>
       <c r="H7" s="19" t="inlineStr">
         <is>
           <t>Complete</t>
@@ -1112,8 +1143,10 @@
           <t>Schema-versioned v2 cache identities and atomic timing sidecars</t>
         </is>
       </c>
-      <c r="K7" s="19" t="n"/>
-      <c r="L7" s="19" t="n"/>
+      <c r="K7" s="19" t="n">
+      </c>
+      <c r="L7" s="19" t="n">
+      </c>
       <c r="M7" s="19" t="inlineStr">
         <is>
           <t>2026-05-13</t>
@@ -1124,10 +1157,12 @@
           <t>ROADMAP_ARCHIVE_2026-05-14.md</t>
         </is>
       </c>
-      <c r="O7" s="19" t="n"/>
+      <c r="O7" s="19" t="n">
+      </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="13">
-      <c r="A8" s="19" t="n"/>
+      <c r="A8" s="19" t="n">
+      </c>
       <c r="B8" s="19" t="inlineStr">
         <is>
           <t>TTS-SYNC-1</t>
@@ -1176,7 +1211,8 @@
           <t>sprint/tts-sync-1-highlight-controller</t>
         </is>
       </c>
-      <c r="L8" s="19" t="n"/>
+      <c r="L8" s="19" t="n">
+      </c>
       <c r="M8" s="19" t="inlineStr">
         <is>
           <t>2026-05-15</t>
@@ -1187,10 +1223,12 @@
           <t>docs/Close-Outs/CloseOut.TTS-SYNC-1.2026-05-15.md</t>
         </is>
       </c>
-      <c r="O8" s="19" t="n"/>
+      <c r="O8" s="19" t="n">
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="13">
-      <c r="A9" s="19" t="n"/>
+      <c r="A9" s="19" t="n">
+      </c>
       <c r="B9" s="19" t="inlineStr">
         <is>
           <t>TTS-DIAG-1</t>
@@ -1239,7 +1277,8 @@
           <t>sprint/tts-diag-1-diagnostics-bundle</t>
         </is>
       </c>
-      <c r="L9" s="19" t="n"/>
+      <c r="L9" s="19" t="n">
+      </c>
       <c r="M9" s="19" t="inlineStr">
         <is>
           <t>2026-05-15</t>
@@ -1250,10 +1289,12 @@
           <t>docs/Close-Outs/CloseOut.TTS-DIAG-1.2026-05-15.md</t>
         </is>
       </c>
-      <c r="O9" s="19" t="n"/>
+      <c r="O9" s="19" t="n">
+      </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="13">
-      <c r="A10" s="20" t="n"/>
+      <c r="A10" s="20" t="n">
+      </c>
       <c r="B10" s="20" t="inlineStr">
         <is>
           <t>ENGINE-DORMANCY-1</t>
@@ -1297,8 +1338,10 @@
           <t>Disable dormant sidecar engines</t>
         </is>
       </c>
-      <c r="K10" s="20" t="n"/>
-      <c r="L10" s="20" t="n"/>
+      <c r="K10" s="20" t="n">
+      </c>
+      <c r="L10" s="20" t="n">
+      </c>
       <c r="M10" s="20" t="inlineStr">
         <is>
           <t>2026-05-16</t>
@@ -1316,7 +1359,8 @@
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="13">
-      <c r="A11" s="20" t="n"/>
+      <c r="A11" s="20" t="n">
+      </c>
       <c r="B11" s="20" t="inlineStr">
         <is>
           <t>TTS-INTEGRATE-1</t>
@@ -1360,10 +1404,14 @@
           <t>Merge sync and diagnostics branches to main</t>
         </is>
       </c>
-      <c r="K11" s="20" t="n"/>
-      <c r="L11" s="20" t="n"/>
-      <c r="M11" s="20" t="n"/>
-      <c r="N11" s="20" t="n"/>
+      <c r="K11" s="20" t="n">
+      </c>
+      <c r="L11" s="20" t="n">
+      </c>
+      <c r="M11" s="20" t="n">
+      </c>
+      <c r="N11" s="20" t="n">
+      </c>
       <c r="O11" s="20" t="inlineStr">
         <is>
           <t>Dispatch-ready; dormancy gate complete.</t>
@@ -1371,7 +1419,8 @@
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="13">
-      <c r="A12" s="12" t="n"/>
+      <c r="A12" s="12" t="n">
+      </c>
       <c r="B12" s="12" t="inlineStr">
         <is>
           <t>TTS-CACHE-HARDEN-1</t>
@@ -1422,7 +1471,8 @@
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="13">
-      <c r="A13" s="20" t="n"/>
+      <c r="A13" s="20" t="n">
+      </c>
       <c r="B13" s="20" t="inlineStr">
         <is>
           <t>TTS-EVENT-SYNC-1</t>
@@ -1471,7 +1521,8 @@
           <t>sprint/tts-event-sync-1-word-boundary-sync</t>
         </is>
       </c>
-      <c r="L13" s="20" t="n"/>
+      <c r="L13" s="20" t="n">
+      </c>
       <c r="M13" s="20" t="inlineStr">
         <is>
           <t>2026-05-16</t>
@@ -1489,7 +1540,8 @@
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="13">
-      <c r="A14" s="20" t="n"/>
+      <c r="A14" s="20" t="n">
+      </c>
       <c r="B14" s="20" t="inlineStr">
         <is>
           <t>NORMALIZER-ENRICH-1</t>
@@ -1538,7 +1590,8 @@
           <t>sprint/normalizer-enrich-1-kokoro-text-normalization</t>
         </is>
       </c>
-      <c r="L14" s="20" t="n"/>
+      <c r="L14" s="20" t="n">
+      </c>
       <c r="M14" s="20" t="inlineStr">
         <is>
           <t>2026-05-17</t>
@@ -1556,7 +1609,8 @@
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="13">
-      <c r="A15" s="20" t="n"/>
+      <c r="A15" s="20" t="n">
+      </c>
       <c r="B15" s="20" t="inlineStr">
         <is>
           <t>TTS-RENDER-MAP-1</t>
@@ -1627,7 +1681,8 @@
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="13">
-      <c r="A16" s="20" t="n"/>
+      <c r="A16" s="20" t="n">
+      </c>
       <c r="B16" s="20" t="inlineStr">
         <is>
           <t>TTS-PIPELINE-1</t>
@@ -1698,7 +1753,8 @@
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="13">
-      <c r="A17" s="20" t="n"/>
+      <c r="A17" s="20" t="n">
+      </c>
       <c r="B17" s="20" t="inlineStr">
         <is>
           <t>TTS-ARCH-DOC-1</t>
@@ -1769,7 +1825,8 @@
       </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="13">
-      <c r="A18" s="21" t="n"/>
+      <c r="A18" s="21" t="n">
+      </c>
       <c r="B18" s="22" t="inlineStr">
         <is>
           <t>TEST-HARNESS-1</t>
@@ -1785,26 +1842,33 @@
           <t>TTS Architecture</t>
         </is>
       </c>
-      <c r="E18" s="21" t="n"/>
+      <c r="E18" s="21" t="n">
+      </c>
       <c r="F18" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="G18" s="21" t="n"/>
+      <c r="G18" s="21" t="n">
+      </c>
       <c r="H18" s="21" t="inlineStr">
         <is>
           <t>Dissolved</t>
         </is>
       </c>
-      <c r="I18" s="21" t="n"/>
+      <c r="I18" s="21" t="n">
+      </c>
       <c r="J18" s="21" t="inlineStr">
         <is>
           <t>Test harness stability work</t>
         </is>
       </c>
-      <c r="K18" s="21" t="n"/>
-      <c r="L18" s="21" t="n"/>
-      <c r="M18" s="21" t="n"/>
-      <c r="N18" s="21" t="n"/>
+      <c r="K18" s="21" t="n">
+      </c>
+      <c r="L18" s="21" t="n">
+      </c>
+      <c r="M18" s="21" t="n">
+      </c>
+      <c r="N18" s="21" t="n">
+      </c>
       <c r="O18" s="21" t="inlineStr">
         <is>
           <t>Dissolved 2026-05-15 — Nano probes irrelevant</t>
@@ -1812,7 +1876,8 @@
       </c>
     </row>
     <row r="19" ht="23.25" customHeight="1" s="13">
-      <c r="A19" s="21" t="n"/>
+      <c r="A19" s="21" t="n">
+      </c>
       <c r="B19" s="22" t="inlineStr">
         <is>
           <t>TTS-CANARY-1</t>
@@ -1828,26 +1893,33 @@
           <t>TTS Architecture</t>
         </is>
       </c>
-      <c r="E19" s="21" t="n"/>
+      <c r="E19" s="21" t="n">
+      </c>
       <c r="F19" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="G19" s="21" t="n"/>
+      <c r="G19" s="21" t="n">
+      </c>
       <c r="H19" s="21" t="inlineStr">
         <is>
           <t>Dissolved</t>
         </is>
       </c>
-      <c r="I19" s="21" t="n"/>
+      <c r="I19" s="21" t="n">
+      </c>
       <c r="J19" s="21" t="inlineStr">
         <is>
           <t>Engine readiness probe system</t>
         </is>
       </c>
-      <c r="K19" s="21" t="n"/>
-      <c r="L19" s="21" t="n"/>
-      <c r="M19" s="21" t="n"/>
-      <c r="N19" s="21" t="n"/>
+      <c r="K19" s="21" t="n">
+      </c>
+      <c r="L19" s="21" t="n">
+      </c>
+      <c r="M19" s="21" t="n">
+      </c>
+      <c r="N19" s="21" t="n">
+      </c>
       <c r="O19" s="21" t="inlineStr">
         <is>
           <t>Dissolved 2026-05-15 — sidecar engines dormant</t>
@@ -1855,7 +1927,8 @@
       </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="13">
-      <c r="A20" s="21" t="n"/>
+      <c r="A20" s="21" t="n">
+      </c>
       <c r="B20" s="22" t="inlineStr">
         <is>
           <t>TTS-REGISTRY-DISPATCH-1</t>
@@ -1871,26 +1944,33 @@
           <t>TTS Architecture</t>
         </is>
       </c>
-      <c r="E20" s="21" t="n"/>
+      <c r="E20" s="21" t="n">
+      </c>
       <c r="F20" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="G20" s="21" t="n"/>
+      <c r="G20" s="21" t="n">
+      </c>
       <c r="H20" s="21" t="inlineStr">
         <is>
           <t>Dissolved</t>
         </is>
       </c>
-      <c r="I20" s="21" t="n"/>
+      <c r="I20" s="21" t="n">
+      </c>
       <c r="J20" s="21" t="inlineStr">
         <is>
           <t>Registry-driven engine dispatch</t>
         </is>
       </c>
-      <c r="K20" s="21" t="n"/>
-      <c r="L20" s="21" t="n"/>
-      <c r="M20" s="21" t="n"/>
-      <c r="N20" s="21" t="n"/>
+      <c r="K20" s="21" t="n">
+      </c>
+      <c r="L20" s="21" t="n">
+      </c>
+      <c r="M20" s="21" t="n">
+      </c>
+      <c r="N20" s="21" t="n">
+      </c>
       <c r="O20" s="21" t="inlineStr">
         <is>
           <t>Dissolved 2026-05-15 — single active engine</t>
@@ -1916,7 +1996,8 @@
           <t>TTS Architecture</t>
         </is>
       </c>
-      <c r="E21" s="23" t="n"/>
+      <c r="E21" s="23" t="n">
+      </c>
       <c r="F21" s="23" t="n">
         <v>8</v>
       </c>
@@ -1940,13 +2021,131 @@
           <t>Long-form audio export from Kokoro</t>
         </is>
       </c>
-      <c r="K21" s="23" t="n"/>
-      <c r="L21" s="23" t="n"/>
-      <c r="M21" s="23" t="n"/>
-      <c r="N21" s="23" t="n"/>
+      <c r="K21" s="23" t="n">
+      </c>
+      <c r="L21" s="23" t="n">
+      </c>
+      <c r="M21" s="23" t="n">
+      </c>
+      <c r="N21" s="23" t="n">
+      </c>
       <c r="O21" s="23" t="inlineStr">
         <is>
           <t>Optional future pointer after TTS Architecture Complete; run roadmap review/backfill before dispatch unless explicitly authorized.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="15" customHeight="1" s="13">
+      <c r="A22" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="B22" s="23" t="inlineStr">
+        <is>
+          <t>NARR-MEDIA-1</t>
+        </is>
+      </c>
+      <c r="C22" s="23" t="inlineStr">
+        <is>
+          <t>MediaSession Controls</t>
+        </is>
+      </c>
+      <c r="D22" s="23" t="inlineStr">
+        <is>
+          <t>Narration UX</t>
+        </is>
+      </c>
+      <c r="E22" s="23" t="inlineStr">
+        <is>
+          <t>Post-Architecture Polish</t>
+        </is>
+      </c>
+      <c r="F22" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" s="23" t="inlineStr">
+        <is>
+          <t>TTS-ARCH-DOC-1</t>
+        </is>
+      </c>
+      <c r="H22" s="23" t="inlineStr">
+        <is>
+          <t>Queued</t>
+        </is>
+      </c>
+      <c r="I22" s="23" t="inlineStr">
+        <is>
+          <t>Full spec</t>
+        </is>
+      </c>
+      <c r="J22" s="23" t="inlineStr">
+        <is>
+          <t>OS media transport controls for active narration</t>
+        </is>
+      </c>
+      <c r="K22" s="23" t="n"/>
+      <c r="L22" s="23" t="n"/>
+      <c r="M22" s="23" t="n"/>
+      <c r="N22" s="23" t="n"/>
+      <c r="O22" s="23" t="inlineStr">
+        <is>
+          <t>Backfill sprint from IDEAS H7; keep queue depth &gt;=3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="15" customHeight="1" s="13">
+      <c r="A23" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="B23" s="23" t="inlineStr">
+        <is>
+          <t>NARR-PAUSE-STATE-1</t>
+        </is>
+      </c>
+      <c r="C23" s="23" t="inlineStr">
+        <is>
+          <t>Named Pause State Machine</t>
+        </is>
+      </c>
+      <c r="D23" s="23" t="inlineStr">
+        <is>
+          <t>Narration UX</t>
+        </is>
+      </c>
+      <c r="E23" s="23" t="inlineStr">
+        <is>
+          <t>Post-Architecture Polish</t>
+        </is>
+      </c>
+      <c r="F23" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="G23" s="23" t="inlineStr">
+        <is>
+          <t>NARR-MEDIA-1</t>
+        </is>
+      </c>
+      <c r="H23" s="23" t="inlineStr">
+        <is>
+          <t>Queued</t>
+        </is>
+      </c>
+      <c r="I23" s="23" t="inlineStr">
+        <is>
+          <t>Full spec</t>
+        </is>
+      </c>
+      <c r="J23" s="23" t="inlineStr">
+        <is>
+          <t>Reason-aware pause and resume state transitions</t>
+        </is>
+      </c>
+      <c r="K23" s="23" t="n"/>
+      <c r="L23" s="23" t="n"/>
+      <c r="M23" s="23" t="n"/>
+      <c r="N23" s="23" t="n"/>
+      <c r="O23" s="23" t="inlineStr">
+        <is>
+          <t>Backfill sprint from IDEAS H8; dispatch after media controls foundation.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(roadmap-review): establish TTS Quality + Reading Exp v2 finish line
- Full roadmap review ceremony (Phases A-D)
- 5 full specs: NARR-MEDIA-1, NARR-PAUSE-1, NARR-CURSOR-2, TTS-EVAL-3, NARR-SPOKEN-1
- 2 stubs: UX-POLISH-1, TTS-QUAL-CI-1
- Archived 8 completed TTS Architecture sprint specs
- sprint-queue.xlsx: 7 new rows, queue GREEN depth 7
- KOKORO-EXPORT-1 close-out (implementation-complete, merge-deferred)
- SRL-040: worktree rebase-readiness checklist lesson
</commit_message>
<xml_diff>
--- a/docs/governance/sprint-queue.xlsx
+++ b/docs/governance/sprint-queue.xlsx
@@ -630,7 +630,7 @@
     </row>
     <row r="3" ht="15" customHeight="1" s="13">
       <c r="B3" s="16" t="n">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="C3" s="16" t="n">
         <v>16</v>
@@ -664,10 +664,8 @@
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="24" t="inlineStr">
-        <is>
-          <t>Queue Depth</t>
-        </is>
+      <c r="B6" s="24" t="n">
+        <v>8</v>
       </c>
       <c r="C6" s="12" t="n">
         <v>3</v>
@@ -676,20 +674,19 @@
     <row r="7">
       <c r="B7" s="24" t="inlineStr">
         <is>
-          <t>Next Sprint</t>
+          <t>NARR-MEDIA-1</t>
         </is>
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
           <t>KOKORO-EXPORT-1</t>
         </is>
-        <v>KOKORO-EXPORT-1</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="24" t="inlineStr">
         <is>
-          <t>Last Updated</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="C8" s="12" t="inlineStr">
@@ -714,7 +711,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O23"/>
+  <dimension ref="A1:O30"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="12" min="1" max="1"/>
@@ -810,8 +807,7 @@
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" s="13">
-      <c r="A2" s="19" t="n">
-      </c>
+      <c r="A2" s="19" t="n"/>
       <c r="B2" s="19" t="inlineStr">
         <is>
           <t>KOKORO-DEEPEN-1</t>
@@ -835,8 +831,7 @@
       <c r="F2" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="G2" s="19" t="n">
-      </c>
+      <c r="G2" s="19" t="n"/>
       <c r="H2" s="19" t="inlineStr">
         <is>
           <t>Complete</t>
@@ -852,23 +847,18 @@
           <t>Kokoro readiness and preflight checks</t>
         </is>
       </c>
-      <c r="K2" s="19" t="n">
-      </c>
-      <c r="L2" s="19" t="n">
-      </c>
+      <c r="K2" s="19" t="n"/>
+      <c r="L2" s="19" t="n"/>
       <c r="M2" s="19" t="inlineStr">
         <is>
           <t>2026-05-11</t>
         </is>
       </c>
-      <c r="N2" s="19" t="n">
-      </c>
-      <c r="O2" s="19" t="n">
-      </c>
+      <c r="N2" s="19" t="n"/>
+      <c r="O2" s="19" t="n"/>
     </row>
     <row r="3" ht="15" customHeight="1" s="13">
-      <c r="A3" s="19" t="n">
-      </c>
+      <c r="A3" s="19" t="n"/>
       <c r="B3" s="19" t="inlineStr">
         <is>
           <t>KOKORO-DEEPEN-2</t>
@@ -892,8 +882,7 @@
       <c r="F3" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="G3" s="19" t="n">
-      </c>
+      <c r="G3" s="19" t="n"/>
       <c r="H3" s="19" t="inlineStr">
         <is>
           <t>Complete</t>
@@ -909,23 +898,18 @@
           <t>Natural chunk highlighting for Kokoro TTS</t>
         </is>
       </c>
-      <c r="K3" s="19" t="n">
-      </c>
-      <c r="L3" s="19" t="n">
-      </c>
+      <c r="K3" s="19" t="n"/>
+      <c r="L3" s="19" t="n"/>
       <c r="M3" s="19" t="inlineStr">
         <is>
           <t>2026-05-11</t>
         </is>
       </c>
-      <c r="N3" s="19" t="n">
-      </c>
-      <c r="O3" s="19" t="n">
-      </c>
+      <c r="N3" s="19" t="n"/>
+      <c r="O3" s="19" t="n"/>
     </row>
     <row r="4" ht="15" customHeight="1" s="13">
-      <c r="A4" s="19" t="n">
-      </c>
+      <c r="A4" s="19" t="n"/>
       <c r="B4" s="19" t="inlineStr">
         <is>
           <t>KOKORO-DEEPEN-3</t>
@@ -949,8 +933,7 @@
       <c r="F4" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="G4" s="19" t="n">
-      </c>
+      <c r="G4" s="19" t="n"/>
       <c r="H4" s="19" t="inlineStr">
         <is>
           <t>Complete</t>
@@ -966,23 +949,18 @@
           <t>Voice mixing feasibility study</t>
         </is>
       </c>
-      <c r="K4" s="19" t="n">
-      </c>
-      <c r="L4" s="19" t="n">
-      </c>
+      <c r="K4" s="19" t="n"/>
+      <c r="L4" s="19" t="n"/>
       <c r="M4" s="19" t="inlineStr">
         <is>
           <t>2026-05-11</t>
         </is>
       </c>
-      <c r="N4" s="19" t="n">
-      </c>
-      <c r="O4" s="19" t="n">
-      </c>
+      <c r="N4" s="19" t="n"/>
+      <c r="O4" s="19" t="n"/>
     </row>
     <row r="5" ht="15" customHeight="1" s="13">
-      <c r="A5" s="19" t="n">
-      </c>
+      <c r="A5" s="19" t="n"/>
       <c r="B5" s="19" t="inlineStr">
         <is>
           <t>TTS-REGISTRY-1</t>
@@ -1006,8 +984,7 @@
       <c r="F5" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="G5" s="19" t="n">
-      </c>
+      <c r="G5" s="19" t="n"/>
       <c r="H5" s="19" t="inlineStr">
         <is>
           <t>Complete</t>
@@ -1023,10 +1000,8 @@
           <t>Provider capability truth in ttsProviderRegistry</t>
         </is>
       </c>
-      <c r="K5" s="19" t="n">
-      </c>
-      <c r="L5" s="19" t="n">
-      </c>
+      <c r="K5" s="19" t="n"/>
+      <c r="L5" s="19" t="n"/>
       <c r="M5" s="19" t="inlineStr">
         <is>
           <t>2026-05-12</t>
@@ -1037,12 +1012,10 @@
           <t>ROADMAP_ARCHIVE_2026-05-14.md</t>
         </is>
       </c>
-      <c r="O5" s="19" t="n">
-      </c>
+      <c r="O5" s="19" t="n"/>
     </row>
     <row r="6" ht="15" customHeight="1" s="13">
-      <c r="A6" s="19" t="n">
-      </c>
+      <c r="A6" s="19" t="n"/>
       <c r="B6" s="19" t="inlineStr">
         <is>
           <t>TTS-NORMALIZE-1</t>
@@ -1066,8 +1039,7 @@
       <c r="F6" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="G6" s="19" t="n">
-      </c>
+      <c r="G6" s="19" t="n"/>
       <c r="H6" s="19" t="inlineStr">
         <is>
           <t>Complete</t>
@@ -1083,10 +1055,8 @@
           <t>English-first spoken-text normalization</t>
         </is>
       </c>
-      <c r="K6" s="19" t="n">
-      </c>
-      <c r="L6" s="19" t="n">
-      </c>
+      <c r="K6" s="19" t="n"/>
+      <c r="L6" s="19" t="n"/>
       <c r="M6" s="19" t="inlineStr">
         <is>
           <t>2026-05-13</t>
@@ -1097,12 +1067,10 @@
           <t>ROADMAP_ARCHIVE_2026-05-14.md</t>
         </is>
       </c>
-      <c r="O6" s="19" t="n">
-      </c>
+      <c r="O6" s="19" t="n"/>
     </row>
     <row r="7" ht="23.25" customHeight="1" s="13">
-      <c r="A7" s="19" t="n">
-      </c>
+      <c r="A7" s="19" t="n"/>
       <c r="B7" s="19" t="inlineStr">
         <is>
           <t>TTS-CACHE-TIMING-1</t>
@@ -1126,8 +1094,7 @@
       <c r="F7" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="G7" s="19" t="n">
-      </c>
+      <c r="G7" s="19" t="n"/>
       <c r="H7" s="19" t="inlineStr">
         <is>
           <t>Complete</t>
@@ -1143,10 +1110,8 @@
           <t>Schema-versioned v2 cache identities and atomic timing sidecars</t>
         </is>
       </c>
-      <c r="K7" s="19" t="n">
-      </c>
-      <c r="L7" s="19" t="n">
-      </c>
+      <c r="K7" s="19" t="n"/>
+      <c r="L7" s="19" t="n"/>
       <c r="M7" s="19" t="inlineStr">
         <is>
           <t>2026-05-13</t>
@@ -1157,12 +1122,10 @@
           <t>ROADMAP_ARCHIVE_2026-05-14.md</t>
         </is>
       </c>
-      <c r="O7" s="19" t="n">
-      </c>
+      <c r="O7" s="19" t="n"/>
     </row>
     <row r="8" ht="15" customHeight="1" s="13">
-      <c r="A8" s="19" t="n">
-      </c>
+      <c r="A8" s="19" t="n"/>
       <c r="B8" s="19" t="inlineStr">
         <is>
           <t>TTS-SYNC-1</t>
@@ -1211,8 +1174,7 @@
           <t>sprint/tts-sync-1-highlight-controller</t>
         </is>
       </c>
-      <c r="L8" s="19" t="n">
-      </c>
+      <c r="L8" s="19" t="n"/>
       <c r="M8" s="19" t="inlineStr">
         <is>
           <t>2026-05-15</t>
@@ -1223,12 +1185,10 @@
           <t>docs/Close-Outs/CloseOut.TTS-SYNC-1.2026-05-15.md</t>
         </is>
       </c>
-      <c r="O8" s="19" t="n">
-      </c>
+      <c r="O8" s="19" t="n"/>
     </row>
     <row r="9" ht="15" customHeight="1" s="13">
-      <c r="A9" s="19" t="n">
-      </c>
+      <c r="A9" s="19" t="n"/>
       <c r="B9" s="19" t="inlineStr">
         <is>
           <t>TTS-DIAG-1</t>
@@ -1277,8 +1237,7 @@
           <t>sprint/tts-diag-1-diagnostics-bundle</t>
         </is>
       </c>
-      <c r="L9" s="19" t="n">
-      </c>
+      <c r="L9" s="19" t="n"/>
       <c r="M9" s="19" t="inlineStr">
         <is>
           <t>2026-05-15</t>
@@ -1289,12 +1248,10 @@
           <t>docs/Close-Outs/CloseOut.TTS-DIAG-1.2026-05-15.md</t>
         </is>
       </c>
-      <c r="O9" s="19" t="n">
-      </c>
+      <c r="O9" s="19" t="n"/>
     </row>
     <row r="10" ht="15" customHeight="1" s="13">
-      <c r="A10" s="20" t="n">
-      </c>
+      <c r="A10" s="20" t="n"/>
       <c r="B10" s="20" t="inlineStr">
         <is>
           <t>ENGINE-DORMANCY-1</t>
@@ -1338,10 +1295,8 @@
           <t>Disable dormant sidecar engines</t>
         </is>
       </c>
-      <c r="K10" s="20" t="n">
-      </c>
-      <c r="L10" s="20" t="n">
-      </c>
+      <c r="K10" s="20" t="n"/>
+      <c r="L10" s="20" t="n"/>
       <c r="M10" s="20" t="inlineStr">
         <is>
           <t>2026-05-16</t>
@@ -1359,8 +1314,7 @@
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="13">
-      <c r="A11" s="20" t="n">
-      </c>
+      <c r="A11" s="20" t="n"/>
       <c r="B11" s="20" t="inlineStr">
         <is>
           <t>TTS-INTEGRATE-1</t>
@@ -1404,14 +1358,10 @@
           <t>Merge sync and diagnostics branches to main</t>
         </is>
       </c>
-      <c r="K11" s="20" t="n">
-      </c>
-      <c r="L11" s="20" t="n">
-      </c>
-      <c r="M11" s="20" t="n">
-      </c>
-      <c r="N11" s="20" t="n">
-      </c>
+      <c r="K11" s="20" t="n"/>
+      <c r="L11" s="20" t="n"/>
+      <c r="M11" s="20" t="n"/>
+      <c r="N11" s="20" t="n"/>
       <c r="O11" s="20" t="inlineStr">
         <is>
           <t>Dispatch-ready; dormancy gate complete.</t>
@@ -1419,8 +1369,7 @@
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="13">
-      <c r="A12" s="12" t="n">
-      </c>
+      <c r="A12" s="12" t="n"/>
       <c r="B12" s="12" t="inlineStr">
         <is>
           <t>TTS-CACHE-HARDEN-1</t>
@@ -1471,8 +1420,7 @@
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="13">
-      <c r="A13" s="20" t="n">
-      </c>
+      <c r="A13" s="20" t="n"/>
       <c r="B13" s="20" t="inlineStr">
         <is>
           <t>TTS-EVENT-SYNC-1</t>
@@ -1521,8 +1469,7 @@
           <t>sprint/tts-event-sync-1-word-boundary-sync</t>
         </is>
       </c>
-      <c r="L13" s="20" t="n">
-      </c>
+      <c r="L13" s="20" t="n"/>
       <c r="M13" s="20" t="inlineStr">
         <is>
           <t>2026-05-16</t>
@@ -1540,8 +1487,7 @@
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="13">
-      <c r="A14" s="20" t="n">
-      </c>
+      <c r="A14" s="20" t="n"/>
       <c r="B14" s="20" t="inlineStr">
         <is>
           <t>NORMALIZER-ENRICH-1</t>
@@ -1590,8 +1536,7 @@
           <t>sprint/normalizer-enrich-1-kokoro-text-normalization</t>
         </is>
       </c>
-      <c r="L14" s="20" t="n">
-      </c>
+      <c r="L14" s="20" t="n"/>
       <c r="M14" s="20" t="inlineStr">
         <is>
           <t>2026-05-17</t>
@@ -1609,8 +1554,7 @@
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="13">
-      <c r="A15" s="20" t="n">
-      </c>
+      <c r="A15" s="20" t="n"/>
       <c r="B15" s="20" t="inlineStr">
         <is>
           <t>TTS-RENDER-MAP-1</t>
@@ -1681,8 +1625,7 @@
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="13">
-      <c r="A16" s="20" t="n">
-      </c>
+      <c r="A16" s="20" t="n"/>
       <c r="B16" s="20" t="inlineStr">
         <is>
           <t>TTS-PIPELINE-1</t>
@@ -1753,8 +1696,7 @@
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="13">
-      <c r="A17" s="20" t="n">
-      </c>
+      <c r="A17" s="20" t="n"/>
       <c r="B17" s="20" t="inlineStr">
         <is>
           <t>TTS-ARCH-DOC-1</t>
@@ -1825,8 +1767,7 @@
       </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="13">
-      <c r="A18" s="21" t="n">
-      </c>
+      <c r="A18" s="21" t="n"/>
       <c r="B18" s="22" t="inlineStr">
         <is>
           <t>TEST-HARNESS-1</t>
@@ -1842,33 +1783,26 @@
           <t>TTS Architecture</t>
         </is>
       </c>
-      <c r="E18" s="21" t="n">
-      </c>
+      <c r="E18" s="21" t="n"/>
       <c r="F18" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="G18" s="21" t="n">
-      </c>
+      <c r="G18" s="21" t="n"/>
       <c r="H18" s="21" t="inlineStr">
         <is>
           <t>Dissolved</t>
         </is>
       </c>
-      <c r="I18" s="21" t="n">
-      </c>
+      <c r="I18" s="21" t="n"/>
       <c r="J18" s="21" t="inlineStr">
         <is>
           <t>Test harness stability work</t>
         </is>
       </c>
-      <c r="K18" s="21" t="n">
-      </c>
-      <c r="L18" s="21" t="n">
-      </c>
-      <c r="M18" s="21" t="n">
-      </c>
-      <c r="N18" s="21" t="n">
-      </c>
+      <c r="K18" s="21" t="n"/>
+      <c r="L18" s="21" t="n"/>
+      <c r="M18" s="21" t="n"/>
+      <c r="N18" s="21" t="n"/>
       <c r="O18" s="21" t="inlineStr">
         <is>
           <t>Dissolved 2026-05-15 — Nano probes irrelevant</t>
@@ -1876,8 +1810,7 @@
       </c>
     </row>
     <row r="19" ht="23.25" customHeight="1" s="13">
-      <c r="A19" s="21" t="n">
-      </c>
+      <c r="A19" s="21" t="n"/>
       <c r="B19" s="22" t="inlineStr">
         <is>
           <t>TTS-CANARY-1</t>
@@ -1893,33 +1826,26 @@
           <t>TTS Architecture</t>
         </is>
       </c>
-      <c r="E19" s="21" t="n">
-      </c>
+      <c r="E19" s="21" t="n"/>
       <c r="F19" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="G19" s="21" t="n">
-      </c>
+      <c r="G19" s="21" t="n"/>
       <c r="H19" s="21" t="inlineStr">
         <is>
           <t>Dissolved</t>
         </is>
       </c>
-      <c r="I19" s="21" t="n">
-      </c>
+      <c r="I19" s="21" t="n"/>
       <c r="J19" s="21" t="inlineStr">
         <is>
           <t>Engine readiness probe system</t>
         </is>
       </c>
-      <c r="K19" s="21" t="n">
-      </c>
-      <c r="L19" s="21" t="n">
-      </c>
-      <c r="M19" s="21" t="n">
-      </c>
-      <c r="N19" s="21" t="n">
-      </c>
+      <c r="K19" s="21" t="n"/>
+      <c r="L19" s="21" t="n"/>
+      <c r="M19" s="21" t="n"/>
+      <c r="N19" s="21" t="n"/>
       <c r="O19" s="21" t="inlineStr">
         <is>
           <t>Dissolved 2026-05-15 — sidecar engines dormant</t>
@@ -1927,8 +1853,7 @@
       </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="13">
-      <c r="A20" s="21" t="n">
-      </c>
+      <c r="A20" s="21" t="n"/>
       <c r="B20" s="22" t="inlineStr">
         <is>
           <t>TTS-REGISTRY-DISPATCH-1</t>
@@ -1944,33 +1869,26 @@
           <t>TTS Architecture</t>
         </is>
       </c>
-      <c r="E20" s="21" t="n">
-      </c>
+      <c r="E20" s="21" t="n"/>
       <c r="F20" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="G20" s="21" t="n">
-      </c>
+      <c r="G20" s="21" t="n"/>
       <c r="H20" s="21" t="inlineStr">
         <is>
           <t>Dissolved</t>
         </is>
       </c>
-      <c r="I20" s="21" t="n">
-      </c>
+      <c r="I20" s="21" t="n"/>
       <c r="J20" s="21" t="inlineStr">
         <is>
           <t>Registry-driven engine dispatch</t>
         </is>
       </c>
-      <c r="K20" s="21" t="n">
-      </c>
-      <c r="L20" s="21" t="n">
-      </c>
-      <c r="M20" s="21" t="n">
-      </c>
-      <c r="N20" s="21" t="n">
-      </c>
+      <c r="K20" s="21" t="n"/>
+      <c r="L20" s="21" t="n"/>
+      <c r="M20" s="21" t="n"/>
+      <c r="N20" s="21" t="n"/>
       <c r="O20" s="21" t="inlineStr">
         <is>
           <t>Dissolved 2026-05-15 — single active engine</t>
@@ -1978,9 +1896,7 @@
       </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="13">
-      <c r="A21" s="23" t="n">
-        <v>1</v>
-      </c>
+      <c r="A21" s="23" t="n"/>
       <c r="B21" s="23" t="inlineStr">
         <is>
           <t>KOKORO-EXPORT-1</t>
@@ -1996,8 +1912,7 @@
           <t>TTS Architecture</t>
         </is>
       </c>
-      <c r="E21" s="23" t="n">
-      </c>
+      <c r="E21" s="23" t="n"/>
       <c r="F21" s="23" t="n">
         <v>8</v>
       </c>
@@ -2008,7 +1923,7 @@
       </c>
       <c r="H21" s="23" t="inlineStr">
         <is>
-          <t>Queued</t>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="I21" s="23" t="inlineStr">
@@ -2021,17 +1936,13 @@
           <t>Long-form audio export from Kokoro</t>
         </is>
       </c>
-      <c r="K21" s="23" t="n">
-      </c>
-      <c r="L21" s="23" t="n">
-      </c>
-      <c r="M21" s="23" t="n">
-      </c>
-      <c r="N21" s="23" t="n">
-      </c>
+      <c r="K21" s="23" t="n"/>
+      <c r="L21" s="23" t="n"/>
+      <c r="M21" s="23" t="n"/>
+      <c r="N21" s="23" t="n"/>
       <c r="O21" s="23" t="inlineStr">
         <is>
-          <t>Optional future pointer after TTS Architecture Complete; run roadmap review/backfill before dispatch unless explicitly authorized.</t>
+          <t>Deferred to post-TTS-Architecture phase. Worktree preserved at .worktrees/kokoro-export-1 (37 tests pass).</t>
         </is>
       </c>
     </row>
@@ -2126,7 +2037,7 @@
       </c>
       <c r="H23" s="23" t="inlineStr">
         <is>
-          <t>Queued</t>
+          <t>Dissolved</t>
         </is>
       </c>
       <c r="I23" s="23" t="inlineStr">
@@ -2145,9 +2056,386 @@
       <c r="N23" s="23" t="n"/>
       <c r="O23" s="23" t="inlineStr">
         <is>
-          <t>Backfill sprint from IDEAS H8; dispatch after media controls foundation.</t>
-        </is>
-      </c>
+          <t>Superseded by new TTS Quality + Reading Exp v2 conveyor (2026-05-17)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>NARR-MEDIA-1</t>
+        </is>
+      </c>
+      <c r="C24" s="12" t="inlineStr">
+        <is>
+          <t>MediaSession Integration</t>
+        </is>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
+        <is>
+          <t>TTS Quality + Reading Exp v2</t>
+        </is>
+      </c>
+      <c r="E24" s="12" t="inlineStr">
+        <is>
+          <t>1a</t>
+        </is>
+      </c>
+      <c r="F24" s="12" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G24" s="12" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H24" s="12" t="inlineStr">
+        <is>
+          <t>Queued</t>
+        </is>
+      </c>
+      <c r="I24" s="12" t="inlineStr">
+        <is>
+          <t>Full Spec</t>
+        </is>
+      </c>
+      <c r="J24" s="12" t="inlineStr">
+        <is>
+          <t>OS media controls via Electron MediaSession API</t>
+        </is>
+      </c>
+      <c r="K24" s="12" t="inlineStr">
+        <is>
+          <t>sprint/narr-media-1-mediasession</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="B25" s="12" t="inlineStr">
+        <is>
+          <t>NARR-PAUSE-1</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="inlineStr">
+        <is>
+          <t>Named-Pause State Machine</t>
+        </is>
+      </c>
+      <c r="D25" s="12" t="inlineStr">
+        <is>
+          <t>TTS Quality + Reading Exp v2</t>
+        </is>
+      </c>
+      <c r="E25" s="12" t="inlineStr">
+        <is>
+          <t>1a</t>
+        </is>
+      </c>
+      <c r="F25" s="12" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="G25" s="12" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H25" s="12" t="inlineStr">
+        <is>
+          <t>Queued</t>
+        </is>
+      </c>
+      <c r="I25" s="12" t="inlineStr">
+        <is>
+          <t>Full Spec</t>
+        </is>
+      </c>
+      <c r="J25" s="12" t="inlineStr">
+        <is>
+          <t>PauseReason discriminant for smarter resume behavior</t>
+        </is>
+      </c>
+      <c r="K25" s="12" t="inlineStr">
+        <is>
+          <t>sprint/narr-pause-1-named-pause</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="B26" s="12" t="inlineStr">
+        <is>
+          <t>NARR-CURSOR-2</t>
+        </is>
+      </c>
+      <c r="C26" s="12" t="inlineStr">
+        <is>
+          <t>Silence-Aware Cursor Hold</t>
+        </is>
+      </c>
+      <c r="D26" s="12" t="inlineStr">
+        <is>
+          <t>TTS Quality + Reading Exp v2</t>
+        </is>
+      </c>
+      <c r="E26" s="12" t="inlineStr">
+        <is>
+          <t>1a</t>
+        </is>
+      </c>
+      <c r="F26" s="12" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G26" s="12" t="inlineStr">
+        <is>
+          <t>NARR-MEDIA-1</t>
+        </is>
+      </c>
+      <c r="H26" s="12" t="inlineStr">
+        <is>
+          <t>Queued</t>
+        </is>
+      </c>
+      <c r="I26" s="12" t="inlineStr">
+        <is>
+          <t>Full Spec</t>
+        </is>
+      </c>
+      <c r="J26" s="12" t="inlineStr">
+        <is>
+          <t>Freeze cursor during inter-word silence using real endTime timestamps</t>
+        </is>
+      </c>
+      <c r="K26" s="12" t="inlineStr">
+        <is>
+          <t>sprint/narr-cursor-2-silence-hold</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B27" s="12" t="inlineStr">
+        <is>
+          <t>TTS-EVAL-3</t>
+        </is>
+      </c>
+      <c r="C27" s="12" t="inlineStr">
+        <is>
+          <t>Quality Evaluation + CI Gate</t>
+        </is>
+      </c>
+      <c r="D27" s="12" t="inlineStr">
+        <is>
+          <t>TTS Quality + Reading Exp v2</t>
+        </is>
+      </c>
+      <c r="E27" s="12" t="inlineStr">
+        <is>
+          <t>1b</t>
+        </is>
+      </c>
+      <c r="F27" s="12" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="G27" s="12" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H27" s="12" t="inlineStr">
+        <is>
+          <t>Queued</t>
+        </is>
+      </c>
+      <c r="I27" s="12" t="inlineStr">
+        <is>
+          <t>Full Spec</t>
+        </is>
+      </c>
+      <c r="J27" s="12" t="inlineStr">
+        <is>
+          <t>Extend eval harness with quality scoring dimensions and CI gate config</t>
+        </is>
+      </c>
+      <c r="K27" s="12" t="inlineStr">
+        <is>
+          <t>sprint/tts-eval-3-quality-ci-gate</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="B28" s="12" t="inlineStr">
+        <is>
+          <t>NARR-SPOKEN-1</t>
+        </is>
+      </c>
+      <c r="C28" s="12" t="inlineStr">
+        <is>
+          <t>Spoken/Display Word Separation</t>
+        </is>
+      </c>
+      <c r="D28" s="12" t="inlineStr">
+        <is>
+          <t>TTS Quality + Reading Exp v2</t>
+        </is>
+      </c>
+      <c r="E28" s="12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F28" s="12" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="G28" s="12" t="inlineStr">
+        <is>
+          <t>NARR-CURSOR-2</t>
+        </is>
+      </c>
+      <c r="H28" s="12" t="inlineStr">
+        <is>
+          <t>Queued</t>
+        </is>
+      </c>
+      <c r="I28" s="12" t="inlineStr">
+        <is>
+          <t>Full Spec</t>
+        </is>
+      </c>
+      <c r="J28" s="12" t="inlineStr">
+        <is>
+          <t>Filter punctuation-only tokens from phoneme alignment input</t>
+        </is>
+      </c>
+      <c r="K28" s="12" t="inlineStr">
+        <is>
+          <t>sprint/narr-spoken-1-word-separation</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="B29" s="12" t="inlineStr">
+        <is>
+          <t>UX-POLISH-1</t>
+        </is>
+      </c>
+      <c r="C29" s="12" t="inlineStr">
+        <is>
+          <t>Library Cards + Command Palette + Space-Bar Mode</t>
+        </is>
+      </c>
+      <c r="D29" s="12" t="inlineStr">
+        <is>
+          <t>TTS Quality + Reading Exp v2</t>
+        </is>
+      </c>
+      <c r="E29" s="12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F29" s="12" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G29" s="12" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H29" s="12" t="inlineStr">
+        <is>
+          <t>Queued</t>
+        </is>
+      </c>
+      <c r="I29" s="12" t="inlineStr">
+        <is>
+          <t>Stub</t>
+        </is>
+      </c>
+      <c r="J29" s="12" t="inlineStr">
+        <is>
+          <t>Reading experience UX improvements batch</t>
+        </is>
+      </c>
+      <c r="K29" s="12" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="B30" s="12" t="inlineStr">
+        <is>
+          <t>TTS-QUAL-CI-1</t>
+        </is>
+      </c>
+      <c r="C30" s="12" t="inlineStr">
+        <is>
+          <t>CI Regression Gate Wiring</t>
+        </is>
+      </c>
+      <c r="D30" s="12" t="inlineStr">
+        <is>
+          <t>TTS Quality + Reading Exp v2</t>
+        </is>
+      </c>
+      <c r="E30" s="12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F30" s="12" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G30" s="12" t="inlineStr">
+        <is>
+          <t>TTS-EVAL-3</t>
+        </is>
+      </c>
+      <c r="H30" s="12" t="inlineStr">
+        <is>
+          <t>Queued</t>
+        </is>
+      </c>
+      <c r="I30" s="12" t="inlineStr">
+        <is>
+          <t>Stub</t>
+        </is>
+      </c>
+      <c r="J30" s="12" t="inlineStr">
+        <is>
+          <t>Wire quality gates into GitHub Actions CI pipeline</t>
+        </is>
+      </c>
+      <c r="K30" s="12" t="inlineStr"/>
     </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>

</xml_diff>

<commit_message>
docs: close NARR-PAUSE-1 and advance queue
</commit_message>
<xml_diff>
--- a/docs/governance/sprint-queue.xlsx
+++ b/docs/governance/sprint-queue.xlsx
@@ -2108,9 +2108,7 @@
       </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="13">
-      <c r="A25" s="12" t="n">
-        <v>1</v>
-      </c>
+      <c r="A25" s="12" t="n"/>
       <c r="B25" s="12" t="inlineStr">
         <is>
           <t>NARR-PAUSE-1</t>
@@ -2143,7 +2141,7 @@
       </c>
       <c r="H25" s="12" t="inlineStr">
         <is>
-          <t>Queued</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="I25" s="12" t="inlineStr">
@@ -2159,12 +2157,22 @@
       <c r="K25" s="12" t="inlineStr">
         <is>
           <t>sprint/narr-pause-1-named-pause</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>CloseOut.NARR-PAUSE-1.2026-05-18.md</t>
         </is>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="13">
       <c r="A26" s="12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B26" s="12" t="inlineStr">
         <is>
@@ -2224,7 +2232,7 @@
     </row>
     <row r="27" ht="15" customHeight="1" s="13">
       <c r="A27" s="12" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B27" s="12" t="inlineStr">
         <is>
@@ -2279,7 +2287,7 @@
     </row>
     <row r="28" ht="15" customHeight="1" s="13">
       <c r="A28" s="12" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B28" s="12" t="inlineStr">
         <is>
@@ -2334,7 +2342,7 @@
     </row>
     <row r="29" ht="15" customHeight="1" s="13">
       <c r="A29" s="12" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B29" s="12" t="inlineStr">
         <is>
@@ -2389,7 +2397,7 @@
     </row>
     <row r="30" ht="15" customHeight="1" s="13">
       <c r="A30" s="12" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B30" s="12" t="inlineStr">
         <is>
@@ -2439,7 +2447,7 @@
     </row>
     <row r="31" ht="15" customHeight="1" s="13">
       <c r="A31" s="12" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B31" s="12" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs(governance): close-out NARR-MEDIA-1, NARR-PAUSE-1, TTS-PARITY-1, NARR-SPOKEN-1 + status checkin
</commit_message>
<xml_diff>
--- a/docs/governance/sprint-queue.xlsx
+++ b/docs/governance/sprint-queue.xlsx
@@ -17,7 +17,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+  </numFmts>
   <fonts count="10">
     <font>
       <name val="Calibri"/>
@@ -154,7 +156,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -225,6 +227,7 @@
     <xf numFmtId="0" fontId="8" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2159,21 +2162,19 @@
           <t>sprint/narr-pause-1-named-pause</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr">
+      <c r="M25" s="12" t="inlineStr">
         <is>
           <t>2026-05-18</t>
         </is>
       </c>
-      <c r="N25" t="inlineStr">
+      <c r="N25" s="12" t="inlineStr">
         <is>
           <t>CloseOut.NARR-PAUSE-1.2026-05-18.md</t>
         </is>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="13">
-      <c r="A26" s="12" t="n">
-        <v>1</v>
-      </c>
+      <c r="A26" s="12" t="n"/>
       <c r="B26" s="12" t="inlineStr">
         <is>
           <t>TTS-PARITY-1</t>
@@ -2206,7 +2207,7 @@
       </c>
       <c r="H26" s="12" t="inlineStr">
         <is>
-          <t>Queued</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="I26" s="12" t="inlineStr">
@@ -2222,6 +2223,14 @@
       <c r="K26" s="12" t="inlineStr">
         <is>
           <t>sprint/tts-parity-1</t>
+        </is>
+      </c>
+      <c r="M26" s="24" t="n">
+        <v>46160</v>
+      </c>
+      <c r="N26" s="12" t="inlineStr">
+        <is>
+          <t>CloseOut.TTS-PARITY-1.2026-05-18.md</t>
         </is>
       </c>
       <c r="O26" s="12" t="inlineStr">
@@ -2232,7 +2241,7 @@
     </row>
     <row r="27" ht="15" customHeight="1" s="13">
       <c r="A27" s="12" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B27" s="12" t="inlineStr">
         <is>
@@ -2287,7 +2296,7 @@
     </row>
     <row r="28" ht="15" customHeight="1" s="13">
       <c r="A28" s="12" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B28" s="12" t="inlineStr">
         <is>
@@ -2341,9 +2350,7 @@
       </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="13">
-      <c r="A29" s="12" t="n">
-        <v>2</v>
-      </c>
+      <c r="A29" s="12" t="n"/>
       <c r="B29" s="12" t="inlineStr">
         <is>
           <t>NARR-SPOKEN-1</t>
@@ -2376,7 +2383,7 @@
       </c>
       <c r="H29" s="12" t="inlineStr">
         <is>
-          <t>Queued</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="I29" s="12" t="inlineStr">
@@ -2392,12 +2399,22 @@
       <c r="K29" s="12" t="inlineStr">
         <is>
           <t>sprint/narr-spoken-1</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>CloseOut.NARR-SPOKEN-1.2026-05-18.md</t>
         </is>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="13">
       <c r="A30" s="12" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B30" s="12" t="inlineStr">
         <is>
@@ -2447,7 +2464,7 @@
     </row>
     <row r="31" ht="15" customHeight="1" s="13">
       <c r="A31" s="12" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B31" s="12" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs: NARR-CURSOR-2 phase closeout — close-out report, SRL-044, governance updates
</commit_message>
<xml_diff>
--- a/docs/governance/sprint-queue.xlsx
+++ b/docs/governance/sprint-queue.xlsx
@@ -2,25 +2,24 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="8880" yWindow="-20205" windowWidth="38700" windowHeight="15285" tabRatio="500" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalog" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
+  <calcPr calcId="0" fullCalcOnLoad="1" iterateDelta="0.0001"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -30,30 +29,13 @@
     </font>
     <font>
       <name val="Arial"/>
-      <family val="0"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <family val="0"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <family val="0"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
       <charset val="1"/>
-      <family val="0"/>
       <b val="1"/>
       <sz val="14"/>
     </font>
     <font>
       <name val="Cambria"/>
       <charset val="1"/>
-      <family val="0"/>
       <b val="1"/>
       <color rgb="FFFFFFFF"/>
       <sz val="11"/>
@@ -61,14 +43,12 @@
     <font>
       <name val="Arial"/>
       <charset val="1"/>
-      <family val="0"/>
       <b val="1"/>
       <sz val="12"/>
     </font>
     <font>
       <name val="Arial"/>
       <charset val="1"/>
-      <family val="0"/>
       <b val="1"/>
       <color rgb="FFFFFFFF"/>
       <sz val="10"/>
@@ -76,13 +56,11 @@
     <font>
       <name val="Arial"/>
       <charset val="1"/>
-      <family val="0"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
       <charset val="1"/>
-      <family val="0"/>
       <strike val="1"/>
       <sz val="10"/>
     </font>
@@ -146,162 +124,46 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="6">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
-      <alignment horizontal="general" vertical="bottom"/>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="13">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="43" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="41" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="44" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
-  </cellStyleXfs>
-  <cellXfs count="25">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="2" builtinId="6"/>
-    <cellStyle name="Currency" xfId="3" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="4" builtinId="7"/>
-    <cellStyle name="Percent" xfId="5" builtinId="5"/>
   </cellStyles>
-  <dxfs count="8">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF003366"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE2EFDA"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFCE4D6"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFFFF"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD9D9D9"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFF2CC"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF000000"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -360,13 +222,21 @@
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF1F4E78"/>
       <rgbColor rgb="FF333333"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
 </styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SprintCatalog" displayName="SprintCatalog" ref="A1:O23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SprintCatalog" displayName="SprintCatalog" ref="A1:O23" headerRowCount="1" totalsRowShown="0">
   <autoFilter ref="A1:O23"/>
   <tableColumns count="15">
     <tableColumn id="1" name="Seq"/>
@@ -385,11 +255,12 @@
     <tableColumn id="14" name="Close-Out File"/>
     <tableColumn id="15" name="Notes"/>
   </tableColumns>
+  <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -431,12 +302,12 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:minorFont>
@@ -465,7 +336,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="1"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -486,7 +357,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -537,7 +408,7 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
           </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -555,133 +426,135 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
           </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr filterMode="0">
+  <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
+    <pageSetUpPr/>
   </sheetPr>
   <dimension ref="B1:H8"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="3" customWidth="1" style="12" min="1" max="1"/>
     <col width="18" customWidth="1" style="12" min="2" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="17.25" customHeight="1" s="13">
-      <c r="B1" s="14" t="inlineStr">
+    <row r="1" ht="17.25" customHeight="1" s="12">
+      <c r="B1" s="11" t="inlineStr">
         <is>
           <t>TTS Architecture Completion — Sprint Dashboard</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1" s="13">
-      <c r="B2" s="15" t="inlineStr">
+    <row r="2" ht="15" customHeight="1" s="12">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>Total Sprints</t>
         </is>
       </c>
-      <c r="C2" s="15" t="inlineStr">
+      <c r="C2" s="1" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="D2" s="15" t="inlineStr">
+      <c r="D2" s="1" t="inlineStr">
         <is>
           <t>Remaining</t>
         </is>
       </c>
-      <c r="E2" s="15" t="inlineStr">
+      <c r="E2" s="1" t="inlineStr">
         <is>
           <t>% Complete</t>
         </is>
       </c>
-      <c r="F2" s="15" t="inlineStr">
+      <c r="F2" s="1" t="inlineStr">
         <is>
           <t>Total LOE</t>
         </is>
       </c>
-      <c r="G2" s="15" t="inlineStr">
+      <c r="G2" s="1" t="inlineStr">
         <is>
           <t>LOE Completed</t>
         </is>
       </c>
-      <c r="H2" s="15" t="inlineStr">
+      <c r="H2" s="1" t="inlineStr">
         <is>
           <t>LOE Remaining</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="15" customHeight="1" s="13">
-      <c r="B3" s="16" t="n">
+    <row r="3" ht="15" customHeight="1" s="12">
+      <c r="B3" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="C3" s="16" t="n">
+      <c r="C3" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="D3" s="16" t="n">
+      <c r="D3" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="E3" s="17" t="n">
+      <c r="E3" s="3" t="n">
         <v>0.7272727273</v>
       </c>
-      <c r="F3" s="16" t="n">
+      <c r="F3" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="G3" s="16" t="n">
+      <c r="G3" s="2" t="n">
         <v>43</v>
       </c>
-      <c r="H3" s="16" t="n">
+      <c r="H3" s="2" t="n">
         <v>17</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" s="13">
-      <c r="B5" s="15" t="inlineStr">
+    <row r="5" ht="15" customHeight="1" s="12">
+      <c r="B5" s="1" t="inlineStr">
         <is>
           <t>Queue Source of Truth</t>
         </is>
       </c>
-      <c r="C5" s="12" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>docs/governance/sprint-queue.xlsx</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" s="13">
-      <c r="B6" s="15" t="n">
+    <row r="6" ht="15" customHeight="1" s="12">
+      <c r="B6" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="C6" s="12" t="n">
+      <c r="C6" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" s="13">
-      <c r="B7" s="15" t="inlineStr">
+    <row r="7" ht="15" customHeight="1" s="12">
+      <c r="B7" s="1" t="inlineStr">
         <is>
           <t>NARR-MEDIA-1</t>
         </is>
       </c>
-      <c r="C7" s="12" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>KOKORO-EXPORT-1</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" s="13">
-      <c r="B8" s="15" t="inlineStr">
+    <row r="8" ht="15" customHeight="1" s="12">
+      <c r="B8" s="1" t="inlineStr">
         <is>
           <t>2026-05-17</t>
         </is>
       </c>
-      <c r="C8" s="12" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>2026-05-17</t>
         </is>
@@ -691,20 +564,19 @@
   <mergeCells count="1">
     <mergeCell ref="B1:H1"/>
   </mergeCells>
-  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr filterMode="0">
+  <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
+    <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O31"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="5" customWidth="1" style="12" min="1" max="1"/>
     <col width="22" customWidth="1" style="12" min="2" max="2"/>
@@ -715,1807 +587,1809 @@
     <col width="25" customWidth="1" style="12" min="7" max="7"/>
     <col width="20" customWidth="1" style="12" min="8" max="8"/>
     <col width="15" customWidth="1" style="12" min="9" max="9"/>
-    <col width="50" customWidth="1" style="12" min="10" max="10"/>
+    <col width="63.88671875" bestFit="1" customWidth="1" style="12" min="10" max="10"/>
     <col width="35" customWidth="1" style="12" min="11" max="11"/>
     <col width="14" customWidth="1" style="12" min="12" max="13"/>
     <col width="50" customWidth="1" style="12" min="14" max="15"/>
   </cols>
   <sheetData>
-    <row r="1" ht="23.25" customHeight="1" s="13">
-      <c r="A1" s="18" t="inlineStr">
+    <row r="1" ht="23.25" customHeight="1" s="12">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Seq</t>
         </is>
       </c>
-      <c r="B1" s="18" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>Sprint Code</t>
         </is>
       </c>
-      <c r="C1" s="18" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="D1" s="18" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>Phase</t>
         </is>
       </c>
-      <c r="E1" s="18" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>Stage</t>
         </is>
       </c>
-      <c r="F1" s="18" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>LOE</t>
         </is>
       </c>
-      <c r="G1" s="18" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>Dependencies</t>
         </is>
       </c>
-      <c r="H1" s="18" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>Implementation Status</t>
         </is>
       </c>
-      <c r="I1" s="18" t="inlineStr">
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>Written Status</t>
         </is>
       </c>
-      <c r="J1" s="18" t="inlineStr">
+      <c r="J1" s="4" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="K1" s="18" t="inlineStr">
+      <c r="K1" s="4" t="inlineStr">
         <is>
           <t>Branch</t>
         </is>
       </c>
-      <c r="L1" s="18" t="inlineStr">
+      <c r="L1" s="4" t="inlineStr">
         <is>
           <t>Date Started</t>
         </is>
       </c>
-      <c r="M1" s="18" t="inlineStr">
+      <c r="M1" s="4" t="inlineStr">
         <is>
           <t>Date Completed</t>
         </is>
       </c>
-      <c r="N1" s="18" t="inlineStr">
+      <c r="N1" s="4" t="inlineStr">
         <is>
           <t>Close-Out File</t>
         </is>
       </c>
-      <c r="O1" s="18" t="inlineStr">
+      <c r="O1" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1" s="13">
-      <c r="A2" s="19" t="n"/>
-      <c r="B2" s="19" t="inlineStr">
+    <row r="2" ht="15" customHeight="1" s="12">
+      <c r="A2" s="5" t="n"/>
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>KOKORO-DEEPEN-1</t>
         </is>
       </c>
-      <c r="C2" s="19" t="inlineStr">
+      <c r="C2" s="5" t="inlineStr">
         <is>
           <t>Kokoro Readiness &amp; Preflight</t>
         </is>
       </c>
-      <c r="D2" s="19" t="inlineStr">
+      <c r="D2" s="5" t="inlineStr">
         <is>
           <t>TTS Architecture</t>
         </is>
       </c>
-      <c r="E2" s="19" t="inlineStr">
+      <c r="E2" s="5" t="inlineStr">
         <is>
           <t>Deepening</t>
         </is>
       </c>
-      <c r="F2" s="19" t="n">
+      <c r="F2" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="G2" s="19" t="n"/>
-      <c r="H2" s="19" t="inlineStr">
+      <c r="G2" s="5" t="n"/>
+      <c r="H2" s="5" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="I2" s="19" t="inlineStr">
+      <c r="I2" s="5" t="inlineStr">
         <is>
           <t>Full spec</t>
         </is>
       </c>
-      <c r="J2" s="19" t="inlineStr">
+      <c r="J2" s="5" t="inlineStr">
         <is>
           <t>Kokoro readiness and preflight checks</t>
         </is>
       </c>
-      <c r="K2" s="19" t="n"/>
-      <c r="L2" s="19" t="n"/>
-      <c r="M2" s="19" t="inlineStr">
+      <c r="K2" s="5" t="n"/>
+      <c r="L2" s="5" t="n"/>
+      <c r="M2" s="5" t="inlineStr">
         <is>
           <t>2026-05-11</t>
         </is>
       </c>
-      <c r="N2" s="19" t="n"/>
-      <c r="O2" s="19" t="n"/>
-    </row>
-    <row r="3" ht="15" customHeight="1" s="13">
-      <c r="A3" s="19" t="n"/>
-      <c r="B3" s="19" t="inlineStr">
+      <c r="N2" s="5" t="n"/>
+      <c r="O2" s="5" t="n"/>
+    </row>
+    <row r="3" ht="15" customHeight="1" s="12">
+      <c r="A3" s="5" t="n"/>
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>KOKORO-DEEPEN-2</t>
         </is>
       </c>
-      <c r="C3" s="19" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>Natural Chunk Highlight</t>
         </is>
       </c>
-      <c r="D3" s="19" t="inlineStr">
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>TTS Architecture</t>
         </is>
       </c>
-      <c r="E3" s="19" t="inlineStr">
+      <c r="E3" s="5" t="inlineStr">
         <is>
           <t>Deepening</t>
         </is>
       </c>
-      <c r="F3" s="19" t="n">
+      <c r="F3" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="G3" s="19" t="n"/>
-      <c r="H3" s="19" t="inlineStr">
+      <c r="G3" s="5" t="n"/>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="I3" s="19" t="inlineStr">
+      <c r="I3" s="5" t="inlineStr">
         <is>
           <t>Full spec</t>
         </is>
       </c>
-      <c r="J3" s="19" t="inlineStr">
+      <c r="J3" s="5" t="inlineStr">
         <is>
           <t>Natural chunk highlighting for Kokoro TTS</t>
         </is>
       </c>
-      <c r="K3" s="19" t="n"/>
-      <c r="L3" s="19" t="n"/>
-      <c r="M3" s="19" t="inlineStr">
+      <c r="K3" s="5" t="n"/>
+      <c r="L3" s="5" t="n"/>
+      <c r="M3" s="5" t="inlineStr">
         <is>
           <t>2026-05-11</t>
         </is>
       </c>
-      <c r="N3" s="19" t="n"/>
-      <c r="O3" s="19" t="n"/>
-    </row>
-    <row r="4" ht="15" customHeight="1" s="13">
-      <c r="A4" s="19" t="n"/>
-      <c r="B4" s="19" t="inlineStr">
+      <c r="N3" s="5" t="n"/>
+      <c r="O3" s="5" t="n"/>
+    </row>
+    <row r="4" ht="15" customHeight="1" s="12">
+      <c r="A4" s="5" t="n"/>
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>KOKORO-DEEPEN-3</t>
         </is>
       </c>
-      <c r="C4" s="19" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>Voice Mixing Feasibility</t>
         </is>
       </c>
-      <c r="D4" s="19" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>TTS Architecture</t>
         </is>
       </c>
-      <c r="E4" s="19" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>Deepening</t>
         </is>
       </c>
-      <c r="F4" s="19" t="n">
+      <c r="F4" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="G4" s="19" t="n"/>
-      <c r="H4" s="19" t="inlineStr">
+      <c r="G4" s="5" t="n"/>
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="I4" s="19" t="inlineStr">
+      <c r="I4" s="5" t="inlineStr">
         <is>
           <t>Full spec</t>
         </is>
       </c>
-      <c r="J4" s="19" t="inlineStr">
+      <c r="J4" s="5" t="inlineStr">
         <is>
           <t>Voice mixing feasibility study</t>
         </is>
       </c>
-      <c r="K4" s="19" t="n"/>
-      <c r="L4" s="19" t="n"/>
-      <c r="M4" s="19" t="inlineStr">
+      <c r="K4" s="5" t="n"/>
+      <c r="L4" s="5" t="n"/>
+      <c r="M4" s="5" t="inlineStr">
         <is>
           <t>2026-05-11</t>
         </is>
       </c>
-      <c r="N4" s="19" t="n"/>
-      <c r="O4" s="19" t="n"/>
-    </row>
-    <row r="5" ht="15" customHeight="1" s="13">
-      <c r="A5" s="19" t="n"/>
-      <c r="B5" s="19" t="inlineStr">
+      <c r="N4" s="5" t="n"/>
+      <c r="O4" s="5" t="n"/>
+    </row>
+    <row r="5" ht="15" customHeight="1" s="12">
+      <c r="A5" s="5" t="n"/>
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>TTS-REGISTRY-1</t>
         </is>
       </c>
-      <c r="C5" s="19" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>Provider Capability Registry</t>
         </is>
       </c>
-      <c r="D5" s="19" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>TTS Architecture</t>
         </is>
       </c>
-      <c r="E5" s="19" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>Foundation</t>
         </is>
       </c>
-      <c r="F5" s="19" t="n">
+      <c r="F5" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="G5" s="19" t="n"/>
-      <c r="H5" s="19" t="inlineStr">
+      <c r="G5" s="5" t="n"/>
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="I5" s="19" t="inlineStr">
+      <c r="I5" s="5" t="inlineStr">
         <is>
           <t>Full spec</t>
         </is>
       </c>
-      <c r="J5" s="19" t="inlineStr">
+      <c r="J5" s="5" t="inlineStr">
         <is>
           <t>Provider capability truth in ttsProviderRegistry</t>
         </is>
       </c>
-      <c r="K5" s="19" t="n"/>
-      <c r="L5" s="19" t="n"/>
-      <c r="M5" s="19" t="inlineStr">
+      <c r="K5" s="5" t="n"/>
+      <c r="L5" s="5" t="n"/>
+      <c r="M5" s="5" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="N5" s="19" t="inlineStr">
+      <c r="N5" s="5" t="inlineStr">
         <is>
           <t>ROADMAP_ARCHIVE_2026-05-14.md</t>
         </is>
       </c>
-      <c r="O5" s="19" t="n"/>
-    </row>
-    <row r="6" ht="15" customHeight="1" s="13">
-      <c r="A6" s="19" t="n"/>
-      <c r="B6" s="19" t="inlineStr">
+      <c r="O5" s="5" t="n"/>
+    </row>
+    <row r="6" ht="15" customHeight="1" s="12">
+      <c r="A6" s="5" t="n"/>
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>TTS-NORMALIZE-1</t>
         </is>
       </c>
-      <c r="C6" s="19" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>Segment Normalizer</t>
         </is>
       </c>
-      <c r="D6" s="19" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>TTS Architecture</t>
         </is>
       </c>
-      <c r="E6" s="19" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>Foundation</t>
         </is>
       </c>
-      <c r="F6" s="19" t="n">
+      <c r="F6" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="G6" s="19" t="n"/>
-      <c r="H6" s="19" t="inlineStr">
+      <c r="G6" s="5" t="n"/>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="I6" s="19" t="inlineStr">
+      <c r="I6" s="5" t="inlineStr">
         <is>
           <t>Full spec</t>
         </is>
       </c>
-      <c r="J6" s="19" t="inlineStr">
+      <c r="J6" s="5" t="inlineStr">
         <is>
           <t>English-first spoken-text normalization</t>
         </is>
       </c>
-      <c r="K6" s="19" t="n"/>
-      <c r="L6" s="19" t="n"/>
-      <c r="M6" s="19" t="inlineStr">
+      <c r="K6" s="5" t="n"/>
+      <c r="L6" s="5" t="n"/>
+      <c r="M6" s="5" t="inlineStr">
         <is>
           <t>2026-05-13</t>
         </is>
       </c>
-      <c r="N6" s="19" t="inlineStr">
+      <c r="N6" s="5" t="inlineStr">
         <is>
           <t>ROADMAP_ARCHIVE_2026-05-14.md</t>
         </is>
       </c>
-      <c r="O6" s="19" t="n"/>
-    </row>
-    <row r="7" ht="23.25" customHeight="1" s="13">
-      <c r="A7" s="19" t="n"/>
-      <c r="B7" s="19" t="inlineStr">
+      <c r="O6" s="5" t="n"/>
+    </row>
+    <row r="7" ht="23.25" customHeight="1" s="12">
+      <c r="A7" s="5" t="n"/>
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>TTS-CACHE-TIMING-1</t>
         </is>
       </c>
-      <c r="C7" s="19" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>Cache Identity &amp; Timing Sidecars</t>
         </is>
       </c>
-      <c r="D7" s="19" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>TTS Architecture</t>
         </is>
       </c>
-      <c r="E7" s="19" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>Foundation</t>
         </is>
       </c>
-      <c r="F7" s="19" t="n">
+      <c r="F7" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="G7" s="19" t="n"/>
-      <c r="H7" s="19" t="inlineStr">
+      <c r="G7" s="5" t="n"/>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="I7" s="19" t="inlineStr">
+      <c r="I7" s="5" t="inlineStr">
         <is>
           <t>Full spec</t>
         </is>
       </c>
-      <c r="J7" s="19" t="inlineStr">
+      <c r="J7" s="5" t="inlineStr">
         <is>
           <t>Schema-versioned v2 cache identities and atomic timing sidecars</t>
         </is>
       </c>
-      <c r="K7" s="19" t="n"/>
-      <c r="L7" s="19" t="n"/>
-      <c r="M7" s="19" t="inlineStr">
+      <c r="K7" s="5" t="n"/>
+      <c r="L7" s="5" t="n"/>
+      <c r="M7" s="5" t="inlineStr">
         <is>
           <t>2026-05-13</t>
         </is>
       </c>
-      <c r="N7" s="19" t="inlineStr">
+      <c r="N7" s="5" t="inlineStr">
         <is>
           <t>ROADMAP_ARCHIVE_2026-05-14.md</t>
         </is>
       </c>
-      <c r="O7" s="19" t="n"/>
-    </row>
-    <row r="8" ht="15" customHeight="1" s="13">
-      <c r="A8" s="19" t="n"/>
-      <c r="B8" s="19" t="inlineStr">
+      <c r="O7" s="5" t="n"/>
+    </row>
+    <row r="8" ht="15" customHeight="1" s="12">
+      <c r="A8" s="5" t="n"/>
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>TTS-SYNC-1</t>
         </is>
       </c>
-      <c r="C8" s="19" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>Highlight Sync Controller</t>
         </is>
       </c>
-      <c r="D8" s="19" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>TTS Architecture</t>
         </is>
       </c>
-      <c r="E8" s="19" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>Sync &amp; Diagnostics</t>
         </is>
       </c>
-      <c r="F8" s="19" t="n">
+      <c r="F8" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="G8" s="19" t="inlineStr">
+      <c r="G8" s="5" t="inlineStr">
         <is>
           <t>TTS-CACHE-TIMING-1</t>
         </is>
       </c>
-      <c r="H8" s="19" t="inlineStr">
+      <c r="H8" s="5" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="I8" s="19" t="inlineStr">
+      <c r="I8" s="5" t="inlineStr">
         <is>
           <t>Full spec</t>
         </is>
       </c>
-      <c r="J8" s="19" t="inlineStr">
+      <c r="J8" s="5" t="inlineStr">
         <is>
           <t>Centralized narration highlight sync policy</t>
         </is>
       </c>
-      <c r="K8" s="19" t="inlineStr">
+      <c r="K8" s="5" t="inlineStr">
         <is>
           <t>sprint/tts-sync-1-highlight-controller</t>
         </is>
       </c>
-      <c r="L8" s="19" t="n"/>
-      <c r="M8" s="19" t="inlineStr">
+      <c r="L8" s="5" t="n"/>
+      <c r="M8" s="5" t="inlineStr">
         <is>
           <t>2026-05-15</t>
         </is>
       </c>
-      <c r="N8" s="19" t="inlineStr">
+      <c r="N8" s="5" t="inlineStr">
         <is>
           <t>docs/Close-Outs/CloseOut.TTS-SYNC-1.2026-05-15.md</t>
         </is>
       </c>
-      <c r="O8" s="19" t="n"/>
-    </row>
-    <row r="9" ht="15" customHeight="1" s="13">
-      <c r="A9" s="19" t="n"/>
-      <c r="B9" s="19" t="inlineStr">
+      <c r="O8" s="5" t="n"/>
+    </row>
+    <row r="9" ht="15" customHeight="1" s="12">
+      <c r="A9" s="5" t="n"/>
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>TTS-DIAG-1</t>
         </is>
       </c>
-      <c r="C9" s="19" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>Narration Diagnostics Bundle</t>
         </is>
       </c>
-      <c r="D9" s="19" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>TTS Architecture</t>
         </is>
       </c>
-      <c r="E9" s="19" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>Sync &amp; Diagnostics</t>
         </is>
       </c>
-      <c r="F9" s="19" t="n">
+      <c r="F9" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="G9" s="19" t="inlineStr">
+      <c r="G9" s="5" t="inlineStr">
         <is>
           <t>TTS-SYNC-1</t>
         </is>
       </c>
-      <c r="H9" s="19" t="inlineStr">
+      <c r="H9" s="5" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="I9" s="19" t="inlineStr">
+      <c r="I9" s="5" t="inlineStr">
         <is>
           <t>Full spec</t>
         </is>
       </c>
-      <c r="J9" s="19" t="inlineStr">
+      <c r="J9" s="5" t="inlineStr">
         <is>
           <t>Provider-neutral diagnostics bundle</t>
         </is>
       </c>
-      <c r="K9" s="19" t="inlineStr">
+      <c r="K9" s="5" t="inlineStr">
         <is>
           <t>sprint/tts-diag-1-diagnostics-bundle</t>
         </is>
       </c>
-      <c r="L9" s="19" t="n"/>
-      <c r="M9" s="19" t="inlineStr">
+      <c r="L9" s="5" t="n"/>
+      <c r="M9" s="5" t="inlineStr">
         <is>
           <t>2026-05-15</t>
         </is>
       </c>
-      <c r="N9" s="19" t="inlineStr">
+      <c r="N9" s="5" t="inlineStr">
         <is>
           <t>docs/Close-Outs/CloseOut.TTS-DIAG-1.2026-05-15.md</t>
         </is>
       </c>
-      <c r="O9" s="19" t="n"/>
-    </row>
-    <row r="10" ht="15" customHeight="1" s="13">
-      <c r="A10" s="20" t="n"/>
-      <c r="B10" s="20" t="inlineStr">
+      <c r="O9" s="5" t="n"/>
+    </row>
+    <row r="10" ht="15" customHeight="1" s="12">
+      <c r="A10" s="6" t="n"/>
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>ENGINE-DORMANCY-1</t>
         </is>
       </c>
-      <c r="C10" s="20" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>Disable MOSS-Nano &amp; Pocket TTS</t>
         </is>
       </c>
-      <c r="D10" s="20" t="inlineStr">
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>TTS Architecture</t>
         </is>
       </c>
-      <c r="E10" s="20" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>Consolidation</t>
         </is>
       </c>
-      <c r="F10" s="20" t="n">
+      <c r="F10" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="G10" s="20" t="inlineStr">
+      <c r="G10" s="6" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="H10" s="20" t="inlineStr">
+      <c r="H10" s="6" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="I10" s="20" t="inlineStr">
+      <c r="I10" s="6" t="inlineStr">
         <is>
           <t>Full spec</t>
         </is>
       </c>
-      <c r="J10" s="20" t="inlineStr">
+      <c r="J10" s="6" t="inlineStr">
         <is>
           <t>Disable dormant sidecar engines</t>
         </is>
       </c>
-      <c r="K10" s="20" t="n"/>
-      <c r="L10" s="20" t="n"/>
-      <c r="M10" s="20" t="inlineStr">
+      <c r="K10" s="6" t="n"/>
+      <c r="L10" s="6" t="n"/>
+      <c r="M10" s="6" t="inlineStr">
         <is>
           <t>2026-05-16</t>
         </is>
       </c>
-      <c r="N10" s="20" t="inlineStr">
+      <c r="N10" s="6" t="inlineStr">
         <is>
           <t>docs/governance/close-outs/CloseOut.ENGINE-DORMANCY-1.2026-05-16.md</t>
         </is>
       </c>
-      <c r="O10" s="20" t="inlineStr">
+      <c r="O10" s="6" t="inlineStr">
         <is>
           <t>Dormant at settings/IPC; code preserved; Nano probes opt-in.</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="15" customHeight="1" s="13">
-      <c r="A11" s="20" t="n"/>
-      <c r="B11" s="20" t="inlineStr">
+    <row r="11" ht="15" customHeight="1" s="12">
+      <c r="A11" s="6" t="n"/>
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>TTS-INTEGRATE-1</t>
         </is>
       </c>
-      <c r="C11" s="20" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>Integrate Sync &amp; Diagnostics</t>
         </is>
       </c>
-      <c r="D11" s="20" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>TTS Architecture</t>
         </is>
       </c>
-      <c r="E11" s="20" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>Consolidation</t>
         </is>
       </c>
-      <c r="F11" s="20" t="n">
+      <c r="F11" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="G11" s="20" t="inlineStr">
+      <c r="G11" s="6" t="inlineStr">
         <is>
           <t>ENGINE-DORMANCY-1</t>
         </is>
       </c>
-      <c r="H11" s="20" t="inlineStr">
+      <c r="H11" s="6" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="I11" s="20" t="inlineStr">
+      <c r="I11" s="6" t="inlineStr">
         <is>
           <t>Full spec</t>
         </is>
       </c>
-      <c r="J11" s="20" t="inlineStr">
+      <c r="J11" s="6" t="inlineStr">
         <is>
           <t>Merge sync and diagnostics branches to main</t>
         </is>
       </c>
-      <c r="K11" s="20" t="n"/>
-      <c r="L11" s="20" t="n"/>
-      <c r="M11" s="20" t="n"/>
-      <c r="N11" s="20" t="n"/>
-      <c r="O11" s="20" t="inlineStr">
+      <c r="K11" s="6" t="n"/>
+      <c r="L11" s="6" t="n"/>
+      <c r="M11" s="6" t="n"/>
+      <c r="N11" s="6" t="n"/>
+      <c r="O11" s="6" t="inlineStr">
         <is>
           <t>Dispatch-ready; dormancy gate complete.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1" s="13">
-      <c r="B12" s="12" t="inlineStr">
+    <row r="12" ht="15" customHeight="1" s="12">
+      <c r="B12" t="inlineStr">
         <is>
           <t>TTS-CACHE-HARDEN-1</t>
         </is>
       </c>
-      <c r="C12" s="12" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>Cache/Pipeline Hardening</t>
         </is>
       </c>
-      <c r="D12" s="12" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>TTS Architecture</t>
         </is>
       </c>
-      <c r="E12" s="12" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>Consolidation</t>
         </is>
       </c>
-      <c r="F12" s="12" t="n">
+      <c r="F12" t="n">
         <v>2</v>
       </c>
-      <c r="G12" s="12" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>TTS-INTEGRATE-1</t>
         </is>
       </c>
-      <c r="H12" s="12" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="I12" s="12" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>Full spec</t>
         </is>
       </c>
-      <c r="J12" s="12" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>Cache-hit timing parity, type harmonization, IPC validation</t>
         </is>
       </c>
-      <c r="O12" s="12" t="inlineStr">
+      <c r="O12" t="inlineStr">
         <is>
           <t>Findings-driven: impl review A8 + lit review §4.6</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="15" customHeight="1" s="13">
-      <c r="A13" s="20" t="n"/>
-      <c r="B13" s="20" t="inlineStr">
+    <row r="13" ht="15" customHeight="1" s="12">
+      <c r="A13" s="6" t="n"/>
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>TTS-EVENT-SYNC-1</t>
         </is>
       </c>
-      <c r="C13" s="20" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>Event-Driven Word Sync</t>
         </is>
       </c>
-      <c r="D13" s="20" t="inlineStr">
+      <c r="D13" s="6" t="inlineStr">
         <is>
           <t>TTS Architecture</t>
         </is>
       </c>
-      <c r="E13" s="20" t="inlineStr">
+      <c r="E13" s="6" t="inlineStr">
         <is>
           <t>Stage 2: Event-Driven Sync</t>
         </is>
       </c>
-      <c r="F13" s="20" t="n">
+      <c r="F13" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="G13" s="20" t="inlineStr">
+      <c r="G13" s="6" t="inlineStr">
         <is>
           <t>TTS-CACHE-HARDEN-1 (completed 2026-05-16)</t>
         </is>
       </c>
-      <c r="H13" s="20" t="inlineStr">
+      <c r="H13" s="6" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="I13" s="20" t="inlineStr">
+      <c r="I13" s="6" t="inlineStr">
         <is>
           <t>Full spec</t>
         </is>
       </c>
-      <c r="J13" s="20" t="inlineStr">
+      <c r="J13" s="6" t="inlineStr">
         <is>
           <t>Event-driven word sync from research</t>
         </is>
       </c>
-      <c r="K13" s="20" t="inlineStr">
+      <c r="K13" s="6" t="inlineStr">
         <is>
           <t>sprint/tts-event-sync-1-word-boundary-sync</t>
         </is>
       </c>
-      <c r="L13" s="20" t="n"/>
-      <c r="M13" s="20" t="inlineStr">
+      <c r="L13" s="6" t="n"/>
+      <c r="M13" s="6" t="inlineStr">
         <is>
           <t>2026-05-16</t>
         </is>
       </c>
-      <c r="N13" s="20" t="inlineStr">
+      <c r="N13" s="6" t="inlineStr">
         <is>
           <t>docs/governance/close-outs/CloseOut.TTS-EVENT-SYNC-1.2026-05-16.md</t>
         </is>
       </c>
-      <c r="O13" s="20" t="inlineStr">
+      <c r="O13" s="6" t="inlineStr">
         <is>
           <t>Research: readest + RealtimeTTS + sioyek; landed a71df02 via 2c946ad; governance commit 800c9e2</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="15" customHeight="1" s="13">
-      <c r="A14" s="20" t="n"/>
-      <c r="B14" s="20" t="inlineStr">
+    <row r="14" ht="15" customHeight="1" s="12">
+      <c r="A14" s="6" t="n"/>
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>NORMALIZER-ENRICH-1</t>
         </is>
       </c>
-      <c r="C14" s="20" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>Normalizer Gap Fill</t>
         </is>
       </c>
-      <c r="D14" s="20" t="inlineStr">
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>TTS Architecture</t>
         </is>
       </c>
-      <c r="E14" s="20" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr">
         <is>
           <t>Stage 2: Normalizer Enrichment</t>
         </is>
       </c>
-      <c r="F14" s="20" t="n">
+      <c r="F14" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="G14" s="20" t="inlineStr">
+      <c r="G14" s="6" t="inlineStr">
         <is>
           <t>TTS-EVENT-SYNC-1</t>
         </is>
       </c>
-      <c r="H14" s="20" t="inlineStr">
+      <c r="H14" s="6" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="I14" s="20" t="inlineStr">
+      <c r="I14" s="6" t="inlineStr">
         <is>
           <t>Full spec</t>
         </is>
       </c>
-      <c r="J14" s="20" t="inlineStr">
+      <c r="J14" s="6" t="inlineStr">
         <is>
           <t>Fill normalizer gaps from abogen research</t>
         </is>
       </c>
-      <c r="K14" s="20" t="inlineStr">
+      <c r="K14" s="6" t="inlineStr">
         <is>
           <t>sprint/normalizer-enrich-1-kokoro-text-normalization</t>
         </is>
       </c>
-      <c r="L14" s="20" t="n"/>
-      <c r="M14" s="20" t="inlineStr">
+      <c r="L14" s="6" t="n"/>
+      <c r="M14" s="6" t="inlineStr">
         <is>
           <t>2026-05-17</t>
         </is>
       </c>
-      <c r="N14" s="20" t="inlineStr">
+      <c r="N14" s="6" t="inlineStr">
         <is>
           <t>docs/governance/close-outs/CloseOut.NORMALIZER-ENRICH-1.2026-05-17.md</t>
         </is>
       </c>
-      <c r="O14" s="20" t="inlineStr">
+      <c r="O14" s="6" t="inlineStr">
         <is>
           <t>Research: abogen. Landed de5b441, merged dcf8a7d, governance closeout 2c7ada8.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="15" customHeight="1" s="13">
-      <c r="A15" s="20" t="n"/>
-      <c r="B15" s="20" t="inlineStr">
+    <row r="15" ht="15" customHeight="1" s="12">
+      <c r="A15" s="6" t="n"/>
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>TTS-RENDER-MAP-1</t>
         </is>
       </c>
-      <c r="C15" s="20" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>Word Position Index</t>
         </is>
       </c>
-      <c r="D15" s="20" t="inlineStr">
+      <c r="D15" s="6" t="inlineStr">
         <is>
           <t>TTS Architecture</t>
         </is>
       </c>
-      <c r="E15" s="20" t="inlineStr">
+      <c r="E15" s="6" t="inlineStr">
         <is>
           <t>Stage 2: Word Position Index</t>
         </is>
       </c>
-      <c r="F15" s="20" t="n">
+      <c r="F15" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="G15" s="20" t="inlineStr">
+      <c r="G15" s="6" t="inlineStr">
         <is>
           <t>NORMALIZER-ENRICH-1</t>
         </is>
       </c>
-      <c r="H15" s="20" t="inlineStr">
+      <c r="H15" s="6" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="I15" s="20" t="inlineStr">
+      <c r="I15" s="6" t="inlineStr">
         <is>
           <t>Full spec</t>
         </is>
       </c>
-      <c r="J15" s="20" t="inlineStr">
+      <c r="J15" s="6" t="inlineStr">
         <is>
           <t>Sioyek-inspired word position index</t>
         </is>
       </c>
-      <c r="K15" s="20" t="inlineStr">
+      <c r="K15" s="6" t="inlineStr">
         <is>
           <t>sprint/tts-render-map-1-word-position-index</t>
         </is>
       </c>
-      <c r="L15" s="20" t="inlineStr">
+      <c r="L15" s="6" t="inlineStr">
         <is>
           <t>2026-05-17</t>
         </is>
       </c>
-      <c r="M15" s="20" t="inlineStr">
+      <c r="M15" s="6" t="inlineStr">
         <is>
           <t>2026-05-17</t>
         </is>
       </c>
-      <c r="N15" s="20" t="inlineStr">
+      <c r="N15" s="6" t="inlineStr">
         <is>
           <t>docs/governance/close-outs/CloseOut.TTS-RENDER-MAP-1.2026-05-17.md</t>
         </is>
       </c>
-      <c r="O15" s="20" t="inlineStr">
+      <c r="O15" s="6" t="inlineStr">
         <is>
           <t>Research: sioyek. Landed 2eabf36, merged 8545895.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="15" customHeight="1" s="13">
-      <c r="A16" s="20" t="n"/>
-      <c r="B16" s="20" t="inlineStr">
+    <row r="16" ht="15" customHeight="1" s="12">
+      <c r="A16" s="6" t="n"/>
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>TTS-PIPELINE-1</t>
         </is>
       </c>
-      <c r="C16" s="20" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>Pipeline Integration Tests</t>
         </is>
       </c>
-      <c r="D16" s="20" t="inlineStr">
+      <c r="D16" s="6" t="inlineStr">
         <is>
           <t>TTS Architecture</t>
         </is>
       </c>
-      <c r="E16" s="20" t="inlineStr">
+      <c r="E16" s="6" t="inlineStr">
         <is>
           <t>Stage 3: Pipeline Truth</t>
         </is>
       </c>
-      <c r="F16" s="20" t="n">
+      <c r="F16" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="G16" s="20" t="inlineStr">
+      <c r="G16" s="6" t="inlineStr">
         <is>
           <t>TTS-RENDER-MAP-1</t>
         </is>
       </c>
-      <c r="H16" s="20" t="inlineStr">
+      <c r="H16" s="6" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="I16" s="20" t="inlineStr">
+      <c r="I16" s="6" t="inlineStr">
         <is>
           <t>Full spec</t>
         </is>
       </c>
-      <c r="J16" s="20" t="inlineStr">
+      <c r="J16" s="6" t="inlineStr">
         <is>
           <t>End-to-end pipeline integration tests</t>
         </is>
       </c>
-      <c r="K16" s="20" t="inlineStr">
+      <c r="K16" s="6" t="inlineStr">
         <is>
           <t>sprint/tts-pipeline-1-integration-test</t>
         </is>
       </c>
-      <c r="L16" s="20" t="inlineStr">
+      <c r="L16" s="6" t="inlineStr">
         <is>
           <t>2026-05-17</t>
         </is>
       </c>
-      <c r="M16" s="20" t="inlineStr">
+      <c r="M16" s="6" t="inlineStr">
         <is>
           <t>2026-05-17</t>
         </is>
       </c>
-      <c r="N16" s="20" t="inlineStr">
+      <c r="N16" s="6" t="inlineStr">
         <is>
           <t>docs/governance/close-outs/CloseOut.TTS-PIPELINE-1.2026-05-17.md</t>
         </is>
       </c>
-      <c r="O16" s="20" t="inlineStr">
+      <c r="O16" s="6" t="inlineStr">
         <is>
           <t>Pipeline identity/integration coverage. Landed 022d161, merged 994f218.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="15" customHeight="1" s="13">
-      <c r="A17" s="20" t="n"/>
-      <c r="B17" s="20" t="inlineStr">
+    <row r="17" ht="15" customHeight="1" s="12">
+      <c r="A17" s="6" t="n"/>
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>TTS-ARCH-DOC-1</t>
         </is>
       </c>
-      <c r="C17" s="20" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>Architecture Decisions Doc</t>
         </is>
       </c>
-      <c r="D17" s="20" t="inlineStr">
+      <c r="D17" s="6" t="inlineStr">
         <is>
           <t>TTS Architecture</t>
         </is>
       </c>
-      <c r="E17" s="20" t="inlineStr">
+      <c r="E17" s="6" t="inlineStr">
         <is>
           <t>Stage 4: Governance</t>
         </is>
       </c>
-      <c r="F17" s="20" t="n">
+      <c r="F17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="G17" s="20" t="inlineStr">
+      <c r="G17" s="6" t="inlineStr">
         <is>
           <t>All above</t>
         </is>
       </c>
-      <c r="H17" s="20" t="inlineStr">
+      <c r="H17" s="6" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="I17" s="20" t="inlineStr">
+      <c r="I17" s="6" t="inlineStr">
         <is>
           <t>Full spec</t>
         </is>
       </c>
-      <c r="J17" s="20" t="inlineStr">
+      <c r="J17" s="6" t="inlineStr">
         <is>
           <t>Architecture decision records for TTS</t>
         </is>
       </c>
-      <c r="K17" s="20" t="inlineStr">
+      <c r="K17" s="6" t="inlineStr">
         <is>
           <t>sprint/tts-arch-doc-1-architecture-decisions</t>
         </is>
       </c>
-      <c r="L17" s="20" t="inlineStr">
+      <c r="L17" s="6" t="inlineStr">
         <is>
           <t>2026-05-17</t>
         </is>
       </c>
-      <c r="M17" s="20" t="inlineStr">
+      <c r="M17" s="6" t="inlineStr">
         <is>
           <t>2026-05-17</t>
         </is>
       </c>
-      <c r="N17" s="20" t="inlineStr">
+      <c r="N17" s="6" t="inlineStr">
         <is>
           <t>docs/governance/close-outs/CloseOut.TTS-ARCH-DOC-1.2026-05-17.md</t>
         </is>
       </c>
-      <c r="O17" s="20" t="inlineStr">
+      <c r="O17" s="6" t="inlineStr">
         <is>
           <t>Architecture decision record. Landed 66a73b1, merged 65629bc.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="15" customHeight="1" s="13">
-      <c r="A18" s="21" t="n"/>
-      <c r="B18" s="22" t="inlineStr">
+    <row r="18" ht="15" customHeight="1" s="12">
+      <c r="A18" s="7" t="n"/>
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>TEST-HARNESS-1</t>
         </is>
       </c>
-      <c r="C18" s="21" t="inlineStr">
+      <c r="C18" s="7" t="inlineStr">
         <is>
           <t>Test Harness Stability</t>
         </is>
       </c>
-      <c r="D18" s="21" t="inlineStr">
+      <c r="D18" s="7" t="inlineStr">
         <is>
           <t>TTS Architecture</t>
         </is>
       </c>
-      <c r="E18" s="21" t="n"/>
-      <c r="F18" s="21" t="n">
+      <c r="E18" s="7" t="n"/>
+      <c r="F18" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="G18" s="21" t="n"/>
-      <c r="H18" s="21" t="inlineStr">
+      <c r="G18" s="7" t="n"/>
+      <c r="H18" s="7" t="inlineStr">
         <is>
           <t>Dissolved</t>
         </is>
       </c>
-      <c r="I18" s="21" t="n"/>
-      <c r="J18" s="21" t="inlineStr">
+      <c r="I18" s="7" t="n"/>
+      <c r="J18" s="7" t="inlineStr">
         <is>
           <t>Test harness stability work</t>
         </is>
       </c>
-      <c r="K18" s="21" t="n"/>
-      <c r="L18" s="21" t="n"/>
-      <c r="M18" s="21" t="n"/>
-      <c r="N18" s="21" t="n"/>
-      <c r="O18" s="21" t="inlineStr">
+      <c r="K18" s="7" t="n"/>
+      <c r="L18" s="7" t="n"/>
+      <c r="M18" s="7" t="n"/>
+      <c r="N18" s="7" t="n"/>
+      <c r="O18" s="7" t="inlineStr">
         <is>
           <t>Dissolved 2026-05-15 — Nano probes irrelevant</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="23.25" customHeight="1" s="13">
-      <c r="A19" s="21" t="n"/>
-      <c r="B19" s="22" t="inlineStr">
+    <row r="19" ht="23.25" customHeight="1" s="12">
+      <c r="A19" s="7" t="n"/>
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>TTS-CANARY-1</t>
         </is>
       </c>
-      <c r="C19" s="21" t="inlineStr">
+      <c r="C19" s="7" t="inlineStr">
         <is>
           <t>Engine Readiness Probes</t>
         </is>
       </c>
-      <c r="D19" s="21" t="inlineStr">
+      <c r="D19" s="7" t="inlineStr">
         <is>
           <t>TTS Architecture</t>
         </is>
       </c>
-      <c r="E19" s="21" t="n"/>
-      <c r="F19" s="21" t="n">
+      <c r="E19" s="7" t="n"/>
+      <c r="F19" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G19" s="21" t="n"/>
-      <c r="H19" s="21" t="inlineStr">
+      <c r="G19" s="7" t="n"/>
+      <c r="H19" s="7" t="inlineStr">
         <is>
           <t>Dissolved</t>
         </is>
       </c>
-      <c r="I19" s="21" t="n"/>
-      <c r="J19" s="21" t="inlineStr">
+      <c r="I19" s="7" t="n"/>
+      <c r="J19" s="7" t="inlineStr">
         <is>
           <t>Engine readiness probe system</t>
         </is>
       </c>
-      <c r="K19" s="21" t="n"/>
-      <c r="L19" s="21" t="n"/>
-      <c r="M19" s="21" t="n"/>
-      <c r="N19" s="21" t="n"/>
-      <c r="O19" s="21" t="inlineStr">
+      <c r="K19" s="7" t="n"/>
+      <c r="L19" s="7" t="n"/>
+      <c r="M19" s="7" t="n"/>
+      <c r="N19" s="7" t="n"/>
+      <c r="O19" s="7" t="inlineStr">
         <is>
           <t>Dissolved 2026-05-15 — sidecar engines dormant</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="15" customHeight="1" s="13">
-      <c r="A20" s="21" t="n"/>
-      <c r="B20" s="22" t="inlineStr">
+    <row r="20" ht="15" customHeight="1" s="12">
+      <c r="A20" s="7" t="n"/>
+      <c r="B20" s="8" t="inlineStr">
         <is>
           <t>TTS-REGISTRY-DISPATCH-1</t>
         </is>
       </c>
-      <c r="C20" s="21" t="inlineStr">
+      <c r="C20" s="7" t="inlineStr">
         <is>
           <t>Registry-Driven Dispatch</t>
         </is>
       </c>
-      <c r="D20" s="21" t="inlineStr">
+      <c r="D20" s="7" t="inlineStr">
         <is>
           <t>TTS Architecture</t>
         </is>
       </c>
-      <c r="E20" s="21" t="n"/>
-      <c r="F20" s="21" t="n">
+      <c r="E20" s="7" t="n"/>
+      <c r="F20" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="G20" s="21" t="n"/>
-      <c r="H20" s="21" t="inlineStr">
+      <c r="G20" s="7" t="n"/>
+      <c r="H20" s="7" t="inlineStr">
         <is>
           <t>Dissolved</t>
         </is>
       </c>
-      <c r="I20" s="21" t="n"/>
-      <c r="J20" s="21" t="inlineStr">
+      <c r="I20" s="7" t="n"/>
+      <c r="J20" s="7" t="inlineStr">
         <is>
           <t>Registry-driven engine dispatch</t>
         </is>
       </c>
-      <c r="K20" s="21" t="n"/>
-      <c r="L20" s="21" t="n"/>
-      <c r="M20" s="21" t="n"/>
-      <c r="N20" s="21" t="n"/>
-      <c r="O20" s="21" t="inlineStr">
+      <c r="K20" s="7" t="n"/>
+      <c r="L20" s="7" t="n"/>
+      <c r="M20" s="7" t="n"/>
+      <c r="N20" s="7" t="n"/>
+      <c r="O20" s="7" t="inlineStr">
         <is>
           <t>Dissolved 2026-05-15 — single active engine</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1" s="13">
-      <c r="A21" s="23" t="n"/>
-      <c r="B21" s="23" t="inlineStr">
+    <row r="21" ht="15" customHeight="1" s="12">
+      <c r="A21" s="9" t="n"/>
+      <c r="B21" s="9" t="inlineStr">
         <is>
           <t>KOKORO-EXPORT-1</t>
         </is>
       </c>
-      <c r="C21" s="23" t="inlineStr">
+      <c r="C21" s="9" t="inlineStr">
         <is>
           <t>Long-Form Audio Export</t>
         </is>
       </c>
-      <c r="D21" s="23" t="inlineStr">
+      <c r="D21" s="9" t="inlineStr">
         <is>
           <t>TTS Architecture</t>
         </is>
       </c>
-      <c r="E21" s="23" t="n"/>
-      <c r="F21" s="23" t="n">
+      <c r="E21" s="9" t="n"/>
+      <c r="F21" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="G21" s="23" t="inlineStr">
+      <c r="G21" s="9" t="inlineStr">
         <is>
           <t>TTS-ARCH-DOC-1</t>
         </is>
       </c>
-      <c r="H21" s="23" t="inlineStr">
+      <c r="H21" s="9" t="inlineStr">
         <is>
           <t>Blocked</t>
         </is>
       </c>
-      <c r="I21" s="23" t="inlineStr">
+      <c r="I21" s="9" t="inlineStr">
         <is>
           <t>Full spec</t>
         </is>
       </c>
-      <c r="J21" s="23" t="inlineStr">
+      <c r="J21" s="9" t="inlineStr">
         <is>
           <t>Long-form audio export from Kokoro</t>
         </is>
       </c>
-      <c r="K21" s="23" t="n"/>
-      <c r="L21" s="23" t="n"/>
-      <c r="M21" s="23" t="n"/>
-      <c r="N21" s="23" t="n"/>
-      <c r="O21" s="23" t="inlineStr">
+      <c r="K21" s="9" t="n"/>
+      <c r="L21" s="9" t="n"/>
+      <c r="M21" s="9" t="n"/>
+      <c r="N21" s="9" t="n"/>
+      <c r="O21" s="9" t="inlineStr">
         <is>
           <t>Deferred to post-TTS-Architecture phase. Worktree preserved at .worktrees/kokoro-export-1 (37 tests pass).</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="15" customHeight="1" s="13">
-      <c r="A22" s="23" t="n"/>
-      <c r="B22" s="23" t="inlineStr">
+    <row r="22" ht="15" customHeight="1" s="12">
+      <c r="A22" s="9" t="n"/>
+      <c r="B22" s="9" t="inlineStr">
         <is>
           <t>NARR-MEDIA-1</t>
         </is>
       </c>
-      <c r="C22" s="23" t="inlineStr">
+      <c r="C22" s="9" t="inlineStr">
         <is>
           <t>MediaSession Controls</t>
         </is>
       </c>
-      <c r="D22" s="23" t="inlineStr">
+      <c r="D22" s="9" t="inlineStr">
         <is>
           <t>Narration UX</t>
         </is>
       </c>
-      <c r="E22" s="23" t="inlineStr">
+      <c r="E22" s="9" t="inlineStr">
         <is>
           <t>Post-Architecture Polish</t>
         </is>
       </c>
-      <c r="F22" s="23" t="n">
+      <c r="F22" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="G22" s="23" t="inlineStr">
+      <c r="G22" s="9" t="inlineStr">
         <is>
           <t>TTS-ARCH-DOC-1</t>
         </is>
       </c>
-      <c r="H22" s="23" t="inlineStr">
+      <c r="H22" s="9" t="inlineStr">
         <is>
           <t>Dissolved</t>
         </is>
       </c>
-      <c r="I22" s="23" t="inlineStr">
+      <c r="I22" s="9" t="inlineStr">
         <is>
           <t>Full spec</t>
         </is>
       </c>
-      <c r="J22" s="23" t="inlineStr">
+      <c r="J22" s="9" t="inlineStr">
         <is>
           <t>OS media transport controls for active narration</t>
         </is>
       </c>
-      <c r="K22" s="23" t="n"/>
-      <c r="L22" s="23" t="n"/>
-      <c r="M22" s="23" t="n"/>
-      <c r="N22" s="23" t="n"/>
-      <c r="O22" s="23" t="inlineStr">
+      <c r="K22" s="9" t="n"/>
+      <c r="L22" s="9" t="n"/>
+      <c r="M22" s="9" t="n"/>
+      <c r="N22" s="9" t="n"/>
+      <c r="O22" s="9" t="inlineStr">
         <is>
           <t>Dissolved — duplicate of completed NARR-MEDIA-1 in TTS Quality phase</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="15" customHeight="1" s="13">
-      <c r="A23" s="23" t="n"/>
-      <c r="B23" s="23" t="inlineStr">
+    <row r="23" ht="15" customHeight="1" s="12">
+      <c r="A23" s="9" t="n"/>
+      <c r="B23" s="9" t="inlineStr">
         <is>
           <t>NARR-PAUSE-STATE-1</t>
         </is>
       </c>
-      <c r="C23" s="23" t="inlineStr">
+      <c r="C23" s="9" t="inlineStr">
         <is>
           <t>Named Pause State Machine</t>
         </is>
       </c>
-      <c r="D23" s="23" t="inlineStr">
+      <c r="D23" s="9" t="inlineStr">
         <is>
           <t>Narration UX</t>
         </is>
       </c>
-      <c r="E23" s="23" t="inlineStr">
+      <c r="E23" s="9" t="inlineStr">
         <is>
           <t>Post-Architecture Polish</t>
         </is>
       </c>
-      <c r="F23" s="23" t="n">
+      <c r="F23" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="G23" s="23" t="inlineStr">
+      <c r="G23" s="9" t="inlineStr">
         <is>
           <t>NARR-MEDIA-1</t>
         </is>
       </c>
-      <c r="H23" s="23" t="inlineStr">
+      <c r="H23" s="9" t="inlineStr">
         <is>
           <t>Dissolved</t>
         </is>
       </c>
-      <c r="I23" s="23" t="inlineStr">
+      <c r="I23" s="9" t="inlineStr">
         <is>
           <t>Full spec</t>
         </is>
       </c>
-      <c r="J23" s="23" t="inlineStr">
+      <c r="J23" s="9" t="inlineStr">
         <is>
           <t>Reason-aware pause and resume state transitions</t>
         </is>
       </c>
-      <c r="K23" s="23" t="n"/>
-      <c r="L23" s="23" t="n"/>
-      <c r="M23" s="23" t="n"/>
-      <c r="N23" s="23" t="n"/>
-      <c r="O23" s="23" t="inlineStr">
+      <c r="K23" s="9" t="n"/>
+      <c r="L23" s="9" t="n"/>
+      <c r="M23" s="9" t="n"/>
+      <c r="N23" s="9" t="n"/>
+      <c r="O23" s="9" t="inlineStr">
         <is>
           <t>Superseded by new TTS Quality + Reading Exp v2 conveyor (2026-05-17)</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="15" customHeight="1" s="13">
-      <c r="A24" s="12" t="n"/>
-      <c r="B24" s="12" t="inlineStr">
+    <row r="24" ht="15" customHeight="1" s="12">
+      <c r="B24" t="inlineStr">
         <is>
           <t>NARR-MEDIA-1</t>
         </is>
       </c>
-      <c r="C24" s="12" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>MediaSession Integration</t>
         </is>
       </c>
-      <c r="D24" s="12" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>TTS Quality + Reading Exp v2</t>
         </is>
       </c>
-      <c r="E24" s="12" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>1a</t>
         </is>
       </c>
-      <c r="F24" s="12" t="inlineStr">
+      <c r="F24" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="G24" s="12" t="inlineStr">
+      <c r="G24" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="H24" s="12" t="inlineStr">
+      <c r="H24" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="I24" s="12" t="inlineStr">
+      <c r="I24" t="inlineStr">
         <is>
           <t>Full Spec</t>
         </is>
       </c>
-      <c r="J24" s="12" t="inlineStr">
+      <c r="J24" t="inlineStr">
         <is>
           <t>OS media controls via Electron MediaSession API</t>
         </is>
       </c>
-      <c r="K24" s="12" t="inlineStr">
+      <c r="K24" t="inlineStr">
         <is>
           <t>sprint/narr-media-1-mediasession</t>
         </is>
       </c>
-      <c r="M24" s="12" t="inlineStr">
+      <c r="M24" t="inlineStr">
         <is>
           <t>2026-05-17</t>
         </is>
       </c>
-      <c r="N24" s="12" t="inlineStr">
+      <c r="N24" t="inlineStr">
         <is>
           <t>CloseOut.NARR-MEDIA-1.2026-05-17.md</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="15" customHeight="1" s="13">
-      <c r="A25" s="12" t="n"/>
-      <c r="B25" s="12" t="inlineStr">
+    <row r="25" ht="15" customHeight="1" s="12">
+      <c r="B25" t="inlineStr">
         <is>
           <t>NARR-PAUSE-1</t>
         </is>
       </c>
-      <c r="C25" s="12" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>Named-Pause State Machine</t>
         </is>
       </c>
-      <c r="D25" s="12" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t>TTS Quality + Reading Exp v2</t>
         </is>
       </c>
-      <c r="E25" s="12" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>1a</t>
         </is>
       </c>
-      <c r="F25" s="12" t="inlineStr">
+      <c r="F25" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="G25" s="12" t="inlineStr">
+      <c r="G25" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="H25" s="12" t="inlineStr">
+      <c r="H25" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="I25" s="12" t="inlineStr">
+      <c r="I25" t="inlineStr">
         <is>
           <t>Full Spec</t>
         </is>
       </c>
-      <c r="J25" s="12" t="inlineStr">
+      <c r="J25" t="inlineStr">
         <is>
           <t>PauseReason discriminant for smarter resume behavior</t>
         </is>
       </c>
-      <c r="K25" s="12" t="inlineStr">
+      <c r="K25" t="inlineStr">
         <is>
           <t>sprint/narr-pause-1-named-pause</t>
         </is>
       </c>
-      <c r="M25" s="12" t="inlineStr">
+      <c r="M25" t="inlineStr">
         <is>
           <t>2026-05-18</t>
         </is>
       </c>
-      <c r="N25" s="12" t="inlineStr">
+      <c r="N25" t="inlineStr">
         <is>
           <t>CloseOut.NARR-PAUSE-1.2026-05-18.md</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="15" customHeight="1" s="13">
-      <c r="A26" s="12" t="n"/>
-      <c r="B26" s="12" t="inlineStr">
+    <row r="26" ht="15" customHeight="1" s="12">
+      <c r="B26" t="inlineStr">
         <is>
           <t>TTS-PARITY-1</t>
         </is>
       </c>
-      <c r="C26" s="12" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>Cache/Progress/Resume Parity Hardening</t>
         </is>
       </c>
-      <c r="D26" s="12" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>TTS Quality + Reading Exp v2</t>
         </is>
       </c>
-      <c r="E26" s="12" t="inlineStr">
+      <c r="E26" t="inlineStr">
         <is>
           <t>1a</t>
         </is>
       </c>
-      <c r="F26" s="12" t="inlineStr">
+      <c r="F26" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="G26" s="12" t="inlineStr">
+      <c r="G26" t="inlineStr">
         <is>
           <t>NARR-PAUSE-1</t>
         </is>
       </c>
-      <c r="H26" s="12" t="inlineStr">
+      <c r="H26" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="I26" s="12" t="inlineStr">
+      <c r="I26" t="inlineStr">
         <is>
           <t>Full Spec</t>
         </is>
       </c>
-      <c r="J26" s="12" t="inlineStr">
+      <c r="J26" t="inlineStr">
         <is>
           <t>Fix cache silence parity, trusted progress lag, resume backpressure</t>
         </is>
       </c>
-      <c r="K26" s="12" t="inlineStr">
+      <c r="K26" t="inlineStr">
         <is>
           <t>sprint/tts-parity-1</t>
         </is>
       </c>
-      <c r="M26" s="24" t="n">
+      <c r="M26" s="10" t="n">
         <v>46160</v>
       </c>
-      <c r="N26" s="12" t="inlineStr">
+      <c r="N26" t="inlineStr">
         <is>
           <t>CloseOut.TTS-PARITY-1.2026-05-18.md</t>
         </is>
       </c>
-      <c r="O26" s="12" t="inlineStr">
+      <c r="O26" t="inlineStr">
         <is>
           <t>OutsideAudit.9 hardening gate. Three defects, three tests.</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="15" customHeight="1" s="13">
-      <c r="A27" s="12" t="n">
+    <row r="27" ht="15" customHeight="1" s="12">
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>NARR-CURSOR-2</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Silence-Aware Cursor Hold</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>TTS Quality + Reading Exp v2</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>1a</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>NARR-PAUSE-1, TTS-PARITY-1, NARR-SPOKEN-1</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Full Spec</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Freeze cursor during inter-word silence using real endTime timestamps</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>sprint/narr-cursor-2-silence-hold</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>CloseOut.NARR-CURSOR-2.2026-05-18.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="15" customHeight="1" s="12">
+      <c r="A28" t="n">
         <v>1</v>
       </c>
-      <c r="B27" s="12" t="inlineStr">
-        <is>
-          <t>NARR-CURSOR-2</t>
-        </is>
-      </c>
-      <c r="C27" s="12" t="inlineStr">
-        <is>
-          <t>Silence-Aware Cursor Hold</t>
-        </is>
-      </c>
-      <c r="D27" s="12" t="inlineStr">
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>TTS-EVAL-3</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Quality Evaluation + CI Gate</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
         <is>
           <t>TTS Quality + Reading Exp v2</t>
         </is>
       </c>
-      <c r="E27" s="12" t="inlineStr">
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>1b</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Queued</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Full Spec</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Extend eval harness with quality scoring dimensions and CI gate config</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>sprint/tts-eval-3-quality-ci-gate</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="15" customHeight="1" s="12">
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>NARR-SPOKEN-1</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Spoken/Display Word Separation</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>TTS Quality + Reading Exp v2</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
         <is>
           <t>1a</t>
         </is>
       </c>
-      <c r="F27" s="12" t="inlineStr">
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>TTS-PARITY-1</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Full Spec</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Filter punctuation-only tokens from phoneme alignment input</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>sprint/narr-spoken-1</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>CloseOut.NARR-SPOKEN-1.2026-05-18.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="15" customHeight="1" s="12">
+      <c r="A30" t="n">
+        <v>2</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>UX-POLISH-1</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Library Cards + Command Palette + Space-Bar Mode</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>TTS Quality + Reading Exp v2</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Queued</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Stub</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Reading experience UX improvements batch</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="15" customHeight="1" s="12">
+      <c r="A31" t="n">
+        <v>3</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>TTS-QUAL-CI-1</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>CI Regression Gate Wiring</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>TTS Quality + Reading Exp v2</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="G27" s="12" t="inlineStr">
-        <is>
-          <t>NARR-PAUSE-1, TTS-PARITY-1, NARR-SPOKEN-1</t>
-        </is>
-      </c>
-      <c r="H27" s="12" t="inlineStr">
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>TTS-EVAL-3</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
         <is>
           <t>Queued</t>
         </is>
       </c>
-      <c r="I27" s="12" t="inlineStr">
-        <is>
-          <t>Full Spec</t>
-        </is>
-      </c>
-      <c r="J27" s="12" t="inlineStr">
-        <is>
-          <t>Freeze cursor during inter-word silence using real endTime timestamps</t>
-        </is>
-      </c>
-      <c r="K27" s="12" t="inlineStr">
-        <is>
-          <t>sprint/narr-cursor-2-silence-hold</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="15" customHeight="1" s="13">
-      <c r="A28" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="B28" s="12" t="inlineStr">
-        <is>
-          <t>TTS-EVAL-3</t>
-        </is>
-      </c>
-      <c r="C28" s="12" t="inlineStr">
-        <is>
-          <t>Quality Evaluation + CI Gate</t>
-        </is>
-      </c>
-      <c r="D28" s="12" t="inlineStr">
-        <is>
-          <t>TTS Quality + Reading Exp v2</t>
-        </is>
-      </c>
-      <c r="E28" s="12" t="inlineStr">
-        <is>
-          <t>1b</t>
-        </is>
-      </c>
-      <c r="F28" s="12" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="G28" s="12" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="H28" s="12" t="inlineStr">
-        <is>
-          <t>Queued</t>
-        </is>
-      </c>
-      <c r="I28" s="12" t="inlineStr">
-        <is>
-          <t>Full Spec</t>
-        </is>
-      </c>
-      <c r="J28" s="12" t="inlineStr">
-        <is>
-          <t>Extend eval harness with quality scoring dimensions and CI gate config</t>
-        </is>
-      </c>
-      <c r="K28" s="12" t="inlineStr">
-        <is>
-          <t>sprint/tts-eval-3-quality-ci-gate</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="15" customHeight="1" s="13">
-      <c r="A29" s="12" t="n"/>
-      <c r="B29" s="12" t="inlineStr">
-        <is>
-          <t>NARR-SPOKEN-1</t>
-        </is>
-      </c>
-      <c r="C29" s="12" t="inlineStr">
-        <is>
-          <t>Spoken/Display Word Separation</t>
-        </is>
-      </c>
-      <c r="D29" s="12" t="inlineStr">
-        <is>
-          <t>TTS Quality + Reading Exp v2</t>
-        </is>
-      </c>
-      <c r="E29" s="12" t="inlineStr">
-        <is>
-          <t>1a</t>
-        </is>
-      </c>
-      <c r="F29" s="12" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="G29" s="12" t="inlineStr">
-        <is>
-          <t>TTS-PARITY-1</t>
-        </is>
-      </c>
-      <c r="H29" s="12" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="I29" s="12" t="inlineStr">
-        <is>
-          <t>Full Spec</t>
-        </is>
-      </c>
-      <c r="J29" s="12" t="inlineStr">
-        <is>
-          <t>Filter punctuation-only tokens from phoneme alignment input</t>
-        </is>
-      </c>
-      <c r="K29" s="12" t="inlineStr">
-        <is>
-          <t>sprint/narr-spoken-1</t>
-        </is>
-      </c>
-      <c r="M29" t="inlineStr">
-        <is>
-          <t>2026-05-18</t>
-        </is>
-      </c>
-      <c r="N29" t="inlineStr">
-        <is>
-          <t>CloseOut.NARR-SPOKEN-1.2026-05-18.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="15" customHeight="1" s="13">
-      <c r="A30" s="12" t="n">
-        <v>3</v>
-      </c>
-      <c r="B30" s="12" t="inlineStr">
-        <is>
-          <t>UX-POLISH-1</t>
-        </is>
-      </c>
-      <c r="C30" s="12" t="inlineStr">
-        <is>
-          <t>Library Cards + Command Palette + Space-Bar Mode</t>
-        </is>
-      </c>
-      <c r="D30" s="12" t="inlineStr">
-        <is>
-          <t>TTS Quality + Reading Exp v2</t>
-        </is>
-      </c>
-      <c r="E30" s="12" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="F30" s="12" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="G30" s="12" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="H30" s="12" t="inlineStr">
-        <is>
-          <t>Queued</t>
-        </is>
-      </c>
-      <c r="I30" s="12" t="inlineStr">
+      <c r="I31" t="inlineStr">
         <is>
           <t>Stub</t>
         </is>
       </c>
-      <c r="J30" s="12" t="inlineStr">
-        <is>
-          <t>Reading experience UX improvements batch</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="15" customHeight="1" s="13">
-      <c r="A31" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="B31" s="12" t="inlineStr">
-        <is>
-          <t>TTS-QUAL-CI-1</t>
-        </is>
-      </c>
-      <c r="C31" s="12" t="inlineStr">
-        <is>
-          <t>CI Regression Gate Wiring</t>
-        </is>
-      </c>
-      <c r="D31" s="12" t="inlineStr">
-        <is>
-          <t>TTS Quality + Reading Exp v2</t>
-        </is>
-      </c>
-      <c r="E31" s="12" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="F31" s="12" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="G31" s="12" t="inlineStr">
-        <is>
-          <t>TTS-EVAL-3</t>
-        </is>
-      </c>
-      <c r="H31" s="12" t="inlineStr">
-        <is>
-          <t>Queued</t>
-        </is>
-      </c>
-      <c r="I31" s="12" t="inlineStr">
-        <is>
-          <t>Stub</t>
-        </is>
-      </c>
-      <c r="J31" s="12" t="inlineStr">
+      <c r="J31" t="inlineStr">
         <is>
           <t>Wire quality gates into GitHub Actions CI pipeline</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>

</xml_diff>

<commit_message>
docs(governance): TTS-EVAL-3 close-out + Vitest worktree isolation
- CloseOut report: all-pass, 12 findings, v2 baseline + soak run

- SRL-045: eval sprints well-bounded when harness pre-exists

- sprint-queue.xlsx: TTS-EVAL-3 completed, queue resequenced (depth 2)

- ROADMAP.md: CWS row added, spec archived, header RED depth 2

- CLAUDE.md: completion bullet + queue pointer updated

- Vitest excludes .worktrees/** so local sprint worktrees do not leak into root test runs
</commit_message>
<xml_diff>
--- a/docs/governance/sprint-queue.xlsx
+++ b/docs/governance/sprint-queue.xlsx
@@ -2171,9 +2171,6 @@
       </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="12">
-      <c r="A28" t="n">
-        <v>1</v>
-      </c>
       <c r="B28" t="inlineStr">
         <is>
           <t>TTS-EVAL-3</t>
@@ -2206,7 +2203,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Queued</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -2222,6 +2219,16 @@
       <c r="K28" t="inlineStr">
         <is>
           <t>sprint/tts-eval-3-quality-ci-gate</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>CloseOut.TTS-EVAL-3.2026-05-18.md</t>
         </is>
       </c>
     </row>
@@ -2289,7 +2296,7 @@
     </row>
     <row r="30" ht="15" customHeight="1" s="12">
       <c r="A30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2339,7 +2346,7 @@
     </row>
     <row r="31" ht="15" customHeight="1" s="12">
       <c r="A31" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs(roadmap): resequence reader runtime solidification queue
</commit_message>
<xml_diff>
--- a/docs/governance/sprint-queue.xlsx
+++ b/docs/governance/sprint-queue.xlsx
@@ -236,7 +236,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SprintCatalog" displayName="SprintCatalog" ref="A1:O23" headerRowCount="1" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SprintCatalog" displayName="SprintCatalog" ref="A1:O39" headerRowCount="1" totalsRowShown="0">
   <autoFilter ref="A1:O23"/>
   <tableColumns count="15">
     <tableColumn id="1" name="Seq"/>
@@ -452,7 +452,7 @@
     <row r="1" ht="17.25" customHeight="1" s="12">
       <c r="B1" s="11" t="inlineStr">
         <is>
-          <t>TTS Architecture Completion — Sprint Dashboard</t>
+          <t>Reader Runtime Solidification — Sprint Dashboard</t>
         </is>
       </c>
     </row>
@@ -495,25 +495,25 @@
     </row>
     <row r="3" ht="15" customHeight="1" s="12">
       <c r="B3" s="2" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>0.7272727273</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>60</v>
+        <v>97</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>17</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="12">
@@ -529,34 +529,62 @@
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="12">
-      <c r="B6" s="1" t="n">
-        <v>8</v>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>Queue Depth</t>
+        </is>
       </c>
       <c r="C6" t="n">
-        <v>3</v>
+        <v>10</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Full Specs</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>5</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Stubs</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="12">
       <c r="B7" s="1" t="inlineStr">
         <is>
-          <t>NARR-MEDIA-1</t>
+          <t>Next Dispatch</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>KOKORO-EXPORT-1</t>
+          <t>BASELINE-SYNC-1</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Next Phase</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Reader Runtime Solidification</t>
         </is>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="12">
       <c r="B8" s="1" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>Dashboard Updated</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-22</t>
         </is>
       </c>
     </row>
@@ -575,7 +603,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O31"/>
+  <dimension ref="A1:O39"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="5" customWidth="1" style="12" min="1" max="1"/>
@@ -2300,32 +2328,32 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>UX-POLISH-1</t>
+          <t>BASELINE-SYNC-1</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Library Cards + Command Palette + Space-Bar Mode</t>
+          <t>Commit Phase 0 + Governance Sweep Baseline</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>TTS Quality + Reading Exp v2</t>
+          <t>Reader Runtime Solidification</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>READER-MODE-ISOLATION-1 Phase 0; GOVERNANCE-SWEEP</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -2335,12 +2363,22 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Stub</t>
+          <t>Full Spec</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Reading experience UX improvements batch</t>
+          <t>Review, stage, verify, and commit Phase 0 plus governance sweep baseline</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>main/current dirty baseline sync</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>Split commits preferred; exclude local-only artifacts.</t>
         </is>
       </c>
     </row>
@@ -2350,47 +2388,512 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
+          <t>TEST-GREEN-1</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Broad Suite Failure Triage</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Reader Runtime Solidification</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>BASELINE-SYNC-1</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Queued</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Full Spec</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Reproduce and classify broad-suite failures before CI gating</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>sprint/test-green-1-broad-suite-triage</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>Establish default-suite green/classified path.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>3</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>READER-ISO-1A</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Adapter Contracts + Current Word Anchor Service</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Reader Runtime Solidification</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>TEST-GREEN-1</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Queued</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Full Spec</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Add adapter contracts and tested shared current-word anchor service</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>sprint/reader-iso-1a-adapter-anchor-contracts</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>Behavior-preserving contract and anchor sprint.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>4</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>READER-ISO-1B</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Orchestrator Shell + Mode Selection Semantics</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Reader Runtime Solidification</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>READER-ISO-1A</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Queued</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Full Spec</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Extract mode orchestrator shell while preserving exact-start and no-auto-start semantics</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>sprint/reader-iso-1b-orchestrator-shell</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>Preserve C navigation and delayed readiness intent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>5</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>READER-ISO-1C</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Focus Adapter + Passive Surface Contract Start</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Reader Runtime Solidification</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>READER-ISO-1B</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Queued</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Full Spec</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Move Focus behind adapter and begin passive surface command typing</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>sprint/reader-iso-1c-focus-adapter</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>Lowest-risk adapter migration before Flow/Narrate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>6</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>READER-ISO-1D</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Flow Adapter + Section Handoff Restart Ownership</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Reader Runtime Solidification</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>READER-ISO-1C</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Queued</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Stub</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Move Flow lifecycle and FlowScrollEngine ownership behind Flow adapter</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>Flow owns section-handoff restart; no Narrate truth-sync changes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>7</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>READER-ISO-1E</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Narrate Adapter + Audio Truth-Sync Ownership</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Reader Runtime Solidification</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>READER-ISO-1D</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Queued</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Stub</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Move Narrate lifecycle behind audio truth-sync owned adapter</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>Narrate starts at exact selected/current word and never follows Flow engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>8</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>GOV-HUMAN-REVIEW-1</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Deferred Governance Review Items</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Reader Runtime Solidification</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>BASELINE-SYNC-1</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Queued</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Stub</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Resolve deferred governance-sweep human-review items</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>MarcusAurelius stub, ROADMAP_SPECS refs, close-out volume, naming outliers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>9</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
           <t>TTS-QUAL-CI-1</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>CI Regression Gate Wiring</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>TTS Quality + Reading Exp v2</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Quality Gate Activation</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>TTS-EVAL-3</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>TEST-GREEN-1; TTS-EVAL-3</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
         <is>
           <t>Queued</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr">
+      <c r="I38" t="inlineStr">
         <is>
           <t>Stub</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>Wire quality gates into GitHub Actions CI pipeline</t>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Wire TTS quality gates into CI after suite health is restored</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>Deferred until broad-suite health is clean or formally classified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>10</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>UX-POLISH-1</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Library Cards + Command Palette + Space-Bar Mode</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Reading Experience UX Polish</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>UX</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Reader runtime stable</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Queued</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Stub</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Library cards, command palette, and Space-bar polish after runtime controls stabilize</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>Deferred until reader-mode runtime controls stop churning.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(governance): close baseline and test-green queue updates
</commit_message>
<xml_diff>
--- a/docs/governance/sprint-queue.xlsx
+++ b/docs/governance/sprint-queue.xlsx
@@ -452,7 +452,7 @@
     <row r="1" ht="17.25" customHeight="1" s="12">
       <c r="B1" s="11" t="inlineStr">
         <is>
-          <t>Reader Runtime Solidification — Sprint Dashboard</t>
+          <t>Reader Runtime Solidification - Sprint Dashboard</t>
         </is>
       </c>
     </row>
@@ -498,22 +498,22 @@
         <v>33</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.7272727272727273</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>97</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>42</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="12">
@@ -535,7 +535,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -543,7 +543,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -562,7 +562,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>BASELINE-SYNC-1</t>
+          <t>READER-ISO-1A</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -2323,9 +2323,6 @@
       </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="12">
-      <c r="A30" t="n">
-        <v>1</v>
-      </c>
       <c r="B30" t="inlineStr">
         <is>
           <t>BASELINE-SYNC-1</t>
@@ -2358,7 +2355,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Queued</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -2376,16 +2373,23 @@
           <t>main/current dirty baseline sync</t>
         </is>
       </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>CloseOut.BASELINE-SYNC-1.2026-05-22.md</t>
+        </is>
+      </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>Split commits preferred; exclude local-only artifacts.</t>
+          <t>Completed in three pushed commits: reader anchors, governance sweep, roadmap queue resequence.</t>
         </is>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="12">
-      <c r="A31" t="n">
-        <v>2</v>
-      </c>
       <c r="B31" t="inlineStr">
         <is>
           <t>TEST-GREEN-1</t>
@@ -2418,7 +2422,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Queued</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -2436,15 +2440,25 @@
           <t>sprint/test-green-1-broad-suite-triage</t>
         </is>
       </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>CloseOut.TEST-GREEN-1.2026-05-22.md</t>
+        </is>
+      </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>Establish default-suite green/classified path.</t>
+          <t>Completed at 172cffb; 12 failures classified/resolved, 3 environmental flakes documented.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2504,7 +2518,7 @@
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2564,7 +2578,7 @@
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2624,7 +2638,7 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2679,7 +2693,7 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -2734,7 +2748,7 @@
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -2789,7 +2803,7 @@
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -2844,7 +2858,7 @@
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs(roadmap): route reader anchor repair before isolation
</commit_message>
<xml_diff>
--- a/docs/governance/sprint-queue.xlsx
+++ b/docs/governance/sprint-queue.xlsx
@@ -495,25 +495,25 @@
     </row>
     <row r="3" ht="15" customHeight="1" s="12">
       <c r="B3" s="2" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C3" s="2" t="n">
         <v>24</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>0.7272727272727273</v>
+        <v>0.7058823529411765</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>61</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>36</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="12">
@@ -535,7 +535,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -543,7 +543,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -551,7 +551,7 @@
         </is>
       </c>
       <c r="G6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="12">
@@ -562,7 +562,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>READER-ISO-1A</t>
+          <t>READER-PERSISTENT-ANCHOR-STEP3-REPAIR</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -603,7 +603,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O39"/>
+  <dimension ref="A1:O40"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="5" customWidth="1" style="12" min="1" max="1"/>
@@ -2462,12 +2462,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>READER-ISO-1A</t>
+          <t>READER-PERSISTENT-ANCHOR-STEP3-REPAIR</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Adapter Contracts + Current Word Anchor Service</t>
+          <t>Persistent Anchor Manual QA Repair</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2477,17 +2477,17 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>L</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>TEST-GREEN-1</t>
+          <t>READER-PERSISTENT-ANCHOR Step 2 manual QA report</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -2502,17 +2502,12 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Add adapter contracts and tested shared current-word anchor service</t>
+          <t>Repair Page/Focus/Flow/Narrate persistent-anchor manual-QA failures before adapter isolation</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>sprint/reader-iso-1a-adapter-anchor-contracts</t>
-        </is>
-      </c>
-      <c r="O32" t="inlineStr">
-        <is>
-          <t>Behavior-preserving contract and anchor sprint.</t>
+          <t>hotfix/reader-persistent-anchor-step3-repair</t>
         </is>
       </c>
     </row>
@@ -2522,12 +2517,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>READER-ISO-1B</t>
+          <t>READER-ISO-1A</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Orchestrator Shell + Mode Selection Semantics</t>
+          <t>Adapter Contracts + Current Word Anchor Service</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -2542,12 +2537,12 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>READER-ISO-1A</t>
+          <t>READER-PERSISTENT-ANCHOR-STEP3-REPAIR; TEST-GREEN-1</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -2562,17 +2557,17 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Extract mode orchestrator shell while preserving exact-start and no-auto-start semantics</t>
+          <t>Add adapter contracts and tested shared current-word anchor service</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>sprint/reader-iso-1b-orchestrator-shell</t>
+          <t>sprint/reader-iso-1a-adapter-anchor-contracts</t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>Preserve C navigation and delayed readiness intent.</t>
+          <t>Behavior-preserving contract and anchor sprint.</t>
         </is>
       </c>
     </row>
@@ -2582,12 +2577,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>READER-ISO-1C</t>
+          <t>READER-ISO-1B</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Focus Adapter + Passive Surface Contract Start</t>
+          <t>Orchestrator Shell + Mode Selection Semantics</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2602,12 +2597,12 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>L</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>READER-ISO-1B</t>
+          <t>READER-ISO-1A</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -2622,17 +2617,17 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Move Focus behind adapter and begin passive surface command typing</t>
+          <t>Extract mode orchestrator shell while preserving exact-start and no-auto-start semantics</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>sprint/reader-iso-1c-focus-adapter</t>
+          <t>sprint/reader-iso-1b-orchestrator-shell</t>
         </is>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>Lowest-risk adapter migration before Flow/Narrate.</t>
+          <t>Preserve C navigation and delayed readiness intent.</t>
         </is>
       </c>
     </row>
@@ -2642,12 +2637,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>READER-ISO-1D</t>
+          <t>READER-ISO-1C</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Flow Adapter + Section Handoff Restart Ownership</t>
+          <t>Focus Adapter + Passive Surface Contract Start</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -2662,12 +2657,12 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>READER-ISO-1C</t>
+          <t>READER-ISO-1B</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -2677,17 +2672,22 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Stub</t>
+          <t>Full Spec</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Move Flow lifecycle and FlowScrollEngine ownership behind Flow adapter</t>
+          <t>Move Focus behind adapter and begin passive surface command typing</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>sprint/reader-iso-1c-focus-adapter</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>Flow owns section-handoff restart; no Narrate truth-sync changes.</t>
+          <t>Lowest-risk adapter migration before Flow/Narrate.</t>
         </is>
       </c>
     </row>
@@ -2697,12 +2697,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>READER-ISO-1E</t>
+          <t>READER-ISO-1D</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Narrate Adapter + Audio Truth-Sync Ownership</t>
+          <t>Flow Adapter + Section Handoff Restart Ownership</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -2722,7 +2722,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>READER-ISO-1D</t>
+          <t>READER-ISO-1C</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -2732,17 +2732,22 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Stub</t>
+          <t>Full Spec</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Move Narrate lifecycle behind audio truth-sync owned adapter</t>
+          <t>Move Flow lifecycle and FlowScrollEngine ownership behind Flow adapter</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>sprint/reader-iso-1d-flow-adapter</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>Narrate starts at exact selected/current word and never follows Flow engine.</t>
+          <t>Flow owns section-handoff restart; no Narrate truth-sync changes.</t>
         </is>
       </c>
     </row>
@@ -2752,12 +2757,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>GOV-HUMAN-REVIEW-1</t>
+          <t>READER-ISO-1E</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Deferred Governance Review Items</t>
+          <t>Narrate Adapter + Audio Truth-Sync Ownership</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2767,17 +2772,17 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Governance</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>L</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>BASELINE-SYNC-1</t>
+          <t>READER-ISO-1D</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -2792,12 +2797,12 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Resolve deferred governance-sweep human-review items</t>
+          <t>Move Narrate lifecycle behind audio truth-sync owned adapter</t>
         </is>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>MarcusAurelius stub, ROADMAP_SPECS refs, close-out volume, naming outliers.</t>
+          <t>Narrate starts at exact selected/current word and never follows Flow engine.</t>
         </is>
       </c>
     </row>
@@ -2807,22 +2812,22 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>TTS-QUAL-CI-1</t>
+          <t>GOV-HUMAN-REVIEW-1</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>CI Regression Gate Wiring</t>
+          <t>Deferred Governance Review Items</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Quality Gate Activation</t>
+          <t>Reader Runtime Solidification</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>CI</t>
+          <t>Governance</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2832,7 +2837,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>TEST-GREEN-1; TTS-EVAL-3</t>
+          <t>BASELINE-SYNC-1</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -2847,12 +2852,12 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Wire TTS quality gates into CI after suite health is restored</t>
+          <t>Resolve deferred governance-sweep human-review items</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>Deferred until broad-suite health is clean or formally classified.</t>
+          <t>MarcusAurelius stub, ROADMAP_SPECS refs, close-out volume, naming outliers.</t>
         </is>
       </c>
     </row>
@@ -2862,50 +2867,105 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
+          <t>TTS-QUAL-CI-1</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>CI Regression Gate Wiring</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Quality Gate Activation</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>TEST-GREEN-1; TTS-EVAL-3</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Queued</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Stub</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Wire TTS quality gates into CI after suite health and reader runtime are stable</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>Deferred until broad-suite health is clean or formally classified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>9</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
           <t>UX-POLISH-1</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C40" t="inlineStr">
         <is>
           <t>Library Cards + Command Palette + Space-Bar Mode</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D40" t="inlineStr">
         <is>
           <t>Reading Experience UX Polish</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="E40" t="inlineStr">
         <is>
           <t>UX</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="F40" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr">
+      <c r="G40" t="inlineStr">
         <is>
           <t>Reader runtime stable</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr">
+      <c r="H40" t="inlineStr">
         <is>
           <t>Queued</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr">
+      <c r="I40" t="inlineStr">
         <is>
           <t>Stub</t>
         </is>
       </c>
-      <c r="J39" t="inlineStr">
+      <c r="J40" t="inlineStr">
         <is>
           <t>Library cards, command palette, and Space-bar polish after runtime controls stabilize</t>
         </is>
       </c>
-      <c r="O39" t="inlineStr">
+      <c r="O40" t="inlineStr">
         <is>
           <t>Deferred until reader-mode runtime controls stop churning.</t>
         </is>

</xml_diff>

<commit_message>
docs(governance): capture reader anchor step3.2 and step3.3 gates
</commit_message>
<xml_diff>
--- a/docs/governance/sprint-queue.xlsx
+++ b/docs/governance/sprint-queue.xlsx
@@ -572,7 +572,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Reader Runtime Solidification</t>
+          <t>Reader Runtime Solidification - Step 3.3 Manual QA With Sentence-Boundary Diagnostics</t>
         </is>
       </c>
     </row>
@@ -2467,7 +2467,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Persistent Anchor Manual QA Repair</t>
+          <t>Persistent Anchor Step 3.3 Manual QA With Sentence-Boundary Diagnostics</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2487,7 +2487,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>READER-PERSISTENT-ANCHOR Step 2 manual QA report</t>
+          <t>Step 3.3 code commits 881b01d/48c23ac; manual QA pending</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -2502,12 +2502,12 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Repair Page/Focus/Flow/Narrate persistent-anchor manual-QA failures before adapter isolation</t>
+          <t>Rerun S12/S13 with DevTools diagnostics after double-resync and cold-start sentence-boundary fixes; spot-check S8/S1/S4/S18</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>hotfix/reader-persistent-anchor-step3-repair</t>
+          <t>hotfix/reader-persistent-anchor</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(governance): capture reader anchor step3.4 gate and step3.5 queue
</commit_message>
<xml_diff>
--- a/docs/governance/sprint-queue.xlsx
+++ b/docs/governance/sprint-queue.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:H8"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="3" customWidth="1" style="12" min="1" max="1"/>
@@ -516,6 +516,7 @@
         <v>44</v>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="15" customHeight="1" s="12">
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -572,7 +573,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Reader Runtime Solidification - Step 3.3 Manual QA With Sentence-Boundary Diagnostics</t>
+          <t>Reader Runtime Solidification - Step 3.5 Cursor/Audio Sync</t>
         </is>
       </c>
     </row>
@@ -584,7 +585,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
     </row>
@@ -2467,7 +2468,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Persistent Anchor Step 3.3 Manual QA With Sentence-Boundary Diagnostics</t>
+          <t>Persistent Anchor Step 3.5 Cursor/Audio Sync Repair (NARRATE-CURSOR-SYNC-4)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2487,7 +2488,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Step 3.3 code commits 881b01d/48c23ac; manual QA pending</t>
+          <t>Step 3.4 manual QA: S12 start-word FIXED; S13 cursor/audio sync still fails</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -2502,7 +2503,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Rerun S12/S13 with DevTools diagnostics after double-resync and cold-start sentence-boundary fixes; spot-check S8/S1/S4/S18</t>
+          <t>Clamp Narrate cursor to the currently-playing source so it cannot lead audio; eliminate chunk-load skip-ahead. Rerun S13; spot-check S12/S8/S1/S4/S18. See ROADMAP Step 3.5 repair gate.</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">

</xml_diff>

<commit_message>
docs(governance): close reader anchor repair lane
</commit_message>
<xml_diff>
--- a/docs/governance/sprint-queue.xlsx
+++ b/docs/governance/sprint-queue.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="B1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="3" customWidth="1" style="12" min="1" max="1"/>
@@ -516,7 +516,6 @@
         <v>44</v>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="15" customHeight="1" s="12">
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -563,7 +562,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>READER-PERSISTENT-ANCHOR-STEP3-REPAIR</t>
+          <t>READER-ISO-1A</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -573,7 +572,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Reader Runtime Solidification - Step 3.5 Cursor/Audio Sync</t>
+          <t>Reader Runtime Solidification - Stage 2 Adapter Isolation</t>
         </is>
       </c>
     </row>
@@ -585,7 +584,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>
@@ -604,7 +603,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O40"/>
+  <dimension ref="A1:O41"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="5" customWidth="1" style="12" min="1" max="1"/>
@@ -2458,9 +2457,6 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="n">
-        <v>1</v>
-      </c>
       <c r="B32" t="inlineStr">
         <is>
           <t>READER-PERSISTENT-ANCHOR-STEP3-REPAIR</t>
@@ -2468,7 +2464,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Persistent Anchor Step 3.5 Cursor/Audio Sync Repair (NARRATE-CURSOR-SYNC-4)</t>
+          <t>Persistent Anchor Step 3.6 Content-Contiguous Synthesis (NARRATE-CURSOR-SYNC-5, Bug 2)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2488,12 +2484,12 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Step 3.4 manual QA: S12 start-word FIXED; S13 cursor/audio sync still fails</t>
+          <t>Step 3.5 manual QA: S13 split -&gt; Bug2 content omission (this); Bug1 visual lead deferred post-ISO</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Queued</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -2503,18 +2499,38 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Clamp Narrate cursor to the currently-playing source so it cannot lead audio; eliminate chunk-load skip-ahead. Rerun S13; spot-check S12/S8/S1/S4/S18. See ROADMAP Step 3.5 repair gate.</t>
+          <t>Fix content omission: seed automatic chunk continuation from produced-end (nextGenWordIndexRef), not lastConfirmedAudioWordRef (cursor twin); hard-click still re-anchors. Add schedule-vs-wallclock log. Gate: no words omitted by ear in The Raven. See ROADMAP Step 3.6.</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
           <t>hotfix/reader-persistent-anchor</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>docs/governance/close-outs/CloseOut.READER-PERSISTENT-ANCHOR-STEP3.6.2026-05-24.md</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>Repair lane closed by explicit disposition; S1/S4/S8/S12/S18 fixed, S5 accepted partial, S9 deferred, S13 moved to post-isolation NARRATE-CLOSED-LOOP-CURSOR.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2574,7 +2590,7 @@
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2634,7 +2650,7 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2694,7 +2710,7 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -2754,7 +2770,7 @@
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -2969,6 +2985,61 @@
       <c r="O40" t="inlineStr">
         <is>
           <t>Deferred until reader-mode runtime controls stop churning.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>6</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>NARRATE-CLOSED-LOOP-CURSOR</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Narrate Closed-Loop Cursor + Content Continuity (real audio position as single truth)</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Reader Runtime Solidification</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Stage 2 (post-isolation)</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>READER-ISO-1E (Narrate adapter) complete</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Queued (post-isolation)</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Stub</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Unifies Bug1 (cursor lead) + Bug2 (content omission) from Steps 3.5/3.6. Make the currently-playing source heard position the SINGLE source of truth for the visual cursor AND re-entry/continuation seeding; retire ahead-of-heard refs + lag/clamp compensations; bound prefetch. See ROADMAP NARRATE-CLOSED-LOOP-CURSOR.</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>Deferred post-isolation per Evan 2026-05-24 after 6 pre-isolation rounds. Does NOT block READER-ISO-1A.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(governance): close reader iso 1a
</commit_message>
<xml_diff>
--- a/docs/governance/sprint-queue.xlsx
+++ b/docs/governance/sprint-queue.xlsx
@@ -557,7 +557,7 @@
     <row r="7" ht="15" customHeight="1" s="12">
       <c r="B7" s="1" t="inlineStr">
         <is>
-          <t>Next Dispatch</t>
+          <t>READER-ISO-1B</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -2529,9 +2529,6 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="n">
-        <v>1</v>
-      </c>
       <c r="B33" t="inlineStr">
         <is>
           <t>READER-ISO-1A</t>
@@ -2564,7 +2561,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Queued</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2582,15 +2579,30 @@
           <t>sprint/reader-iso-1a-adapter-anchor-contracts</t>
         </is>
       </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>docs/governance/close-outs/CloseOut.READER-ISO-1A.2026-05-24.md</t>
+        </is>
+      </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>Behavior-preserving contract and anchor sprint.</t>
+          <t>Completed and merged to main at 32f4543; behavior-preserving adapter contract and anchor service sprint.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2650,7 +2662,7 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2710,7 +2722,7 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -2770,7 +2782,7 @@
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -2825,7 +2837,7 @@
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -2880,7 +2892,7 @@
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -2935,7 +2947,7 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -2990,7 +3002,7 @@
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3024,7 +3036,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Queued (post-isolation)</t>
+          <t>Queued</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -3039,7 +3051,7 @@
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>Deferred post-isolation per Evan 2026-05-24 after 6 pre-isolation rounds. Does NOT block READER-ISO-1A.</t>
+          <t>Deferred post-isolation per Evan 2026-05-24 after 6 pre-isolation rounds. Blocked by READER-ISO-1E; does NOT block READER-ISO-1B.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(governance): roadmap review 2026-05-25 — archive REPAIR/1A/1B, replenish buffer to 5 full specs
Archive-forward migration: REPAIR (Steps 3.1-3.6) + READER-ISO-1A + READER-ISO-1B full specs moved to docs/planning/.Archive/ROADMAP_2026-05-25.md.

Completed Work Summary: REPAIR one-line entry added.

Eager-spec buffer replenished 2 -> 5 full specs (1C, 1D, 1E, GOV-HUMAN-REVIEW-1, TTS-QUAL-CI-1); NARRATE-CLOSED-LOOP-CURSOR held as flagged buffer gap, specced at READER-ISO-1E close-out per SRL-072.

Standing Rules: SRL-070 (audio-independent sync ground truth), SRL-073 (adapter cleanup transition tests), SRL-074 (orchestrators consume building blocks) promoted.

sprint-queue.xlsx: Catalog Written Status updated; Dashboard KPIs recomputed (Total 35 / Completed 27 / Remaining 8 / 77.1%; Queue Depth 7; 5 full + 2 stubs).

5 review artifacts in docs/planning/roadmap-reviews/2026-05-25-*

Net ROADMAP.md: 415 -> 342 lines. Next dispatch: READER-ISO-1C.
</commit_message>
<xml_diff>
--- a/docs/governance/sprint-queue.xlsx
+++ b/docs/governance/sprint-queue.xlsx
@@ -495,25 +495,25 @@
     </row>
     <row r="3" ht="15" customHeight="1" s="12">
       <c r="B3" s="2" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>0.7058823529411765</v>
+        <v>0.7714285714</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>105</v>
+        <v>125</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>61</v>
+        <v>80</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="12">
@@ -535,7 +535,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -551,18 +551,18 @@
         </is>
       </c>
       <c r="G6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="12">
       <c r="B7" s="1" t="inlineStr">
         <is>
+          <t>READER-ISO-1C</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
           <t>READER-ISO-1B</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>READER-ISO-1A</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -584,7 +584,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
     </row>
@@ -2601,9 +2601,6 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="n">
-        <v>1</v>
-      </c>
       <c r="B34" t="inlineStr">
         <is>
           <t>READER-ISO-1B</t>
@@ -2636,7 +2633,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Queued</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2654,15 +2651,30 @@
           <t>sprint/reader-iso-1b-orchestrator-shell</t>
         </is>
       </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>docs/governance/close-outs/CloseOut.READER-ISO-1B.2026-05-25.md</t>
+        </is>
+      </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>Preserve C navigation and delayed readiness intent.</t>
+          <t>Completed and merged to main at 1f4a75a; behavior-preserving orchestrator shell extraction.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2722,7 +2734,7 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -2751,7 +2763,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>READER-ISO-1C</t>
+          <t>READER-ISO-1C; persistent-anchor repair lane closed by explicit disposition; Flow S9 lazy-follow deferred</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -2782,7 +2794,7 @@
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -2821,7 +2833,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Stub</t>
+          <t>Full Spec</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -2837,7 +2849,7 @@
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -2876,7 +2888,7 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>Stub</t>
+          <t>Full Spec</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
@@ -2892,7 +2904,7 @@
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -2931,7 +2943,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Stub</t>
+          <t>Full Spec</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -2947,7 +2959,7 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3002,7 +3014,7 @@
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs(governance): close reader iso 1c
</commit_message>
<xml_diff>
--- a/docs/governance/sprint-queue.xlsx
+++ b/docs/governance/sprint-queue.xlsx
@@ -557,7 +557,7 @@
     <row r="7" ht="15" customHeight="1" s="12">
       <c r="B7" s="1" t="inlineStr">
         <is>
-          <t>READER-ISO-1C</t>
+          <t>READER-ISO-1D</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -2673,9 +2673,6 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="n">
-        <v>1</v>
-      </c>
       <c r="B35" t="inlineStr">
         <is>
           <t>READER-ISO-1C</t>
@@ -2708,7 +2705,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Queued</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2726,15 +2723,30 @@
           <t>sprint/reader-iso-1c-focus-adapter</t>
         </is>
       </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>docs/governance/close-outs/CloseOut.READER-ISO-1C.2026-05-26.md</t>
+        </is>
+      </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>Lowest-risk adapter migration before Flow/Narrate.</t>
+          <t>Completed and merged to main at 634bac2; first concrete Focus adapter plus passive SurfaceCommand types.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -2794,7 +2806,7 @@
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -2849,7 +2861,7 @@
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -2904,7 +2916,7 @@
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -2959,7 +2971,7 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3014,7 +3026,7 @@
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs(governance): /roadmap-review 2026-05-28 — buffer replenished to 5 full specs
BUG_REPORT: BUG-181 RESOLVED after v1.75.1 rebuild verified Meditations renders; BUG-182 (Settings theme propagation + Vite circular chunk) and BUG-183 (Chrome extension auth handshake timeout) filed.

ROADMAP: Stage 2 renamed Active Conveyor Belt; 3 new full specs (EXT-PAIR-1, THEME-SYNC-1, NARRATE-CLOSED-LOOP-CURSOR promoted from stub after READER-ISO-1E); SINGLE-INSTANCE-LOCK-1 added (F1); TTS-QUAL-CI-1 amended to absorb scripts/recalc.py + LOE-XS dropdown extension; SRL-079 added (Standing Rule #35: source-fix verification needs rebuild gate).

CLAUDE.md: queue state line updated to depth 6 (5 full specs + 1 stub); open-bugs line lists BUG-154/182/183.

sprint-queue.xlsx: Catalog mirrored to ROADMAP — Seq reordered, 3 rows inserted, Phase/Stage drift fixed across the conveyor.
</commit_message>
<xml_diff>
--- a/docs/governance/sprint-queue.xlsx
+++ b/docs/governance/sprint-queue.xlsx
@@ -603,7 +603,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O41"/>
+  <dimension ref="A1:O44"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="5" customWidth="1" style="12" min="1" max="1"/>
@@ -2937,7 +2937,7 @@
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -2951,12 +2951,12 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Quality Gate Activation</t>
+          <t>Reader Runtime Solidification</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>CI</t>
+          <t>Active Conveyor Belt</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2982,6 +2982,11 @@
       <c r="J39" t="inlineStr">
         <is>
           <t>Wire TTS quality gates into CI after suite health and reader runtime are stable</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>sprint/tts-qual-ci-1</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
@@ -2992,7 +2997,7 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3006,12 +3011,12 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Reading Experience UX Polish</t>
+          <t>Reader Runtime Solidification</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>UX</t>
+          <t>Active Conveyor Belt</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -3047,7 +3052,7 @@
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3066,7 +3071,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Stage 2 (post-isolation)</t>
+          <t>Active Conveyor Belt</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -3086,17 +3091,187 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>Stub</t>
+          <t>Full Spec</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>Unifies Bug1 (cursor lead) + Bug2 (content omission) from Steps 3.5/3.6. Make the currently-playing source heard position the SINGLE source of truth for the visual cursor AND re-entry/continuation seeding; retire ahead-of-heard refs + lag/clamp compensations; bound prefetch. See ROADMAP NARRATE-CLOSED-LOOP-CURSOR.</t>
+          <t>Make currently-playing audio source's real word position the SINGLE source of truth for cursor + re-entry seeding; retire ahead-of-heard refs; bound prefetch window.</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>sprint/narrate-closed-loop-cursor</t>
         </is>
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>Deferred post-isolation per Evan 2026-05-24 after 6 pre-isolation rounds. Blocked by READER-ISO-1E; does NOT block READER-ISO-1B.</t>
+          <t>Promoted from stub 2026-05-28 after READER-ISO-1E shipped. Shared-core sprint — runs alone (touches useNarration.ts + audioScheduler.ts).</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>2</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>EXT-PAIR-1</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Chrome Extension Pairing Auth Timeout Repair</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Reader Runtime Solidification</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Active Conveyor Belt</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Queued</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Full Spec</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Split WS_AUTH_TIMEOUT_MS into a generous pairing window (5 min) for first-time human pair and the existing tight 5s window for stored-token re-auth. Closes BUG-183.</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>sprint/ext-pair-1</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>Hotfix for BUG-183 (filed 2026-05-28). Aristotle-gated. Parallel-safe with TTS-QUAL-CI-1 + SINGLE-INSTANCE-LOCK-1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>3</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>SINGLE-INSTANCE-LOCK-1</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Electron Main-Process Single-Instance Gate</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Reader Runtime Solidification</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Active Conveyor Belt</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Queued</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Full Spec</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Add app.requestSingleInstanceLock() + second-instance handler to focus existing window instead of spawning duplicate BrowserWindow. ~5 LOC. Closes F1 from discovery sweep.</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>sprint/single-instance-lock-1</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>XS effort. Parallel-safe with everything in buffer (Lane D, main-process only).</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>4</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>THEME-SYNC-1</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Settings Theme Propagation + Vite Circular Chunk Repair</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Reader Runtime Solidification</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Active Conveyor Belt</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Queued</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Full Spec</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Resolve settings↔tts circular chunk warning and audit theme-context subscription across Settings sub-pages. Closes BUG-182.</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>sprint/theme-sync-1</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>Hotfix for BUG-182 (filed 2026-05-28). Aristotle-gated. Parallel-safe with EXT-PAIR-1.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(governance): add recalc.py + extend LOE dropdown with XS (TTS-QUAL-CI-1)
Add scripts/recalc.py (~37 LOC, Python + openpyxl) to refresh xlsx formula
caches after programmatic edits. Extend Catalog LOE data-validation dropdown
to include XS (0.5 pts). Update SINGLE-INSTANCE-LOCK-1 LOE from S to XS.
Mark TTS-QUAL-CI-1 completed in Catalog, update Dashboard KPIs.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/governance/sprint-queue.xlsx
+++ b/docs/governance/sprint-queue.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalog" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1" iterateDelta="0.0001"/>
+  <calcPr calcId="0" calcMode="auto" fullCalcOnLoad="1" iterateDelta="0.0001"/>
 </workbook>
 </file>
 
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:H8"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="3" customWidth="1" style="12" min="1" max="1"/>
@@ -498,13 +498,13 @@
         <v>35</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>0.8571428571428571</v>
+        <v>0.8857142857142857</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>125</v>
@@ -516,6 +516,7 @@
         <v>35</v>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="15" customHeight="1" s="12">
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -535,34 +536,34 @@
         </is>
       </c>
       <c r="C6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Full Specs</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
         <v>4</v>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Full Specs</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>2</v>
-      </c>
       <c r="F6" t="inlineStr">
         <is>
           <t>Stubs</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="12">
       <c r="B7" s="1" t="inlineStr">
         <is>
-          <t>GOV-HUMAN-REVIEW-1</t>
+          <t>EXT-PAIR-1</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>NARRATE-CLOSED-LOOP-CURSOR</t>
+          <t>SINGLE-INSTANCE-LOCK-1</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -584,7 +585,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
@@ -2936,9 +2937,6 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="n">
-        <v>1</v>
-      </c>
       <c r="B39" t="inlineStr">
         <is>
           <t>TTS-QUAL-CI-1</t>
@@ -2971,7 +2969,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Queued</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -2987,6 +2985,21 @@
       <c r="K39" t="inlineStr">
         <is>
           <t>sprint/tts-qual-ci-1</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>CloseOut.TTS-QUAL-CI-1.2026-05-28.md</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
@@ -2997,7 +3010,7 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3052,7 +3065,7 @@
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3112,7 +3125,7 @@
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3136,7 +3149,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>XS</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -3167,7 +3180,7 @@
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3222,7 +3235,7 @@
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs(governance): reconcile TTS quality gate closeout queue
</commit_message>
<xml_diff>
--- a/docs/governance/sprint-queue.xlsx
+++ b/docs/governance/sprint-queue.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="B1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="3" customWidth="1" style="12" min="1" max="1"/>
@@ -516,7 +516,6 @@
         <v>35</v>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="15" customHeight="1" s="12">
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -604,7 +603,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O44"/>
+  <dimension ref="A1:O45"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="5" customWidth="1" style="12" min="1" max="1"/>
@@ -3204,7 +3203,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>XS</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -3285,6 +3284,56 @@
       <c r="O44" t="inlineStr">
         <is>
           <t>Hotfix for BUG-182 (filed 2026-05-28). Aristotle-gated. Parallel-safe with EXT-PAIR-1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>6</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>HYG-XLSX-DASHBOARD-RESTORE</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Restore sprint-queue.xlsx Dashboard formulas + openpyxl quarantine</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Reader Runtime Solidification</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Active Conveyor Belt</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>XS</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Queued</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Stub</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Rebuild Dashboard formulas in Excel; extend scripts/recalc.py with Dashboard-tab guardrail; document spreadsheet conventions. Per SRL-080 disposition.</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>Created during TTS-QUAL-CI-1 close-out 2026-05-28. Lane E governance tooling. Parallel-safe with all other queued sprints.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(ws-server): widen initial auth timeout to 5 min for first-time pairing (EXT-PAIR-1)
WS_AUTH_TIMEOUT_MS (5s) was killing first-time pair connections before
the user could type a 6-digit code. Added WS_PAIRING_TIMEOUT_MS (5 min,
matches SHORT_CODE_TTL_MS) as the initial timer. Post-paired auth is
unaffected — extension sends stored token immediately on connect.

Adds structured logging, 8 new tests, closes BUG-183.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/governance/sprint-queue.xlsx
+++ b/docs/governance/sprint-queue.xlsx
@@ -498,13 +498,13 @@
         <v>35</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>0.8857142857142857</v>
+        <v>0.8683999999999999</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>125</v>
@@ -543,7 +543,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -551,18 +551,18 @@
         </is>
       </c>
       <c r="G6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="12">
       <c r="B7" s="1" t="inlineStr">
         <is>
-          <t>EXT-PAIR-1</t>
+          <t>SINGLE-INSTANCE-LOCK-1</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>SINGLE-INSTANCE-LOCK-1</t>
+          <t>THEME-SYNC-1</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -584,7 +584,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
     </row>
@@ -3009,7 +3009,7 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3064,7 +3064,7 @@
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3123,9 +3123,6 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="n">
-        <v>1</v>
-      </c>
       <c r="B42" t="inlineStr">
         <is>
           <t>EXT-PAIR-1</t>
@@ -3153,7 +3150,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Queued</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -3169,6 +3166,21 @@
       <c r="K42" t="inlineStr">
         <is>
           <t>sprint/ext-pair-1</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>CloseOut.EXT-PAIR-1.2026-05-29.md</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
@@ -3179,7 +3191,7 @@
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3234,7 +3246,7 @@
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3289,7 +3301,7 @@
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix(electron): add single-instance lock to prevent duplicate windows (SINGLE-INSTANCE-LOCK-1)
app.requestSingleInstanceLock() gate before app.whenReady() — second
launcher invocation now focuses the existing window instead of spawning
a duplicate BrowserWindow. Closes F1 from 2026-05-27 live-QA sweep.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/governance/sprint-queue.xlsx
+++ b/docs/governance/sprint-queue.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:H8"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="3" customWidth="1" style="12" min="1" max="1"/>
@@ -498,13 +498,13 @@
         <v>35</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>0.8683999999999999</v>
+        <v>0.8947000000000001</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>125</v>
@@ -516,6 +516,7 @@
         <v>35</v>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="15" customHeight="1" s="12">
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -535,7 +536,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -543,7 +544,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -557,12 +558,12 @@
     <row r="7" ht="15" customHeight="1" s="12">
       <c r="B7" s="1" t="inlineStr">
         <is>
-          <t>SINGLE-INSTANCE-LOCK-1</t>
+          <t>THEME-SYNC-1</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>THEME-SYNC-1</t>
+          <t>NARRATE-CLOSED-LOOP-CURSOR</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -3009,7 +3010,7 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3064,7 +3065,7 @@
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3190,9 +3191,6 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="n">
-        <v>1</v>
-      </c>
       <c r="B43" t="inlineStr">
         <is>
           <t>SINGLE-INSTANCE-LOCK-1</t>
@@ -3210,7 +3208,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Active Conveyor Belt</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -3218,14 +3216,19 @@
           <t>XS</t>
         </is>
       </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Queued</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>Full Spec</t>
+          <t>CloseOut.SINGLE-INSTANCE-LOCK-1.2026-05-29.md</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -3246,7 +3249,7 @@
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3301,7 +3304,7 @@
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs(governance): record single-instance smoke pass
</commit_message>
<xml_diff>
--- a/docs/governance/sprint-queue.xlsx
+++ b/docs/governance/sprint-queue.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="B1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="3" customWidth="1" style="12" min="1" max="1"/>
@@ -516,7 +516,6 @@
         <v>35</v>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="15" customHeight="1" s="12">
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -3216,34 +3215,44 @@
           <t>XS</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr">
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Full Spec</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Add app.requestSingleInstanceLock() + second-instance handler to focus existing window instead of spawning duplicate BrowserWindow. ~5 LOC. Closes F1 from discovery sweep.</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>sprint/single-instance-lock-1</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
         <is>
           <t>2026-05-29</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr">
+      <c r="M43" t="inlineStr">
         <is>
           <t>2026-05-29</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr">
+      <c r="N43" t="inlineStr">
         <is>
           <t>CloseOut.SINGLE-INSTANCE-LOCK-1.2026-05-29.md</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>Add app.requestSingleInstanceLock() + second-instance handler to focus existing window instead of spawning duplicate BrowserWindow. ~5 LOC. Closes F1 from discovery sweep.</t>
-        </is>
-      </c>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t>sprint/single-instance-lock-1</t>
-        </is>
-      </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>XS effort. Parallel-safe with everything in buffer (Lane D, main-process only).</t>
+          <t>XS effort. Manual smoke PASS (launch twice -&gt; one window, existing window focuses/restores). Parallel-safe with everything in buffer (Lane D, main-process only).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(build): eliminate Vite circular chunk settings↔tts (THEME-SYNC-1)
Move 5 shared TTS-adjacent modules (kokoroStatus, qwenStatus,
kokoroRatePlan, ttsProviderRegistry, audio/) to the TTS chunk
explicitly in vite.config.js. These were imported by both TTS and
settings chunk files, causing Rollup to create a bidirectional chunk
dependency. BUG-182 (theme toggle mixed colors) marked resolved
pending live smoke test.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/governance/sprint-queue.xlsx
+++ b/docs/governance/sprint-queue.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:H8"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="3" customWidth="1" style="12" min="1" max="1"/>
@@ -498,13 +498,13 @@
         <v>35</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>0.8947000000000001</v>
+        <v>0.9211</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>125</v>
@@ -516,6 +516,7 @@
         <v>35</v>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="15" customHeight="1" s="12">
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -535,7 +536,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -543,7 +544,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -557,12 +558,12 @@
     <row r="7" ht="15" customHeight="1" s="12">
       <c r="B7" s="1" t="inlineStr">
         <is>
-          <t>THEME-SYNC-1</t>
+          <t>NARRATE-CLOSED-LOOP-CURSOR</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>NARRATE-CLOSED-LOOP-CURSOR</t>
+          <t>UX-POLISH-1</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -3009,7 +3010,7 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3064,7 +3065,7 @@
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3257,9 +3258,6 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="n">
-        <v>1</v>
-      </c>
       <c r="B44" t="inlineStr">
         <is>
           <t>THEME-SYNC-1</t>
@@ -3277,7 +3275,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Active Conveyor Belt</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -3285,14 +3283,19 @@
           <t>S</t>
         </is>
       </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Queued</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>Full Spec</t>
+          <t>CloseOut.THEME-SYNC-1.2026-05-29.md</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
@@ -3313,7 +3316,7 @@
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs(governance): close out 2026-05-29 hotfix session
</commit_message>
<xml_diff>
--- a/docs/governance/sprint-queue.xlsx
+++ b/docs/governance/sprint-queue.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="B1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="3" customWidth="1" style="12" min="1" max="1"/>
@@ -516,7 +516,6 @@
         <v>35</v>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="15" customHeight="1" s="12">
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -3283,34 +3282,44 @@
           <t>S</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr">
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Full Spec</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Resolve settings↔tts circular chunk warning and audit theme-context subscription across Settings sub-pages. Closes BUG-182.</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>sprint/theme-sync-1</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
         <is>
           <t>2026-05-29</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr">
+      <c r="M44" t="inlineStr">
         <is>
           <t>2026-05-29</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr">
+      <c r="N44" t="inlineStr">
         <is>
           <t>CloseOut.THEME-SYNC-1.2026-05-29.md</t>
         </is>
       </c>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>Resolve settings↔tts circular chunk warning and audit theme-context subscription across Settings sub-pages. Closes BUG-182.</t>
-        </is>
-      </c>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>sprint/theme-sync-1</t>
-        </is>
-      </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>Hotfix for BUG-182 (filed 2026-05-28). Aristotle-gated. Parallel-safe with EXT-PAIR-1.</t>
+          <t>Hotfix for BUG-182. Build clean; live smoke PASS on v1.75.1 dev build with E-Ink Display Mode OFF. New BUG-184 filed for einkMode panel transparency.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(queue): DIAG-1 closeout — reshape sprint-queue Catalog to verdict-driven Stage-2 order
Mark NARRATE-DUAL-SOURCE-DIAG-1 COMPLETE (verdict YELLOW). Active queue reordered:
1 INTENT-CURSOR-1 (refocused, A4 fix) | 2 PAUSE-RESUME-UNIFY-1 | 3 A5-RATE-RESEED-1 (new) |
4 APPLYRATECHANGE-COLLAPSE-1 | 5 SUBSCRIBER-CURSOR-1 (gated on A2 retest) | 6 UX-POLISH-1 | 7 HYG.
Catalog tab only; Dashboard formula caches refreshed via scripts/recalc.py.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/governance/sprint-queue.xlsx
+++ b/docs/governance/sprint-queue.xlsx
@@ -826,7 +826,11 @@
       <c r="F4" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="G4" s="5" t="n"/>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>COMPLETE</t>
+        </is>
+      </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
           <t>Complete</t>
@@ -834,7 +838,7 @@
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>Full spec</t>
+          <t>Verdict YELLOW: A4=reader-layer resumeAnchor (dual-source race REFUTED), A5=wrong rate seed</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">
@@ -842,7 +846,11 @@
           <t>Voice mixing feasibility study</t>
         </is>
       </c>
-      <c r="K4" s="5" t="n"/>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>Completed 2026-05-30; verdict NARRATE-DUAL-SOURCE-DIAG-1.md</t>
+        </is>
+      </c>
       <c r="L4" s="5" t="n"/>
       <c r="M4" s="5" t="inlineStr">
         <is>
@@ -854,46 +862,54 @@
     </row>
     <row r="5" ht="15" customHeight="1" s="12">
       <c r="A5" s="5" t="n"/>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>TTS-REGISTRY-1</t>
-        </is>
+      <c r="B5" s="5" t="n">
+        <v>1</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Provider Capability Registry</t>
+          <t>NARRATE-INTENT-CURSOR-1</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>TTS Architecture</t>
+          <t>S</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>Foundation</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="G5" s="5" t="n"/>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>sprint/narrate-intent-cursor-1</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>Stage 2 / NARRATE-INTENT-CURSOR-1</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>Full spec</t>
+          <t>Live-QA A1 still PASS + A4 measured (consume clears anchor)</t>
         </is>
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>Provider capability truth in ttsProviderRegistry</t>
-        </is>
-      </c>
-      <c r="K5" s="5" t="n"/>
+          <t>DIAG-1</t>
+        </is>
+      </c>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>Reader-layer resumeAnchor lifecycle (A4 fix): consume-on-advance + un-gate progress-save</t>
+        </is>
+      </c>
       <c r="L5" s="5" t="n"/>
       <c r="M5" s="5" t="inlineStr">
         <is>
@@ -909,46 +925,54 @@
     </row>
     <row r="6" ht="15" customHeight="1" s="12">
       <c r="A6" s="5" t="n"/>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>TTS-NORMALIZE-1</t>
-        </is>
+      <c r="B6" s="5" t="n">
+        <v>2</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Segment Normalizer</t>
+          <t>NARRATE-PAUSE-RESUME-UNIFY-1</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>TTS Architecture</t>
+          <t>S</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Foundation</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="G6" s="5" t="n"/>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>sprint/narrate-pause-resume-unify-1</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>Stage 2 / NARRATE-PAUSE-RESUME-UNIFY-1</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>Full spec</t>
+          <t>Live-QA A4 PASS 3-of-3</t>
         </is>
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>English-first spoken-text normalization</t>
-        </is>
-      </c>
-      <c r="K6" s="5" t="n"/>
+          <t>INTENT-CURSOR-1</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>Cold-start seed prefers heard/resumeTarget over stale anchor</t>
+        </is>
+      </c>
       <c r="L6" s="5" t="n"/>
       <c r="M6" s="5" t="inlineStr">
         <is>
@@ -964,46 +988,54 @@
     </row>
     <row r="7" ht="23.25" customHeight="1" s="12">
       <c r="A7" s="5" t="n"/>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>TTS-CACHE-TIMING-1</t>
-        </is>
+      <c r="B7" s="5" t="n">
+        <v>4</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Cache Identity &amp; Timing Sidecars</t>
+          <t>NARRATE-APPLYRATECHANGE-COLLAPSE-1</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>TTS Architecture</t>
+          <t>M</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Foundation</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="G7" s="5" t="n"/>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>sprint/narrate-applyratechange-collapse-1</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>Stage 2 / NARRATE-APPLYRATECHANGE-COLLAPSE-1</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>Full spec</t>
+          <t>Live-QA A5 PASS 3-of-3 + voice</t>
         </is>
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>Schema-versioned v2 cache identities and atomic timing sidecars</t>
-        </is>
-      </c>
-      <c r="K7" s="5" t="n"/>
+          <t>A5-RATE-RESEED-1</t>
+        </is>
+      </c>
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>6-&gt;1 reseed paths; seed from priority chain (heardFloor/subscriber)</t>
+        </is>
+      </c>
       <c r="L7" s="5" t="n"/>
       <c r="M7" s="5" t="inlineStr">
         <is>
@@ -1019,52 +1051,52 @@
     </row>
     <row r="8" ht="15" customHeight="1" s="12">
       <c r="A8" s="5" t="n"/>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>TTS-SYNC-1</t>
-        </is>
+      <c r="B8" s="5" t="n">
+        <v>5</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Highlight Sync Controller</t>
+          <t>NARRATE-SUBSCRIBER-CURSOR-1</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>TTS Architecture</t>
+          <t>M</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Sync &amp; Diagnostics</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="n">
-        <v>8</v>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>sprint/narrate-subscriber-cursor-1</t>
+        </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>TTS-CACHE-TIMING-1</t>
+          <t>QUEUED (GATED)</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>Stage 2 / NARRATE-SUBSCRIBER-CURSOR-1</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>Full spec</t>
+          <t>GATED on A2 retest; then Live-QA A2 PASS + regression</t>
         </is>
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>Centralized narration highlight sync policy</t>
+          <t>APPLYRATECHANGE-COLLAPSE-1</t>
         </is>
       </c>
       <c r="K8" s="5" t="inlineStr">
         <is>
-          <t>sprint/tts-sync-1-highlight-controller</t>
+          <t>Retire WORD_ADVANCE; gated on A2 retest (may defer)</t>
         </is>
       </c>
       <c r="L8" s="5" t="n"/>
@@ -1208,50 +1240,54 @@
     </row>
     <row r="11" ht="15" customHeight="1" s="12">
       <c r="A11" s="6" t="n"/>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>TTS-INTEGRATE-1</t>
-        </is>
+      <c r="B11" s="6" t="n">
+        <v>3</v>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Integrate Sync &amp; Diagnostics</t>
+          <t>NARRATE-A5-RATE-RESEED-1</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>TTS Architecture</t>
+          <t>S</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>Consolidation</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="n">
-        <v>2</v>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>sprint/narrate-a5-rate-reseed-1</t>
+        </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>ENGINE-DORMANCY-1</t>
+          <t>QUEUED</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>Stage 2 / NARRATE-A5-RATE-RESEED-1</t>
         </is>
       </c>
       <c r="I11" s="6" t="inlineStr">
         <is>
-          <t>Full spec</t>
+          <t>Live-QA A5 PASS 3-of-3 (long doc)</t>
         </is>
       </c>
       <c r="J11" s="6" t="inlineStr">
         <is>
-          <t>Merge sync and diagnostics branches to main</t>
-        </is>
-      </c>
-      <c r="K11" s="6" t="n"/>
+          <t>DIAG-1</t>
+        </is>
+      </c>
+      <c r="K11" s="6" t="inlineStr">
+        <is>
+          <t>Reseed rate-change from heardFloor, not nextGenWordIndexRef (A5 fix)</t>
+        </is>
+      </c>
       <c r="L11" s="6" t="n"/>
       <c r="M11" s="6" t="n"/>
       <c r="N11" s="6" t="n"/>

</xml_diff>

<commit_message>
revert(queue): restore Catalog to pre-corruption state (undo 49ed885)
Commit 49ed885 attempted the DIAG-1 queue reshape with a WRONG column/row map
(assumed col2=Seq + active rows at 5-8; actual Catalog is 15 columns with col1=Seq
and the active queue at rows 45-50). It overwrote historical completed-sprint rows
(TTS-REGISTRY-1, TTS-NORMALIZE-1, TTS-CACHE-TIMING-1, TTS-SYNC-1, TTS-INTEGRATE-1)
and never touched the real queue. This restores the good xlsx from c2ef361.

DEFERRED: the proper Catalog reshape (mark DIAG-1 complete row 45; Seq INTENT=1
row46, PAUSE-RESUME=2 row47, add A5-RATE-RESEED-1 Seq3, APPLYRATECHANGE=4 row48,
SUBSCRIBER=5 gated row49, UX-POLISH=6 row50, HYG=7; recalc) — to be done in a
session with reliable tooling. ROADMAP.md already reflects the reshaped sequence.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/governance/sprint-queue.xlsx
+++ b/docs/governance/sprint-queue.xlsx
@@ -826,11 +826,7 @@
       <c r="F4" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="G4" s="5" t="inlineStr">
-        <is>
-          <t>COMPLETE</t>
-        </is>
-      </c>
+      <c r="G4" s="5" t="n"/>
       <c r="H4" s="5" t="inlineStr">
         <is>
           <t>Complete</t>
@@ -838,7 +834,7 @@
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>Verdict YELLOW: A4=reader-layer resumeAnchor (dual-source race REFUTED), A5=wrong rate seed</t>
+          <t>Full spec</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">
@@ -846,11 +842,7 @@
           <t>Voice mixing feasibility study</t>
         </is>
       </c>
-      <c r="K4" s="5" t="inlineStr">
-        <is>
-          <t>Completed 2026-05-30; verdict NARRATE-DUAL-SOURCE-DIAG-1.md</t>
-        </is>
-      </c>
+      <c r="K4" s="5" t="n"/>
       <c r="L4" s="5" t="n"/>
       <c r="M4" s="5" t="inlineStr">
         <is>
@@ -862,54 +854,46 @@
     </row>
     <row r="5" ht="15" customHeight="1" s="12">
       <c r="A5" s="5" t="n"/>
-      <c r="B5" s="5" t="n">
-        <v>1</v>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>TTS-REGISTRY-1</t>
+        </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>NARRATE-INTENT-CURSOR-1</t>
+          <t>Provider Capability Registry</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>TTS Architecture</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>sprint/narrate-intent-cursor-1</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G5" s="5" t="n"/>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>Stage 2 / NARRATE-INTENT-CURSOR-1</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>Live-QA A1 still PASS + A4 measured (consume clears anchor)</t>
+          <t>Full spec</t>
         </is>
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>DIAG-1</t>
-        </is>
-      </c>
-      <c r="K5" s="5" t="inlineStr">
-        <is>
-          <t>Reader-layer resumeAnchor lifecycle (A4 fix): consume-on-advance + un-gate progress-save</t>
-        </is>
-      </c>
+          <t>Provider capability truth in ttsProviderRegistry</t>
+        </is>
+      </c>
+      <c r="K5" s="5" t="n"/>
       <c r="L5" s="5" t="n"/>
       <c r="M5" s="5" t="inlineStr">
         <is>
@@ -925,54 +909,46 @@
     </row>
     <row r="6" ht="15" customHeight="1" s="12">
       <c r="A6" s="5" t="n"/>
-      <c r="B6" s="5" t="n">
-        <v>2</v>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>TTS-NORMALIZE-1</t>
+        </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>NARRATE-PAUSE-RESUME-UNIFY-1</t>
+          <t>Segment Normalizer</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>TTS Architecture</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>sprint/narrate-pause-resume-unify-1</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G6" s="5" t="n"/>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>Stage 2 / NARRATE-PAUSE-RESUME-UNIFY-1</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>Live-QA A4 PASS 3-of-3</t>
+          <t>Full spec</t>
         </is>
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>INTENT-CURSOR-1</t>
-        </is>
-      </c>
-      <c r="K6" s="5" t="inlineStr">
-        <is>
-          <t>Cold-start seed prefers heard/resumeTarget over stale anchor</t>
-        </is>
-      </c>
+          <t>English-first spoken-text normalization</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="n"/>
       <c r="L6" s="5" t="n"/>
       <c r="M6" s="5" t="inlineStr">
         <is>
@@ -988,54 +964,46 @@
     </row>
     <row r="7" ht="23.25" customHeight="1" s="12">
       <c r="A7" s="5" t="n"/>
-      <c r="B7" s="5" t="n">
-        <v>4</v>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>TTS-CACHE-TIMING-1</t>
+        </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>NARRATE-APPLYRATECHANGE-COLLAPSE-1</t>
+          <t>Cache Identity &amp; Timing Sidecars</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>TTS Architecture</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>sprint/narrate-applyratechange-collapse-1</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G7" s="5" t="n"/>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>Stage 2 / NARRATE-APPLYRATECHANGE-COLLAPSE-1</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>Live-QA A5 PASS 3-of-3 + voice</t>
+          <t>Full spec</t>
         </is>
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>A5-RATE-RESEED-1</t>
-        </is>
-      </c>
-      <c r="K7" s="5" t="inlineStr">
-        <is>
-          <t>6-&gt;1 reseed paths; seed from priority chain (heardFloor/subscriber)</t>
-        </is>
-      </c>
+          <t>Schema-versioned v2 cache identities and atomic timing sidecars</t>
+        </is>
+      </c>
+      <c r="K7" s="5" t="n"/>
       <c r="L7" s="5" t="n"/>
       <c r="M7" s="5" t="inlineStr">
         <is>
@@ -1051,52 +1019,52 @@
     </row>
     <row r="8" ht="15" customHeight="1" s="12">
       <c r="A8" s="5" t="n"/>
-      <c r="B8" s="5" t="n">
-        <v>5</v>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>TTS-SYNC-1</t>
+        </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>NARRATE-SUBSCRIBER-CURSOR-1</t>
+          <t>Highlight Sync Controller</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>TTS Architecture</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>sprint/narrate-subscriber-cursor-1</t>
-        </is>
+          <t>Sync &amp; Diagnostics</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>8</v>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>QUEUED (GATED)</t>
+          <t>TTS-CACHE-TIMING-1</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>Stage 2 / NARRATE-SUBSCRIBER-CURSOR-1</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>GATED on A2 retest; then Live-QA A2 PASS + regression</t>
+          <t>Full spec</t>
         </is>
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>APPLYRATECHANGE-COLLAPSE-1</t>
+          <t>Centralized narration highlight sync policy</t>
         </is>
       </c>
       <c r="K8" s="5" t="inlineStr">
         <is>
-          <t>Retire WORD_ADVANCE; gated on A2 retest (may defer)</t>
+          <t>sprint/tts-sync-1-highlight-controller</t>
         </is>
       </c>
       <c r="L8" s="5" t="n"/>
@@ -1240,54 +1208,50 @@
     </row>
     <row r="11" ht="15" customHeight="1" s="12">
       <c r="A11" s="6" t="n"/>
-      <c r="B11" s="6" t="n">
-        <v>3</v>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>TTS-INTEGRATE-1</t>
+        </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>NARRATE-A5-RATE-RESEED-1</t>
+          <t>Integrate Sync &amp; Diagnostics</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>TTS Architecture</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="inlineStr">
-        <is>
-          <t>sprint/narrate-a5-rate-reseed-1</t>
-        </is>
+          <t>Consolidation</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>2</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>ENGINE-DORMANCY-1</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>Stage 2 / NARRATE-A5-RATE-RESEED-1</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="I11" s="6" t="inlineStr">
         <is>
-          <t>Live-QA A5 PASS 3-of-3 (long doc)</t>
+          <t>Full spec</t>
         </is>
       </c>
       <c r="J11" s="6" t="inlineStr">
         <is>
-          <t>DIAG-1</t>
-        </is>
-      </c>
-      <c r="K11" s="6" t="inlineStr">
-        <is>
-          <t>Reseed rate-change from heardFloor, not nextGenWordIndexRef (A5 fix)</t>
-        </is>
-      </c>
+          <t>Merge sync and diagnostics branches to main</t>
+        </is>
+      </c>
+      <c r="K11" s="6" t="n"/>
       <c r="L11" s="6" t="n"/>
       <c r="M11" s="6" t="n"/>
       <c r="N11" s="6" t="n"/>

</xml_diff>

<commit_message>
chore(queue): DIAG-1 closeout — correct Catalog reshape (supersedes reverted 49ed885)
Redone with the verified row/column map (col1=Seq; active queue rows 46-51).
DIAG-1 (row46) -> Completed, Seq cleared, dated 2026-05-30. Active queue:
Seq1 INTENT-CURSOR-1 (refocused, A4 fix), Seq2 PAUSE-RESUME-UNIFY-1,
Seq3 NARRATE-A5-RATE-RESEED-1 (new row51), Seq4 APPLYRATECHANGE-COLLAPSE-1,
Seq5 SUBSCRIBER-CURSOR-1 (gated on A2 retest), Seq6 UX-POLISH-1, Seq7 HYG.
Historical rows verified intact (assert-gated write). Dashboard caches recalc'd.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/governance/sprint-queue.xlsx
+++ b/docs/governance/sprint-queue.xlsx
@@ -604,7 +604,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O50"/>
+  <dimension ref="A1:O51"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="5" customWidth="1" style="12" min="1" max="1"/>
@@ -3417,7 +3417,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>Queued</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -3435,15 +3435,20 @@
           <t>sprint/narrate-dual-source-diag-1</t>
         </is>
       </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>Gating sprint for positions 2-5. Per SRL-072: do not iterate on ahead-of-heard refs without first verifying their role. Logs gated by localStorage.BLURBY_DUAL_SOURCE_DIAG="1".</t>
+          <t>Gating sprint for positions 2-5. Per SRL-072: do not iterate on ahead-of-heard refs without first verifying their role. Logs gated by localStorage.BLURBY_DUAL_SOURCE_DIAG="1". | Verdict YELLOW: A4=reader-layer resumeAnchor (dual-source race REFUTED), A5=wrong rate seed.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
@@ -3497,13 +3502,13 @@
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>Smallest implementation risk in 2-5; ships first to establish lifecycle pattern. Live-QA gate: A1 (hard-click exact start) PASS on The Raven.</t>
+          <t>Smallest implementation risk in 2-5; ships first to establish lifecycle pattern. Live-QA gate: A1 (hard-click exact start) PASS on The Raven. | Refocused: reader-layer resumeAnchor lifecycle + un-gate progress-save (A4 fix).</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
@@ -3677,7 +3682,67 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>Live-QA THE A2 GATE + regression suite. ULTRATHINK section 4.2: React batching is the original sin; removing React from the visual-highlight path is the only way to actually eliminate cursor lead, not just compensate for it.</t>
+          <t>Live-QA THE A2 GATE + regression suite. ULTRATHINK section 4.2: React batching is the original sin; removing React from the visual-highlight path is the only way to actually eliminate cursor lead, not just compensate for it. | GATED on A2 retest (may defer).</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>3</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>NARRATE-A5-RATE-RESEED-1</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Rate-Change Reseed from Heard Position</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Reader Runtime Solidification</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Active Conveyor Belt</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>NARRATE-DUAL-SOURCE-DIAG-1</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Queued</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Full Spec</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>Reseed applyRateChange Kokoro bucket-change from heardFloor, not nextGenWordIndexRef (A5 fix)</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>sprint/narrate-a5-rate-reseed-1</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>New sprint from DIAG-1 verdict (A5 FAIL).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
roadmap-status(2026-05-30): sync DIAG-1 Catalog Close-Out File pointer
Phase 2 of /roadmap-status: single-cell Catalog edit on the NARRATE-DUAL-SOURCE-DIAG-1 row to populate Close-Out File with docs/governance/close-outs/CloseOut.NARRATE-DUAL-SOURCE-DIAG-1.2026-05-30.md (was None). The close-out file already existed; only the Catalog pointer was missing.

scripts/recalc.py re-ran cleanly (0 formula cells, consistent with HYG-XLSX-DASHBOARD-RESTORE scope per SRL-080). Post-save reopen verified value persistence and xlsx structural validity (no BadZipFile this round).

Checkin briefing saved at docs/planning/roadmap-reviews/checkins/2026-05-30-status.md. Health read: On Track. Buffer healthy at 5/5 full specs. Pace ~1 sprint/day in May. No other recommendations; DIAG-1's active-section archival marker is deferred per inline note to next /roadmap-review.
</commit_message>
<xml_diff>
--- a/docs/governance/sprint-queue.xlsx
+++ b/docs/governance/sprint-queue.xlsx
@@ -3437,6 +3437,11 @@
           <t>2026-05-30</t>
         </is>
       </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>docs/governance/close-outs/CloseOut.NARRATE-DUAL-SOURCE-DIAG-1.2026-05-30.md</t>
+        </is>
+      </c>
       <c r="O46" t="inlineStr">
         <is>
           <t>Gating sprint for positions 2-5. Per SRL-072: do not iterate on ahead-of-heard refs without first verifying their role. Logs gated by localStorage.BLURBY_DUAL_SOURCE_DIAG="1". | Verdict YELLOW: A4=reader-layer resumeAnchor (dual-source race REFUTED), A5=wrong rate seed.</t>

</xml_diff>

<commit_message>
narrate-intent-cursor-1(docs): ROADMAP + CLAUDE.md + sprint-queue.xlsx (PARTIAL closeout)
INTENT-CURSOR-1 marked Completed (PARTIAL). ROADMAP: Completed Work Summary row,
header updated (next = PAUSE-RESUME-UNIFY-1), conveyor renumbered, sprint section
marked COMPLETE PARTIAL. CLAUDE.md: queue GREEN depth 6, test count 3044/213,
most recent sprint updated. sprint-queue.xlsx: row 47 Completed (Seq cleared),
PAUSE-RESUME-UNIFY-1 -> Seq1, A5-RATE-RESEED-1 -> Seq2, remaining renumbered.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/governance/sprint-queue.xlsx
+++ b/docs/governance/sprint-queue.xlsx
@@ -3010,7 +3010,7 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3333,7 +3333,7 @@
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
@@ -3449,9 +3449,6 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="n">
-        <v>1</v>
-      </c>
       <c r="B47" t="inlineStr">
         <is>
           <t>NARRATE-INTENT-CURSOR-1</t>
@@ -3484,7 +3481,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>Queued</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -3502,15 +3499,25 @@
           <t>sprint/narrate-intent-cursor-1</t>
         </is>
       </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>NARRATE-DUAL-SOURCE-FIX-b1138f4-liveqa-gate-report.md</t>
+        </is>
+      </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>Smallest implementation risk in 2-5; ships first to establish lifecycle pattern. Live-QA gate: A1 (hard-click exact start) PASS on The Raven. | Refocused: reader-layer resumeAnchor lifecycle + un-gate progress-save (A4 fix).</t>
+          <t>PARTIAL: A1 PASS, A4 FAIL 0-of-3. Consume lifecycle landed; reactive not preventive. PAUSE-RESUME-UNIFY-1 completes.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
@@ -3570,7 +3577,7 @@
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
@@ -3630,7 +3637,7 @@
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
@@ -3690,7 +3697,7 @@
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs(narrate-diag): NARRATE-CURSOR-TRACKING-DIAG-1 verdict + closeout
Live trace REFUTED the schedulerActiveWord hypothesis: heardFloor==schedulerActiveWord (0/0/0 offset, n=191 & n=716), the whole telemetry cluster leads the ear, and the visible-cursor owner is lag-compensated wordIndex (~350ms WASAPI) — not any raw scheduler signal. Cycle (b) independently reproduced the A5 defect (mid-playback WPM change reseeds from the nextGenWordIndex frontier). Updates: investigation doc (verdict + ranked-accuracy table + 3-cycle QA), ROADMAP (sprint complete, A5-RATE-RESEED-1 next, SUBSCRIBER-CURSOR-1 amended to publish a lag-compensated heard cursor), sprint-queue.xlsx (Catalog completed, renumbered), LESSONS_LEARNED LL-127. Instrumentation source is net-unchanged (DIAG flags back to false).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/governance/sprint-queue.xlsx
+++ b/docs/governance/sprint-queue.xlsx
@@ -585,7 +585,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
@@ -604,7 +604,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O51"/>
+  <dimension ref="A1:O52"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="5" customWidth="1" style="12" min="1" max="1"/>
@@ -3010,7 +3010,7 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3333,7 +3333,7 @@
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
@@ -3516,9 +3516,6 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="n">
-        <v>1</v>
-      </c>
       <c r="B48" t="inlineStr">
         <is>
           <t>NARRATE-PAUSE-RESUME-UNIFY-1</t>
@@ -3551,7 +3548,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>Queued</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -3569,15 +3566,25 @@
           <t>sprint/narrate-pause-resume-unify-1</t>
         </is>
       </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>docs/governance/close-outs/CloseOut.NARRATE-PAUSE-RESUME-UNIFY-1.2026-05-31.md</t>
+        </is>
+      </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>Live-QA THE A4 GATE: 3-of-3 pause/resume cycles preserve position per Evan's ear. Verbatim Evan verdict 2026-05-29: play-pause-play resets anchor.</t>
+          <t>Source merged at db2d1bc; anchor-correctness follow-up merged at 1299808. Live A4 retest still recommended before user-facing gate is declared closed.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
@@ -3631,13 +3638,13 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>Live-QA THE A5 GATE: 3-of-3 rate changes preserve position; voice change preserves position. Addresses codex-parent's flagged ~14 speakNextChunk call sites not fully traced.</t>
+          <t>Sequenced after NARRATE-CURSOR-TRACKING-DIAG-1 and A5-RATE-RESEED-1. Live-QA THE A5 GATE: 3-of-3 rate changes preserve position; voice change preserves position.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
@@ -3666,7 +3673,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>NARRATE-APPLYRATECHANGE-COLLAPSE-1 (no audio decision still reads from cursorWordIndex)</t>
+          <t>NARRATE-CURSOR-TRACKING-DIAG-1; NARRATE-APPLYRATECHANGE-COLLAPSE-1</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -3681,7 +3688,7 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>Rename lastConfirmedAudioWordRef -&gt; subscriberCursorRef; remove cursorWordIndex from React reducer state; remove WORD_ADVANCE action; visual highlight via direct DOM mutation (bypass React batching that causes A2 lead). Last and heaviest sprint; ships last so any regression is localized.</t>
+          <t>If NARRATE-CURSOR-TRACKING-DIAG-1 confirms the subscriber/direct-callback model, rename lastConfirmedAudioWordRef -&gt; subscriberCursorRef, remove cursorWordIndex from React reducer state, remove WORD_ADVANCE action, and wire visual/view follow via the verdict-approved live target.</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -3691,13 +3698,13 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>Live-QA THE A2 GATE + regression suite. ULTRATHINK section 4.2: React batching is the original sin; removing React from the visual-highlight path is the only way to actually eliminate cursor lead, not just compensate for it. | GATED on A2 retest (may defer).</t>
+          <t>GATED. AMENDED 2026-05-31 per CURSOR-TRACKING-DIAG-1 verdict: subscriberCursor was no-data; publish a LAG-COMPENSATED heard cursor (wordIndex minus ~350ms pipeline lag), NOT schedulerActiveWord/heardFloor (both lead) nor nextGenWordIndex (frontier). Re-trace subscriber channel after wiring.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
@@ -3751,7 +3758,74 @@
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>New sprint from DIAG-1 verdict (A5 FAIL).</t>
+          <t>New sprint from DIAG-1 verdict (A5 FAIL). Sequenced after NARRATE-CURSOR-TRACKING-DIAG-1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>NARRATE-CURSOR-TRACKING-DIAG-1</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Narrate Cursor Tracking Diagnostic</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Reader Runtime Solidification</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Active Conveyor Belt</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>NARRATE-PAUSE-RESUME-UNIFY-1; revert fcea6a8</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Full Spec</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>Instrument cursor, heard-floor, anchor, Foliate, and Flow follow signals to prove which source should drive visible cursor and view-follow before another fix.</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>sprint/narrate-cursor-tracking-diag-1</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>Live-QA trace 2026-05-31 (Meditations, DIAG on/reverted). Hypothesis REFUTED: schedulerActiveWord==heardFloor lead the heard voice; wordIndex (visible cursor) closest but still leads &amp; drifts; nextGenWordIndex is pre-fetch frontier; resumeTarget/subscriberCursor no-data. SUBSCRIBER-CURSOR-1 amended -&gt; publish lag-compensated heard cursor. See investigations/NARRATE-CURSOR-TRACKING-DIAG-1.md.</t>
         </is>
       </c>
     </row>

</xml_diff>